<commit_message>
chore: alinear entregable final con DB, re-correr LLM y config externalizada
- Re-corrida del LLM (7 casos originales + 2 parsing) → 0 errores de parsing,
  0 casos sin señales en las 250 filas
- Excel entregable regenerado desde DB: 150/150 con recomendación, justificación
  y señales, sin discrepancias (150: 67 APROBAR / 57 RECHAZAR / 26 ESCALAR)
- README y diccionario de datos con distribución final
- Config del LLM externalizada en src/config/ (model.yaml + prompts + .env.example)
- Consolidación resolution_case (renombra 05_analisis_casos → 05_resolution_case),
  backfill de justificaciones de reglas y seed regenerado
- Tests: 98 passed; ./init.sh OK
</commit_message>
<xml_diff>
--- a/data/150casos_analizados.xlsx
+++ b/data/150casos_analizados.xlsx
@@ -646,19 +646,19 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. El reclamo es coherente y no activa reglas de rechazo o escalación.</t>
+          <t>Usuario con antigüedad superior a 4 años y 0 flags de fraude. Reclamo operativo sin señales de abuso o inconsistencia.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario conservador y sin historial negativo valida la solicitud. | Reclamo operativo estándar en cuenta antigua sin señales de riesgo o inconsistencia.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Error de preparación del restaurante en usuario antiguo y limpio, sin evidencia de fraude.</t>
         </is>
       </c>
     </row>
@@ -755,17 +755,18 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', activando el protocolo de seguridad de marca que requiere revisión humana inmediata. Aunque el GPS es parcial y existe un flag previo, la mención de riesgo de salud anula la automatización.</t>
+          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas que obliga a escalación por riesgo de salud/marca. Aunque el GPS es parcial y existe un flag previo, la mención de condiciones médicas supera cualquier análisis automatizado.</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | entrega_gps_parcial</t>
+          <t>palabras_criticas_seguridad | evidencia_gps_parcial | flag_fraude_previo</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -775,7 +776,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene término crítico de salud ('alergia') que exige revisión manual según política de seguridad de marca. | Reclamo por alergia alimentaria con evidencia GPS parcial y flag de fraude previo. La palabra crítica activa escalación obligatoria.</t>
+          <t>ESCALAR: contiene palabra crítica 'alergia' que implica riesgo de salud y responsabilidad legal, requiriendo validación manual según política de seguridad de marca. | Reclamo por alergia alimentaria en cuenta con flag previo y GPS parcial, sujeto a revisión humana obligatoria por términos de seguridad de marca.</t>
         </is>
       </c>
     </row>
@@ -857,7 +858,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -867,24 +868,24 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>El usuario presenta un flag de fraude previo combinado con un ratio de compensación muy alto (0.8975). El reclamo por faltantes es subjetivo y carece de validación GPS, lo que incrementa significativamente el riesgo de abuso.</t>
+          <t>Reclamo por faltantes coherente, pero la cuenta tiene 1 flag de fraude previo y ratio de compensación alto (0.89). Se requiere validación manual para cruzar evidencia y revisar el antecedente.</t>
         </is>
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | compensacion_elevada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>RECHAZAR: historial con flag de fraude, ratio de compensación elevado y falta de evidencia objetiva para faltantes menores. | Reclamo por faltantes sin evidencia objetiva en cuenta con historial de fraude y alta tasa de compensación.</t>
+          <t>ESCALAR: flag de fraude previo combinado con compensación elevada exige revisión humana para validar legitimidad. | Solicitud de faltantes en cuenta con historial mixto y alta frecuencia de pagos.</t>
         </is>
       </c>
     </row>
@@ -981,19 +982,19 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Cuenta antigua y sin historial de fraude, pero la pérdida de señal GPS impide corroborar la entrega. El ratio de compensación cercano a 1.0 y la falta de evidencia objetiva requieren validación manual.</t>
+          <t>Cuenta antigua y sin historial de fraude, pero la evidencia GPS está perdida lo que impide validar o refutar la entrega. Reclamo subjetivo sin corroboración objetiva.</t>
         </is>
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>evidencia_gps_parcial | compensacion_elevada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por señal GPS perdida y ratio de compensación elevado que impiden decisión automatizada segura. | Reclamo por no recepción con evidencia GPS incompleta en usuario de larga antigüedad.</t>
+          <t>ESCALAR: falta de evidencia GPS para confirmar entrega y naturaleza subjetiva del reclamo requieren revisión humana. | Reclamo de no recepción con señal GPS perdida en cuenta confiable de larga antigüedad.</t>
         </is>
       </c>
     </row>
@@ -1090,15 +1091,19 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Usuario con 4+ años de antigüedad, sin flags ni frecuencia de reclamos. Reclamo de discrepancia de cobro objetivo y monto dentro de parámetros normales.</t>
+          <t>Usuario con 1458 días de antigüedad y 0 flags. Reclamo administrativo sobre cobro sin señales de fraude ni inconsistencia.</t>
         </is>
       </c>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr"/>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>descripcion_incoherente</t>
+        </is>
+      </c>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de error de facturación en usuario con historial impecable y sin señales de fraude. | Discrepancia de cobro en cuenta limpia y antigua sin señales de fraude.</t>
+          <t>APROBAR: reclamo legítimo de discrepancia de cobro en cuenta sin riesgos. | Discrepancia de monto reportada por usuario leal sin historial de reclamos recientes.</t>
         </is>
       </c>
     </row>
@@ -1192,7 +1197,8 @@
       <c r="W7" t="inlineStr"/>
       <c r="X7" t="inlineStr">
         <is>
-          <t>R4 — Compensación solicitada &gt; p99 del dataset original</t>
+          <t>R4 — Compensación solicitada &gt; p99 del dataset original
+Solo el 1% de las compensaciones supera este monto: es atípico y se rechaza automáticamente.</t>
         </is>
       </c>
       <c r="Y7" t="inlineStr"/>
@@ -1296,19 +1302,19 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Perfil de usuario sólido (655 días de antigüedad, 0 flags, 2 reclamos en 90d). Aunque la verificación de caducidad es subjetiva y el GPS se perdió, no existen inconsistencias ni patrones de abuso que respalden un rechazo.</t>
+          <t>Usuario con antigüedad superior a 6 meses, baja frecuencia de reclamos y sin flags de fraude. No se activaron reglas de riesgo ni palabras críticas.</t>
         </is>
       </c>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo | entrega_gps_no_confirmada</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>APROBAR: usuario con historial conservador y sin indicadores de riesgo que invaliden el reclamo. | Reclamo por producto caducado en cuenta antigua y limpia, sin señales de fraude detectadas.</t>
+          <t>APROBAR: reclamo legítimo sin señales de fraude ni criterios de rechazo o escalación. | Reclamo por producto caducado en cuenta limpia, sin inconsistencias operativas ni señales de abuso detectadas.</t>
         </is>
       </c>
     </row>
@@ -1405,7 +1411,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad de 312 días, 0 flags de fraude y baja frecuencia de reclamos. El reporte de doble cobro es un error operativo frecuente y coherente con la información disponible.</t>
+          <t>Perfil de usuario limpio con antigüedad moderada y baja frecuencia de reclamos. El tipo de incidencia (cobro duplicado) es operativo y no presenta inconsistencias con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X9" t="inlineStr"/>
@@ -1417,7 +1423,7 @@
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo por error de cobro duplicado en usuario con historial limpio y perfil conservador. | Error de facturación en cuenta limpia sin indicadores de abuso o inconsistencia crítica.</t>
+          <t>APROBAR: reclamo operativo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Reclamo por cobro duplicado en cuenta sin historial de fraude ni señales de abuso. Evidencia GPS no aplicable al tipo de incidencia.</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1517,8 @@
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr"/>
@@ -1615,19 +1622,19 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Usuario veterano con 1656 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado es proporcional al pedido y la falta de confirmación GPS es irrelevante para incidencias de faltantes.</t>
+          <t>Usuario con 1656 días de antigüedad y 0 flags de fraude. El reclamo por faltante de producto es operativo, coherente y no activa reglas de riesgo.</t>
         </is>
       </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y monto razonable. | Reclamo por faltantes operativos en cuenta de alto valor e historial impecable.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario antiguo y sin señales de fraude. | Reclamo por faltante parcial validado para usuario confiable de larga data sin inconsistencias.</t>
         </is>
       </c>
     </row>
@@ -1721,7 +1728,10 @@
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y12" t="inlineStr"/>
@@ -1822,7 +1832,8 @@
       <c r="W13" t="inlineStr"/>
       <c r="X13" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y13" t="inlineStr"/>
@@ -1926,19 +1937,19 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Usuario con más de 2 años de antigüedad, historial limpio y única reclamación reciente. La cancelación del restaurante es un evento operativo coherente y verificable sin contradicciones.</t>
+          <t>Usuario con 843 días de antigüedad y 0 flags de fraude. Reclamo operativo estándar por cobro tras cancelación, sin patrones abusivos ni palabras críticas.</t>
         </is>
       </c>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo sin señales de fraude o inconsistencia. | Solicitud de reembolso por cancelación operativa en cuenta establecida y sin riesgos previos.</t>
+          <t>APROBAR: reclamo legítimo sin señales de fraude o inconsistencias operativas relevantes. | Solicitud de reembolso por cargo pendiente tras cancelación del restaurante en cuenta antigua y limpia.</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2043,8 @@
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y15" t="inlineStr"/>
@@ -2136,19 +2148,19 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años y 0 flags de fraude. El reclamo es subjetivo pero coherente con fallas de calidad alimentaria, sin contradicciones evidentes.</t>
+          <t>Usuario con antigüedad superior a 2 años y 0 flags de fraude. Reclamo por calidad de alimento sin inconsistencias ni patrones de abuso.</t>
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo | entrega_gps_no_confirmada</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable y reclamo sin señales de fraude o inconsistencia crítica. | Reclamo por olor desagradable en cuenta estable sin historial abusivo.</t>
+          <t>APROBAR: reclamo coherente con perfil de usuario confiable y sin señales de fraude. | Reclamo legítimo por deterioro percibido en cuenta estable y sin historial negativo.</t>
         </is>
       </c>
     </row>
@@ -2230,7 +2242,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2240,24 +2252,24 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>Cuenta nueva (75d) con alta frecuencia de reclamos (6 en 90d) y sin evidencia GPS. Requiere revisión para validar lógica de cupones vs patrón de uso.</t>
+          <t>Cuenta nueva (75 días) con 6 reclamos en 90 días, lo que activa la regla de sospecha por múltiples reclamos en periodo reciente. El reclamo por cupón carece de evidencia objetiva y se combina con un patrón de alta frecuencia.</t>
         </is>
       </c>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>antiguedad_moderada_con_alta_reincidencia | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>antiguedad_moderada_con_alta_reincidencia | alta_frecuencia_reclamos | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>ESCALAR: cuenta nueva con múltiples reclamos y datos insuficientes para verificación automática, riesgo de abuso detectado. | Reclamo por error de cupón en cuenta reciente con alta densidad de solicitudes y falta de corroboración GPS.</t>
+          <t>RECHAZAR: cuenta nueva con múltiples reclamos en 90 días y patrón de alta frecuencia que sugiere abuso potencial. | Reclamo por error de cupón en cuenta nueva con alta densidad de solicitudes en 90 días.</t>
         </is>
       </c>
     </row>
@@ -2354,19 +2366,19 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>Reclamo por cobro tras cancelación del restaurante. Sin flags de fraude ni palabras críticas, pero la alta frecuencia (6 en 90d) y la evidencia GPS parcial generan ambigüedad operativa que requiere validación manual.</t>
+          <t>Usuario con antigüedad moderada y 6 reclamos en 90 días. Evidencia GPS parcial y disputa de cobro generan ambigüedad operativa.</t>
         </is>
       </c>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | evidencia_gps_parcial</t>
+          <t>alta_frecuencia_reclamos | evidencia_gps_parcial | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>ESCALAR: alta frecuencia de reclamos y evidencia GPS parcial requieren validación manual del estado real del pedido y política de reembolso. | Disputa de cobro por cancelación con patrón de frecuencia elevada y GPS inconclusa.</t>
+          <t>ESCALAR: alta frecuencia de reclamos combinada con GPS parcial y naturaleza de disputa financiera requieren validación humana con pasarela/restaurante. | Reclamo por cargo pendiente tras cancelación del restaurante, con alta frecuencia de actividad y evidencia de ubicación incompleta.</t>
         </is>
       </c>
     </row>
@@ -2460,7 +2472,10 @@
       <c r="W19" t="inlineStr"/>
       <c r="X19" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.</t>
         </is>
       </c>
       <c r="Y19" t="inlineStr"/>
@@ -2561,7 +2576,10 @@
       <c r="W20" t="inlineStr"/>
       <c r="X20" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d
+Cuenta nueva (&lt; 90 días) con récord de reclamos: la señal de fraude más fuerte del dataset.</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr"/>
@@ -2665,7 +2683,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a un año, historial limpio y baja frecuencia de reclamos. El reclamo describe un error operativo común sin términos críticos ni inconsistencias.</t>
+          <t>Usuario con 609 días de antigüedad y historial limpio. Reclamo por error de preparación sin contradicciones con la evidencia disponible. Monto solicitado dentro de parámetros normales y sin indicadores de abuso.</t>
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
@@ -2677,7 +2695,7 @@
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de riesgo. | Reclamo por producto incorrecto en cuenta estable sin indicadores de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Error operativo aislado en cuenta estable sin señales de riesgo.</t>
         </is>
       </c>
     </row>
@@ -2759,7 +2777,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2769,20 +2787,24 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>Historial con alta frecuencia de reclamos y ratio de compensación elevado, combinado con ausencia de evidencia GPS. La verificación de producto caducado requiere revisión manual.</t>
+          <t>Usuario con flag de fraude previo y alta frecuencia de reclamos (5 en 90d). La falta de confirmación GPS y la naturaleza subjetiva del reclamo (producto caducado) sin evidencia digital refuerzan el riesgo de abuso.</t>
         </is>
       </c>
       <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>flag_fraude_previo | alta_frecuencia_reclamos | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+        </is>
+      </c>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de alta frecuencia, ratio de compensación elevado y falta de evidencia GPS requiere validación humana. | Reclamo por vencimiento de producto en cuenta con patrón de compensaciones frecuentes y sin validación geolocalizada.</t>
+          <t>RECHAZAR: combinación de flag de fraude previo, alta frecuencia de reclamos y falta de evidencia GPS para validar una solicitud subjetiva. | Reclamo por producto caducado en cuenta con historial de fraude, alta densidad de solicitudes y sin validación geoespacial.</t>
         </is>
       </c>
     </row>
@@ -2879,7 +2901,7 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad &gt;1 año y 0 flags de fraude. Reclamo por error de cupón sin inconsistencias críticas.</t>
+          <t>Perfil limpio con 377 días de antigüedad y 0 flags. El reclamo corresponde a una discrepancia de precios/cupones, típica de errores operativos.</t>
         </is>
       </c>
       <c r="X23" t="inlineStr"/>
@@ -2891,7 +2913,7 @@
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude o patrones de abuso detectados. | Solicitud de ajuste por cupón no aplicado en cuenta estable sin historial abusivo.</t>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de abuso o inconsistencia crítica. | Reclamo por aplicación incorrecta de cupón en cuenta antigua sin historial de fraude.</t>
         </is>
       </c>
     </row>
@@ -2985,7 +3007,8 @@
       <c r="W24" t="inlineStr"/>
       <c r="X24" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y24" t="inlineStr"/>
@@ -3089,19 +3112,19 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad de 325 días y 0 flags de fraude. Reclamo por faltante operativo sin señales de abuso, inconsistencia GPS o palabras críticas.</t>
+          <t>Usuario con 325 días de antigüedad y sin historial de fraude. El reclamo por ítem faltante es coherente con errores operativos habituales. No se detectan patrones de abuso, inconsistencias GPS críticas ni términos de riesgo.</t>
         </is>
       </c>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente y sin señales de fraude detectadas. | Reclamo legítimo de faltante en cuenta verificada sin historial de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sin riesgos detectados. | Reclamo estándar por producto faltante en cuenta con buen historial y sin señales de fraude.</t>
         </is>
       </c>
     </row>
@@ -3198,19 +3221,19 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>Usuario con historial de 1 flag de fraude y 6 reclamos en 90 días. Evidencia GPS parcial que no respalda la afirmación de doble cobro.</t>
+          <t>El perfil presenta señales de riesgo acumuladas: alta frecuencia de reclamos, flag de fraude previo, evidencia GPS parcial y ratio de compensación elevado, lo que contradice la coherencia esperada en un error operativo aislado.</t>
         </is>
       </c>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | evidencia_gps_parcial</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_parcial | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>RECHAZAR: patrón de abuso confirmado por alta frecuencia de reclamos, flag de fraude previo e inconsistencia en evidencia GPS. | Reclamo de doble cobro en cuenta con alta frecuencia de incidencias y señal previa de fraude, sin validación geoespacial completa.</t>
+          <t>RECHAZAR: combinación de flag de fraude, alta frecuencia y GPS parcial indica patrón de abuso o inconsistencia verificable. | Reclamo por doble cobro en cuenta con historial negativo y evidencia logística incompleta.</t>
         </is>
       </c>
     </row>
@@ -3304,7 +3327,12 @@
       <c r="W27" t="inlineStr"/>
       <c r="X27" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d
+Cuenta nueva (&lt; 90 días) con récord de reclamos: la señal de fraude más fuerte del dataset.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y27" t="inlineStr"/>
@@ -3405,7 +3433,8 @@
       <c r="W28" t="inlineStr"/>
       <c r="X28" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y28" t="inlineStr"/>
@@ -3506,7 +3535,8 @@
       <c r="W29" t="inlineStr"/>
       <c r="X29" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y29" t="inlineStr"/>
@@ -3607,7 +3637,8 @@
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y30" t="inlineStr"/>
@@ -3711,19 +3742,19 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, historial limpio y cero reclamos recientes. La falta de salsas y cubiertos es un error operativo frecuente y coherente con la evidencia disponible.</t>
+          <t>Usuario con antigüedad superior a 3 años, historial limpio y cero reclamos recientes. La omisión de elementos es un error operativo común y coherente.</t>
         </is>
       </c>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario confiable y sin indicadores de abuso. | Reclamo por artículos faltantes en cuenta antigua y sin señales de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario sin riesgos detectados. | Reclamo por artículos faltantes validado por perfil de usuario consolidado y sin indicadores de fraude.</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3851,7 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>Usuario con 1016 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El reclamo por producto caducado es coherente y no activa umbrales de riesgo ni palabras críticas.</t>
+          <t>Usuario con más de 2 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. La solicitud por producto caducado es un reclamo de calidad estándar sin contradicciones con la evidencia disponible ni términos críticos de riesgo legal o sanitario.</t>
         </is>
       </c>
       <c r="X32" t="inlineStr"/>
@@ -3832,7 +3863,7 @@
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable con historial limpio y reclamo plausible sin señales de fraude. | Reclamo de calidad alimentaria en cuenta veterana y limpia, sin inconsistencias operativas ni evidencia de abuso.</t>
+          <t>APROBAR: perfil de usuario confiable, sin señales de riesgo y reclamo coherente con las reglas de negocio. | Reclamo de calidad alimentaria en cuenta antigua y limpia sin indicadores de fraude, abuso o inconsistencia operativa.</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3957,8 @@
       <c r="W33" t="inlineStr"/>
       <c r="X33" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y33" t="inlineStr"/>
@@ -4030,19 +4062,19 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>Perfil de usuario consolidado (&gt;2 años) con historial limpio y baja frecuencia. Ausencia de contradicciones GPS o palabras críticas. El reporte de no entrega es coherente con la evidencia disponible.</t>
+          <t>Usuario con 925 días de antigüedad, historial limpio y baja frecuencia de reclamos. Sin señales de fraude detectadas.</t>
         </is>
       </c>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr"/>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil conservador y ausencia de inconsistencias operativas o de fraude. | Solicitud por retraso/no entrega en cuenta antigua sin indicadores de fraude.</t>
+          <t>APROBAR: reclamo legítimo de un usuario sin historial de fraude. | Reclamo por retraso y no entrega en cuenta antigua sin indicadores de riesgo.</t>
         </is>
       </c>
     </row>
@@ -4136,7 +4168,8 @@
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y35" t="inlineStr"/>
@@ -4240,19 +4273,19 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, sin historial de fraude y baja frecuencia de reclamos. El motivo reportado (cancelación por falta de repartidor) es un fallo operativo estándar y coherente.</t>
+          <t>Usuario con antigüedad de 988 días, 0 flags de fraude y baja frecuencia de reclamos. La justificación de cancelación operativa es coherente y no contradice la evidencia disponible.</t>
         </is>
       </c>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el perfil del usuario y sin señales de fraude. | Reclamo por cancelación operativa en cuenta antigua y confiable sin indicadores de riesgo.</t>
+          <t>APROBAR: reclamo consistente con perfil de usuario sano y sin indicadores de fraude. | Reclamo legítimo por cancelación de pedido en cuenta antigua y sin historial de riesgo.</t>
         </is>
       </c>
     </row>
@@ -4349,7 +4382,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>Cuenta con antigüedad superior a un año y un flag previo, pero el reclamo es subjetivo y la evidencia GPS es parcial, lo que impide verificar objetivamente el estado del producto.</t>
+          <t>El reclamo es subjetivo y la evidencia GPS es parcial, lo que impide verificar objetivamente el estado del producto. La existencia de un flag de fraude previo requiere validación manual.</t>
         </is>
       </c>
       <c r="X37" t="inlineStr"/>
@@ -4361,7 +4394,7 @@
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por evidencia GPS parcial y naturaleza subjetiva del reclamo, requiere revisión humana para validar fotos o reportes del restaurante/repartidor. | Reclamo por comida en mal estado sin evidencia objetiva clara ni GPS definitivo, con historial mixto.</t>
+          <t>ESCALAR: ambigüedad por GPS parcial y naturaleza subjetiva del reclamo en cuenta con flag previo. | Reclamo de calidad con evidencia limitada y historial mixto que exige revisión humana.</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4491,7 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>Usuario con 1760 días de antigüedad, 0 flags y baja frecuencia de reclamos. El motivo (espera extrema e incapacidad de contacto con el repartidor) es coherente y no presenta indicadores de fraude.</t>
+          <t>Usuario con 1760 días de antigüedad y 0 flags de fraude. El reclamo por retraso y repartidor inalcanzable es coherente con la pérdida de señal GPS. No se detectan patrones de abuso ni inconsistencias operativas.</t>
         </is>
       </c>
       <c r="X38" t="inlineStr"/>
@@ -4470,7 +4503,7 @@
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo respaldado por perfil de usuario altamente confiable y ausencia de señales de abuso o inconsistencias graves. | Reclamo por no entrega tras larga espera en cuenta antigua y confiable, con GPS perdido pero sin contradicciones operativas.</t>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y falta de evidencia GPS que refute la versión del cliente. | Cuenta antigua y limpia reporta no recepción por falla logística; la ausencia de GPS no contradice el reporte y el perfil sugiere legitimidad.</t>
         </is>
       </c>
     </row>
@@ -4567,19 +4600,19 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y frecuencia de reclamos baja. El motivo de cancelación por falta de repartidor es un evento operativo común y coherente. No se detectan indicadores de abuso o inconsistencia.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. La cancelación por falta de repartidor es un evento operativo coherente y verificable.</t>
         </is>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de fraude. | Reclamo legítimo por cancelación operativa en cuenta establecida y sin historial negativo.</t>
+          <t>APROBAR: perfil de usuario confiable con historial limpio y motivo operativo válido. | Reclamo legítimo por cancelación operativa en cuenta antigua y limpia sin inconsistencias.</t>
         </is>
       </c>
     </row>
@@ -4676,19 +4709,19 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>Perfil de usuario altamente confiable con casi 3 años de antigüedad, 0 flags y baja frecuencia de reclamos. El monto solicitado es razonable y no existen inconsistencias que sugieran fraude.</t>
+          <t>Usuario con antigüedad superior a 2 años, sin historial de fraude y baja frecuencia de reclamos. El reporte de bebida incorrecta es coherente con un fallo operativo estándar.</t>
         </is>
       </c>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con un perfil de usuario sin historial negativo y sin señales de fraude. | Error operativo de surtido en cuenta antigua y limpia, sin indicadores de riesgo o abuso.</t>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario estable y monto dentro de parámetros normales. | Reclamo por producto equivocado en cuenta antigua y confiable, sin indicadores de abuso o inconsistencia crítica.</t>
         </is>
       </c>
     </row>
@@ -4782,7 +4815,8 @@
       <c r="W41" t="inlineStr"/>
       <c r="X41" t="inlineStr">
         <is>
-          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y41" t="inlineStr"/>
@@ -4886,7 +4920,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>Usuario con 4+ años de antigüedad, sin flags de fraude y baja frecuencia de reclamos. El retraso es un incidente operativo común y coherente con la evidencia disponible.</t>
+          <t>Usuario con 1765 días de antigüedad, 0 flags y baja frecuencia de reclamos. Queja por retraso operativo coherente y sin evidencia contradictoria.</t>
         </is>
       </c>
       <c r="X42" t="inlineStr"/>
@@ -4898,7 +4932,7 @@
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y ausencia de indicadores de fraude. | Reclamo por retraso de entrega en cuenta antigua y limpia, sin inconsistencias ni señales de abuso.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo por demora en entrega de usuario histórico sin señales de fraude.</t>
         </is>
       </c>
     </row>
@@ -4995,19 +5029,19 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>Usuario con 1 flag de fraude previo y evidencia GPS parcial para un reclamo de artículos faltantes que requiere verificación manual.</t>
+          <t>Cuenta con 1 flag de fraude previo y evidencia GPS parcial para un reclamo de artículos faltantes difícil de verificar objetivamente.</t>
         </is>
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | evidencia_gps_parcial</t>
+          <t>flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>ESCALAR: presencia de flag de fraude previo y GPS parcial requieren validación humana del inventario faltante. | Reclamo por falta de salsas y cubiertos en cuenta con historial mixto y cobertura GPS incompleta.</t>
+          <t>ESCALAR: combinación de flag de fraude previo, GPS parcial y naturaleza subjetiva del reclamo requiere revisión humana para evitar errores operativos o falsos positivos. | Reclamo por falta de salsas y cubiertos en cuenta con historial mixto y GPS inconclusa.</t>
         </is>
       </c>
     </row>
@@ -5089,7 +5123,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>APROBAR</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5099,20 +5133,24 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>APROBAR</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>Perfil de usuario altamente confiable (cuenta antigua, 0 flags, baja frecuencia). La ausencia de evidencia GPS genera ambigüedad operativa que impide la validación automática.</t>
+          <t>Usuario con 1796 días de antigüedad y 0 flags de fraude. Aunque la evidencia GPS está perdida, el perfil extremadamente conservador y la baja frecuencia de reclamos indican un incidente operativo legítimo.</t>
         </is>
       </c>
       <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
+      <c r="Y44" t="inlineStr">
+        <is>
+          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
+        </is>
+      </c>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>ESCALAR: evidencia GPS insuficiente ('señal perdida') requiere revisión manual de registros del repartidor para confirmar ubicación de entrega. | Disputa de entrega sin rastreo GPS en cuenta limpia y antigua.</t>
+          <t>APROBAR: perfil de usuario altamente confiable y sin señales de abuso que justifican la compensación pese a la falta de validación GPS. | Reclamo por entrega no recibida en cuenta veterana sin antecedentes, con evidencia GPS incompleta.</t>
         </is>
       </c>
     </row>
@@ -5209,7 +5247,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>Usuario con 510 días de antigüedad, historial limpio y 0 reclamos recientes. El motivo de cancelación del restaurante es coherente y el monto solicitado está dentro de parámetros normales.</t>
+          <t>Usuario con 510 días de antigüedad, 0 flags de fraude y 0 reclamos recientes. El motivo descrito corresponde a un error de facturación estándar por cancelación del restaurante, sin inconsistencias ni señales de riesgo.</t>
         </is>
       </c>
       <c r="X45" t="inlineStr"/>
@@ -5221,7 +5259,7 @@
       <c r="Z45" t="inlineStr"/>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con evidencia operativa, usuario sin señales de fraude ni patrones abusivos. | Reclamo operativo por cancelación de restaurante y cobro pendiente en cuenta establecida sin historial de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con la evidencia disponible y perfil de usuario confiable. | Cobro indebido por cancelación operativa en cuenta estable y sin historial de fraude.</t>
         </is>
       </c>
     </row>
@@ -5318,7 +5356,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>Usuario con 1706 días de antigüedad y 0 flags de fraude. El reclamo por discrepancia de cobro es coherente con errores operativos comunes y no presenta indicadores de abuso.</t>
+          <t>Usuario con 4+ años de antigüedad y 0 flags de fraude. Reclamo de discrepancia monetaria sin indicadores de abuso o inconsistencia crítica.</t>
         </is>
       </c>
       <c r="X46" t="inlineStr"/>
@@ -5330,7 +5368,7 @@
       <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente de usuario confiable sin patrones de fraude. | Discrepancia de cobro en cuenta antigua y limpia sin señales de riesgo.</t>
+          <t>APROBAR: reclamo operativo legítimo de usuario con historial limpio y baja frecuencia. | Discrepancia de cobro en cuenta antigua y confiable, sin señales de fraude ni palabras críticas.</t>
         </is>
       </c>
     </row>
@@ -5424,7 +5462,12 @@
       <c r="W47" t="inlineStr"/>
       <c r="X47" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y47" t="inlineStr"/>
@@ -5525,7 +5568,10 @@
       <c r="W48" t="inlineStr"/>
       <c r="X48" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y48" t="inlineStr"/>
@@ -5629,19 +5675,19 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>Usuario con 4+ años de antigüedad y 0 flags de fraude. Reclamo por cancelación operativa sin inconsistencias ni señales de abuso.</t>
+          <t>Usuario de larga antigüedad (1655d) sin historial de fraude ni alta frecuencia de reclamos. El motivo de cancelación por falta de repartidor es coherente con un error operativo estándar. No se activaron reglas de riesgo ni palabras críticas.</t>
         </is>
       </c>
       <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr"/>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario sin riesgos. | Solicitud de reembolso por cancelación de pedido sin repartidor en cuenta antigua y confiable.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin indicios de fraude. | Reclamo por cancelación operativa en cuenta confiable sin señales de abuso o inconsistencias.</t>
         </is>
       </c>
     </row>
@@ -5735,7 +5781,8 @@
       <c r="W50" t="inlineStr"/>
       <c r="X50" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y50" t="inlineStr"/>
@@ -5839,15 +5886,19 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>Usuario con 306 días de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La discrepancia de monto es un error operativo estándar verificable por sistema.</t>
+          <t>Perfil limpio con antigüedad &gt;8 meses y baja frecuencia. Discrepancia de cobro típica sin indicadores de fraude.</t>
         </is>
       </c>
       <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
+      <c r="Y51" t="inlineStr">
+        <is>
+          <t>reclamo_subjetivo | evidencia_gps_parcial</t>
+        </is>
+      </c>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de tipo financiero sin indicadores de fraude. | Reclamo por diferencia en resumen de cargo. Perfil conservador sin señales de riesgo.</t>
+          <t>APROBAR: reclamo de discrepancia administrativa sin señales de abuso o inconsistencia crítica. | Reclamo por diferencia de monto en resumen. Usuario con historial estable y GPS parcial no relevante para el tipo de incidencia.</t>
         </is>
       </c>
     </row>
@@ -5944,15 +5995,19 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad de 906 días, sin flags de fraude y sin reclamos recientes. El reporte de artículos faltantes es un error operativo común y coherente, sin contradicciones con la evidencia disponible.</t>
+          <t>Usuario con más de 2 años de antigüedad, 0 flags y 0 reclamos recientes. El reclamo por artículos faltantes es un error operativo común y coherente. La ausencia de GPS no aplica a este tipo de incidencia.</t>
         </is>
       </c>
       <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>reclamo_subjetivo</t>
+        </is>
+      </c>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Incidencia operativa por falta de salsas y cubiertos en cuenta antigua y sin historial de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Reclamo estándar de artículos faltantes en cuenta antigua y limpia sin indicadores de riesgo.</t>
         </is>
       </c>
     </row>
@@ -6046,7 +6101,8 @@
       <c r="W53" t="inlineStr"/>
       <c r="X53" t="inlineStr">
         <is>
-          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y53" t="inlineStr"/>
@@ -6150,19 +6206,19 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La pérdida de señal GPS impide verificar la entrega, pero la narrativa es coherente y el perfil es conservador.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. Aunque la evidencia GPS está ausente, el perfil del usuario es conservador y el reclamo es coherente con disputas operativas comunes.</t>
         </is>
       </c>
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable sin señales de fraude, la ausencia de GPS se compensa con historial positivo y narrativa plausible. | Reclamo por entrega no recibida en cuenta antigua y limpia, sin evidencia GPS contradictoria.</t>
+          <t>APROBAR: perfil de usuario confiable sin señales de fraude, se compensa ante la falta de evidencia GPS concluyente. | Reclamo por entrega marcada incorrectamente en cuenta antigua y limpia, sin evidencia GPS disponible para verificación objetiva.</t>
         </is>
       </c>
     </row>
@@ -6256,7 +6312,8 @@
       <c r="W55" t="inlineStr"/>
       <c r="X55" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y55" t="inlineStr"/>
@@ -6357,7 +6414,8 @@
       <c r="W56" t="inlineStr"/>
       <c r="X56" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y56" t="inlineStr"/>
@@ -6461,19 +6519,19 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>Usuario con flag de fraude previo y 6 reclamos en 90 días. Ratio de compensación elevado (0.81) sin evidencia GPS que respalde la cancelación reportada.</t>
+          <t>Alta frecuencia de reclamos (6 en 90d) combinada con flag de fraude previo y ausencia de evidencia GPS valida.</t>
         </is>
       </c>
       <c r="X57" t="inlineStr"/>
       <c r="Y57" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z57" t="inlineStr"/>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>RECHAZAR: evidencia clara de abuso por historial con flag previo, alta frecuencia de reclamos y ratio de compensación elevado sin validación técnica. | Patrón de abuso confirmado por alta frecuencia, historial negativo y compensación desproporcionada sin soporte técnico.</t>
+          <t>RECHAZAR: patrón de alta frecuencia y flag de fraude previo sin corroboración GPS. | Reclamo por cancelación operativa en cuenta con historial de reincidencia y sin validación geolocal.</t>
         </is>
       </c>
     </row>
@@ -6570,19 +6628,19 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>Usuario con 373 días de antigüedad y 0 flags de fraude. Frecuencia de reclamos moderada y ratio de compensación aceptable. La evidencia GPS es parcial pero no contradice el reporte, y el reclamo por calidad alimentaria es coherente con el contexto.</t>
+          <t>Usuario con antigüedad de 373 días y 0 flags de fraude. El reclamo por calidad de alimento es coherente y el monto está dentro de parámetros normales. La evidencia GPS es parcial pero no contradice el reporte.</t>
         </is>
       </c>
       <c r="X58" t="inlineStr"/>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo | entrega_gps_parcial</t>
+          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z58" t="inlineStr"/>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo por calidad de producto en cuenta sana con evidencia GPS ambigua pero sin inconsistencias.</t>
+          <t>APROBAR: reclamo legítimo sin indicadores de fraude, consistente con políticas de compensación por calidad. | Reclamo por estado del alimento en cuenta antigua y limpia, sin patrones de abuso.</t>
         </is>
       </c>
     </row>
@@ -6676,7 +6734,10 @@
       <c r="W59" t="inlineStr"/>
       <c r="X59" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y59" t="inlineStr"/>
@@ -6777,7 +6838,8 @@
       <c r="W60" t="inlineStr"/>
       <c r="X60" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y60" t="inlineStr"/>
@@ -6878,7 +6940,8 @@
       <c r="W61" t="inlineStr"/>
       <c r="X61" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y61" t="inlineStr"/>
@@ -6979,7 +7042,12 @@
       <c r="W62" t="inlineStr"/>
       <c r="X62" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R2 — Compensación solicitada &gt; 99% del valor de la orden; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R2 — Compensación solicitada &gt; 99% del valor de la orden
+Pide como compensación más del 99% del valor de la orden, cuando lo típico es ~80%. Pedir el valor completo es señal de fraude.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y62" t="inlineStr"/>
@@ -7080,7 +7148,12 @@
       <c r="W63" t="inlineStr"/>
       <c r="X63" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d
+Cuenta nueva (&lt; 90 días) con récord de reclamos: la señal de fraude más fuerte del dataset.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y63" t="inlineStr"/>
@@ -7181,7 +7254,8 @@
       <c r="W64" t="inlineStr"/>
       <c r="X64" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y64" t="inlineStr"/>
@@ -7285,19 +7359,19 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>Usuario con flag de fraude previo y GPS sin señal. El reclamo por discrepancia de cobro requiere validación manual de logs internos.</t>
+          <t>Reclamo de discrepancia de cargo con GPS perdido y un flag de fraude previo. La falta de evidencia geolocalizada y el historial mixto impiden una decisión automatizada segura.</t>
         </is>
       </c>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada | flag_fraude_previo | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>ESCALAR: requiere auditoría manual para conciliar cobros y evaluar impacto del flag previo ante GPS perdida. | Discrepancia monetaria en cuenta con historial de riesgo y sin evidencia geolocalizable.</t>
+          <t>ESCALAR: ambigüedad por GPS perdido y flag previo en reclamo de facturación requiere revisión humana. | Disputa de facturación con evidencia GPS insuficiente y antecedentes de riesgo moderado que requieren validación manual.</t>
         </is>
       </c>
     </row>
@@ -7379,7 +7453,7 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -7389,24 +7463,24 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>Cuenta con 1 flag de fraude previo y 6 reclamos en 90 días. La evidencia GPS está perdida y el motivo (comida fría) es subjetivo y difícil de verificar objetivamente.</t>
+          <t>Cuenta con 1 flag de fraude previo y 6 reclamos en 90 días. La señal GPS perdida imposibilita verificar el retraso alegado, y el estado 'fría' es subjetivo. Se requiere análisis humano para equilibrar riesgo de fraude con posible queja legítima.</t>
         </is>
       </c>
       <c r="X66" t="inlineStr"/>
       <c r="Y66" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>RECHAZAR: patrón de alta frecuencia combinado con flag de fraude previo y ausencia de evidencia GPS objetiva valida el rechazo por posible abuso. | Reclamo por temperatura del pedido sin soporte GPS verificable en usuario con historial de fraude y alta frecuencia.</t>
+          <t>ESCALAR: combinación de alta frecuencia de reclamos, flag de fraude previo y falta de evidencia GPS objetiva requiere revisión manual para determinar legitimidad. | Reclamo por retraso y temperatura inadecuada en cuenta con historial de riesgo y evidencia GPS incompleta.</t>
         </is>
       </c>
     </row>
@@ -7503,7 +7577,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, sin flags de fraude y baja frecuencia de reclamos. El error en la aplicación del cupón es un incidente operativo coherente y verificable.</t>
+          <t>Usuario con más de 2 años de antigüedad y 0 flags de fraude. El reclamo por error de cupón es coherente y no activa umbrales de riesgo operativos.</t>
         </is>
       </c>
       <c r="X67" t="inlineStr"/>
@@ -7515,7 +7589,7 @@
       <c r="Z67" t="inlineStr"/>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable. | Error técnico en descuento en cuenta antigua sin historial negativo.</t>
+          <t>APROBAR: reclamo legítimo de usuario confiable sin inconsistencias ni riesgos detectados. | Disputa por descuento no aplicado en cuenta antigua sin historial de abuso.</t>
         </is>
       </c>
     </row>
@@ -7612,7 +7686,7 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. El reclamo por ítem faltante es un error operativo común y coherente. No se activaron reglas de riesgo ni hay señales de abuso.</t>
+          <t>Usuario con antigüedad superior a 4 años, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado es razonable y no contiene palabras críticas. La falta de confirmación GPS no contradice el reporte de ítem faltante.</t>
         </is>
       </c>
       <c r="X68" t="inlineStr"/>
@@ -7624,7 +7698,7 @@
       <c r="Z68" t="inlineStr"/>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin señales de fraude. | Error operativo de restaurante (bebida faltante) en usuario confiable de larga data sin patrones sospechosos.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo por producto faltante en cuenta antigua y sin historial de riesgo.</t>
         </is>
       </c>
     </row>
@@ -7718,7 +7792,10 @@
       <c r="W69" t="inlineStr"/>
       <c r="X69" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.</t>
         </is>
       </c>
       <c r="Y69" t="inlineStr"/>
@@ -7822,7 +7899,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>Cuenta antigua con 0 flags y baja frecuencia. Monto y ratio dentro de parámetros normales. Sin contradicciones ni términos críticos.</t>
+          <t>Usuario con más de 3 años de antigüedad y sin historial de fraude. El reclamo por doble cobro es un error financiero verificable, sin patrones de abuso ni inconsistencias.</t>
         </is>
       </c>
       <c r="X70" t="inlineStr"/>
@@ -7834,7 +7911,7 @@
       <c r="Z70" t="inlineStr"/>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario sano y consolidado sin señales de fraude detectadas. | Reclamo por doble cobro en usuario consolidado sin indicadores de riesgo operativo.</t>
+          <t>APROBAR: reclamo legítimo de usuario con trayectoria consolidada y sin indicadores de fraude. | Duplicidad de cobro reportada en cuenta antigua y confiable, sin señales de riesgo.</t>
         </is>
       </c>
     </row>
@@ -7931,19 +8008,19 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>Usuario con 1660 días de antigüedad y 0 flags de fraude. Reclamo por error de cupón sin señales de inconsistencia o abuso.</t>
+          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. El reclamo por error de cupón es un incidente operativo común y coherente.</t>
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z71" t="inlineStr"/>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario antiguo sin historial de fraude ni patrones sospechosos. | Error operativo en la aplicación de descuento para cuenta confiable de larga data.</t>
+          <t>APROBAR: reclamo legítimo sin señales de fraude ni inconsistencias operativas. | Error técnico en la aplicación de descuento para cuenta confiable de larga data.</t>
         </is>
       </c>
     </row>
@@ -8040,19 +8117,19 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>Historial con flag de fraude previo, alta frecuencia de reclamos y ratio de compensación elevado sugieren patrón de abuso.</t>
+          <t>Usuario con flag de fraude previo, alta frecuencia de reclamos (4 en 90d) y ratio de compensación elevado (0.91). Ausencia de evidencia GPS que valide la entrega o el faltante reportado.</t>
         </is>
       </c>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | alta_frecuencia_reclamos | compensacion_elevada | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | compensacion_elevada | alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z72" t="inlineStr"/>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>RECHAZAR: combinación de flag de fraude previo, alta frecuencia de reclamos y ratio de compensación elevado indica riesgo de abuso sistemático. | Reclamo por faltantes sin evidencia verificable en usuario con historial de riesgo y alta tasa de compensaciones.</t>
+          <t>RECHAZAR: combinación de flag de fraude, alta frecuencia y ratio de compensación elevado sin evidencia GPS confirma patrón de abuso. | Reclamo por artículos faltantes en cuenta con historial de riesgo y ratio de compensación alto, sin soporte geoespacial.</t>
         </is>
       </c>
     </row>
@@ -8149,12 +8226,13 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>El reclamo contiene la palabra 'alergia', lo que activa la regla de palabras críticas de seguridad de marca. Aunque el usuario tiene un perfil limpio y antigüedad alta, la mención de un riesgo de salud requiere revisión humana para evitar responsabilidades legales o daños a la reputación.</t>
+          <t>El reclamo contiene el término 'alergia', un indicador crítico de riesgo sanitario y legal que activa protocolos de seguridad de marca y exige revisión humana.</t>
         </is>
       </c>
       <c r="X73" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y73" t="inlineStr">
@@ -8169,7 +8247,7 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>ESCALAR: mención de término crítico ('alergia') que implica riesgo de salud y requiere validación humana antes de resolver. | Reclamo por error de restaurante en cuenta antigua, pero la mención de alergia obliga a escalar por protocolo de seguridad y salud.</t>
+          <t>ESCALAR: mención de término crítico de salud que implica responsabilidad legal y sanitaria, requiriendo validación manual conforme a políticas de seguridad de marca. | Usuario antiguo sin historial de fraude reporta error en pedido por alergia alimentaria. Aunque el perfil es sano y la frecuencia es baja, la mención de riesgo de salud obliga a escalar.</t>
         </is>
       </c>
     </row>
@@ -8266,7 +8344,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años y 0 flags de fraude. Reclamo por ítem incorrecto sin señales de abuso o inconsistencia crítica.</t>
+          <t>Usuario con antigüedad superior a 4 años, sin flags de fraude y baja frecuencia de reclamos. El error de entrega coincide con un incidente operativo común.</t>
         </is>
       </c>
       <c r="X74" t="inlineStr"/>
@@ -8278,7 +8356,7 @@
       <c r="Z74" t="inlineStr"/>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Error operativo menor en cuenta antigua y limpia. Sin evidencia de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por producto incorrecto en cuenta antigua y sin historial de riesgo. Sin inconsistencias ni señales de abuso.</t>
         </is>
       </c>
     </row>
@@ -8375,17 +8453,18 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas de seguridad de marca que requiere revisión humana inmediata para mitigar riesgos sanitarios y legales.</t>
+          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas que exige revisión humana por implicaciones de salud y responsabilidad civil. Aunque el usuario tiene un flag de fraude previo y GPS no confirmado, el riesgo de marca/salud domina la decisión.</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y75" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad</t>
+          <t>palabras_criticas_seguridad | flag_fraude_previo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z75" t="inlineStr">
@@ -8395,7 +8474,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabra crítica ('alergia') que implica riesgo de salud/legal, requiriendo validación humana según protocolo de seguridad de marca. | Reclamo por posible reacción alérgica en cuenta con 1 flag previo y GPS no confirmada, escalado automáticamente por término crítico de salud.</t>
+          <t>ESCALAR: contiene palabra crítica 'alergia' que implica riesgo de salud y posible responsabilidad legal, requiriendo validación humana obligatoria según política de marca. | Reclamo por alergia alimentaria en cuenta con historial mixto y sin evidencia GPS, sujeto a revisión por riesgo legal y de salud.</t>
         </is>
       </c>
     </row>
@@ -8489,7 +8568,10 @@
       <c r="W76" t="inlineStr"/>
       <c r="X76" t="inlineStr">
         <is>
-          <t>R2 — Compensación solicitada &gt; 99% del valor de la orden; R4 — Compensación solicitada &gt; p99 del dataset original</t>
+          <t>R2 — Compensación solicitada &gt; 99% del valor de la orden
+Pide como compensación más del 99% del valor de la orden, cuando lo típico es ~80%. Pedir el valor completo es señal de fraude.
+R4 — Compensación solicitada &gt; p99 del dataset original
+Solo el 1% de las compensaciones supera este monto: es atípico y se rechaza automáticamente.</t>
         </is>
       </c>
       <c r="Y76" t="inlineStr"/>
@@ -8593,19 +8675,19 @@
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>Perfil de usuario limpio sin historial de fraude ni alta frecuencia. La pérdida de señal GPS impide verificar objetivamente la entrega, generando ambigüedad.</t>
+          <t>GPS perdido impide verificar la entrega. Usuario con antigüedad y perfil limpio, pero la falta de evidencia objetiva genera ambigüedad.</t>
         </is>
       </c>
       <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z77" t="inlineStr"/>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>ESCALAR: ausencia de evidencia GPS objetiva requiere validación manual para evitar errores operativos o fraude encubierto. | Reclamo por no recepción con evidencia geolocalizada ausente en cuenta con historial conservador.</t>
+          <t>ESCALAR: evidencia GPS perdida genera ambigüedad que requiere revisión humana para validar la entrega. | Reclamo de no recepción con señal GPS perdida y sin indicadores de fraude, requiriendo validación manual.</t>
         </is>
       </c>
     </row>
@@ -8702,7 +8784,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>Usuario con 4+ años de antigüedad y perfil limpio sin reclamos previos. El retraso reportado es coherente y no presenta indicadores de fraude.</t>
+          <t>Usuario con antigüedad superior a 4 años, sin historial de fraude ni reclamos recientes. El retraso reportado es un incidente operativo común y coherente con la promesa de entrega.</t>
         </is>
       </c>
       <c r="X78" t="inlineStr"/>
@@ -8714,7 +8796,7 @@
       <c r="Z78" t="inlineStr"/>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario con historial impecable y sin señales de abuso. | Reclamo por retraso de entrega en cuenta antigua y confiable. Señal GPS perdida pero sin contradicción con el reporte.</t>
+          <t>APROBAR: reclamo legítimo basado en perfil de alto riesgo negativo y motivo operativo coherente. | Reclamo por retraso en entrega de usuario veterano y confiable. Sin señales de abuso o contradicciones graves.</t>
         </is>
       </c>
     </row>
@@ -8808,7 +8890,8 @@
       <c r="W79" t="inlineStr"/>
       <c r="X79" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y79" t="inlineStr"/>
@@ -8909,7 +8992,10 @@
       <c r="W80" t="inlineStr"/>
       <c r="X80" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y80" t="inlineStr"/>
@@ -9010,7 +9096,8 @@
       <c r="W81" t="inlineStr"/>
       <c r="X81" t="inlineStr">
         <is>
-          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y81" t="inlineStr"/>
@@ -9111,7 +9198,8 @@
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y82" t="inlineStr"/>
@@ -9215,7 +9303,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años, sin flags de fraude y frecuencia baja de reclamos. El retraso reportado es un motivo válido y el monto solicitado está dentro del rango normal.</t>
+          <t>Usuario antiguo (1598d) sin flags de fraude y baja frecuencia de reclamos. El retraso de 1.5h es una causa coherente para que la comida pierda calidad. Monto dentro de límites y ratio aceptable.</t>
         </is>
       </c>
       <c r="X83" t="inlineStr"/>
@@ -9227,7 +9315,7 @@
       <c r="Z83" t="inlineStr"/>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en historial limpio, antigüedad alta y monto dentro de parámetros normales. | Reclamo por retraso en entrega en cuenta antigua y limpia, consistente con el perfil del usuario.</t>
+          <t>APROBAR: reclamo legítimo basado en historial positivo, monto controlado y justificación coherente con el retraso reportado. | Reclamo por retraso y calidad en cuenta antigua y limpia. Sin inconsistencias ni señales de abuso.</t>
         </is>
       </c>
     </row>
@@ -9324,19 +9412,19 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>Usuario con 474 días de antigüedad, 0 flags de fraude y frecuencia de reclamos dentro de lo normal. Al no existir evidencia GPS que confirme la entrega, no hay contradicción objetiva que respalde un rechazo.</t>
+          <t>Usuario con 474 días de antigüedad y 0 flags de fraude. La evidencia GPS no confirma la entrega, por lo que no existe contradicción objetiva con su reporte. Bajo riesgo de abuso.</t>
         </is>
       </c>
       <c r="X84" t="inlineStr"/>
       <c r="Y84" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y ausencia de señales de abuso. | Disputa de entrega no verificable por GPS en cuenta con historial limpio y monto razonable.</t>
+          <t>APROBAR: reclamo legítimo sin señales de fraude ni evidencia contradictoria. | Disputa por entrega no recibida en cuenta limpia con evidencia GPS inconclusa.</t>
         </is>
       </c>
     </row>
@@ -9430,7 +9518,8 @@
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y85" t="inlineStr"/>
@@ -9534,19 +9623,19 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>Usuario con 704 días de antigüedad y 0 flags de fraude. El motivo de cancelación por falta de repartidor es operativo y coherente. No se activan reglas de fraude, el monto solicitado está dentro del umbral y la frecuencia es baja.</t>
+          <t>Usuario con antigüedad estable (704d), historial limpio y baja frecuencia. El motivo de cancelación por falta de repartidor es coherente y el monto solicitado es razonable. La pérdida de señal GPS no contradice la evidencia operativa.</t>
         </is>
       </c>
       <c r="X86" t="inlineStr"/>
       <c r="Y86" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z86" t="inlineStr"/>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude, consistente con el contexto operativo y perfil de usuario sano. | Reclamo operativo estándar por cancelación de plataforma en cuenta antigua y sin historial negativo.</t>
+          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario confiable. | Reclamo operativo estándar por cancelación de pedido en cuenta estable sin señales de fraude.</t>
         </is>
       </c>
     </row>
@@ -9643,7 +9732,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, 0 flags de fraude y baja frecuencia de reclamos. La narrativa de espera prolongada y falta de respuesta del conductor es coherente con la pérdida de señal GPS reportada.</t>
+          <t>Usuario antiguo (1222d) con 0 flags y baja frecuencia de reclamos. Aunque la señal GPS se perdió, la coherencia del reporte y el perfil conservador del cliente respaldan la acción.</t>
         </is>
       </c>
       <c r="X87" t="inlineStr"/>
@@ -9655,7 +9744,7 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario antiguo sin señales de fraude, narrativa coherente ante ausencia de datos GPS. | Reclamo por entrega no completada en cuenta confiable y antigua, sin evidencia GPS pero con perfil limpio y relato consistente.</t>
+          <t>APROBAR: perfil de alto confianza sin contradicciones graves, se autoriza ante ausencia de evidencia GPS que refute el reclamo. | Reclamo por no entrega/retraso en cuenta confiable con evidencia GPS ausente pero sin indicadores de fraude.</t>
         </is>
       </c>
     </row>
@@ -9749,7 +9838,12 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y88" t="inlineStr"/>
@@ -9853,7 +9947,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>Usuario con 522 días de antigüedad y historial limpio. Reclamo por producto faltante sin contradicciones ni señales de fraude.</t>
+          <t>Usuario con 522 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El perfil es conservador y no presenta indicadores de abuso. Aunque el GPS no confirma la entrega, la ausencia de señales de riesgo y la naturaleza del reclamo apuntan a un error operativo legítimo.</t>
         </is>
       </c>
       <c r="X89" t="inlineStr"/>
@@ -9865,7 +9959,7 @@
       <c r="Z89" t="inlineStr"/>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Reclamo operativo estándar en cuenta verificada sin patrones abusivos.</t>
+          <t>APROBAR: perfil de usuario confiable sin historial de fraude o alta frecuencia, se aprueba como error operativo. | Reclamo por producto faltante en cuenta limpia y antigua, sin evidencia GPS pero sin patrones sospechosos.</t>
         </is>
       </c>
     </row>
@@ -9959,7 +10053,8 @@
       <c r="W90" t="inlineStr"/>
       <c r="X90" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y90" t="inlineStr"/>
@@ -10063,19 +10158,19 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>Usuario con 757 días de antigüedad, 0 flags y 1 reclamo en 90 días. La cancelación por falta de repartidor es un evento operativo coherente. No hay contradicciones GPS ni palabras críticas.</t>
+          <t>Usuario antiguo (757d) con historial limpio y baja frecuencia. Cancelación por falta de repartidor es un evento operativo coherente y sin contradicciones.</t>
         </is>
       </c>
       <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>antiguedad_moderada_con_alta_reincidencia</t>
         </is>
       </c>
       <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario confiable. | Reclamo estándar por cancelación operativa en cuenta antigua y sin historial de riesgo.</t>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y motivo operativo coherente. | Reclamo por cancelación operativa en cuenta estable sin señales de fraude o inconsistencias.</t>
         </is>
       </c>
     </row>
@@ -10169,7 +10264,8 @@
       <c r="W92" t="inlineStr"/>
       <c r="X92" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y92" t="inlineStr"/>
@@ -10258,7 +10354,7 @@
       </c>
       <c r="T93" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U93" t="inlineStr">
@@ -10268,24 +10364,24 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>Usuario con flag de fraude previo y GPS sin señal que impide validar entrega. Reclamo subjetivo sin evidencia corroborante.</t>
+          <t>Antecedente de fraude previo combinado con pérdida de señal GPS crea ambigüedad crítica para la validación automática.</t>
         </is>
       </c>
       <c r="X93" t="inlineStr"/>
       <c r="Y93" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z93" t="inlineStr"/>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>RECHAZAR: flag de fraude previo combinado con GPS perdido y falta de evidencia objetiva para validar la no entrega. | Reclamo por no llegada de pedido en cuenta con historial de fraude y sin rastreo GPS válido.</t>
+          <t>ESCALAR: ambigüedad por evidencia GPS parcial y riesgo histórico requieren revisión manual. | Reclamo por no entrega con GPS perdido y flag histórico de fraude que impide confirmación objetiva.</t>
         </is>
       </c>
     </row>
@@ -10379,7 +10475,8 @@
       <c r="W94" t="inlineStr"/>
       <c r="X94" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y94" t="inlineStr"/>
@@ -10483,7 +10580,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, sin flags de fraude, baja frecuencia de reclamos y monto solicitado dentro de parámetros normales. La descripción es coherente con un problema operativo o de calidad.</t>
+          <t>Usuario con antigüedad superior a 2 años, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado está dentro de parámetros normales y la queja por calidad de alimento es coherente con el perfil.</t>
         </is>
       </c>
       <c r="X95" t="inlineStr"/>
@@ -10495,7 +10592,7 @@
       <c r="Z95" t="inlineStr"/>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por calidad de producto en cuenta antigua y sin historial negativo.</t>
+          <t>APROBAR: reclamo legítimo de usuario con historial limpio y métricas dentro de lo esperado. | Reclamo por deterioro de alimento en cuenta confiable sin inconsistencias operativas ni señales de abuso.</t>
         </is>
       </c>
     </row>
@@ -10589,7 +10686,12 @@
       <c r="W96" t="inlineStr"/>
       <c r="X96" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y96" t="inlineStr"/>
@@ -10693,7 +10795,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y frecuencia de reclamos baja. El reporte de faltante es un error operativo común y coherente.</t>
+          <t>Usuario con antigüedad superior a 3 años, 0 flags de fraude y baja frecuencia de reclamos. El faltante de productos es un error operativo común sin señales de abuso.</t>
         </is>
       </c>
       <c r="X97" t="inlineStr"/>
@@ -10705,7 +10807,7 @@
       <c r="Z97" t="inlineStr"/>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude o inconsistencias operativas. | Reclamo por faltante de producto en cuenta antigua y confiable, sin indicadores de riesgo ni inconsistencias.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por faltante de ítems en cuenta antigua y sin historial negativo.</t>
         </is>
       </c>
     </row>
@@ -10802,19 +10904,19 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>Cuenta nueva (80d) con flag de fraude previo y 3 reclamos en 90d. Ausencia de evidencia GPS que valide el error operativo. Patrón consistente con riesgo de abuso.</t>
+          <t>Cuenta nueva (80d) con 3 reclamos en 90d y 1 flag de fraude previo. Sin evidencia GPS que valide el caso.</t>
         </is>
       </c>
       <c r="X98" t="inlineStr"/>
       <c r="Y98" t="inlineStr">
         <is>
-          <t>antiguedad_moderada_con_alta_reincidencia | flag_fraude_previo | entrega_gps_no_confirmada</t>
+          <t>account_abuse | flag_fraude_previo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z98" t="inlineStr"/>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>RECHAZAR: cuenta nueva con flag de fraude previo y alta frecuencia de reclamos sin evidencia GPS que respalde el caso. | Reclamo por producto equivocado en cuenta reciente con historial negativo y sin validación geolocalizada.</t>
+          <t>RECHAZAR: cuenta nueva con alta frecuencia de reclamos y flag de fraude previo, sin evidencia GPS que respalde la inconsistencia. | Reclamo por error de producto en perfil de alto riesgo sin validación geoespacial.</t>
         </is>
       </c>
     </row>
@@ -10911,7 +11013,7 @@
       </c>
       <c r="W99" t="inlineStr">
         <is>
-          <t>Cuenta con antigüedad moderada y sin flags de fraude, pero presenta GPS parcial que impide validar la cancelación del restaurante, sumado a un ratio de compensación elevado y frecuencia de reclamos notable en 90 días.</t>
+          <t>Evidencia GPS parcial y ratio de compensación alto generan ambigüedad para validar cancelación real sin revisión humana.</t>
         </is>
       </c>
       <c r="X99" t="inlineStr"/>
@@ -10923,7 +11025,7 @@
       <c r="Z99" t="inlineStr"/>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>ESCALAR: evidencia GPS parcial y métricas elevadas (ratio y frecuencia) impiden decisión automatizada segura. | Reclamo por cargo no reflejado tras supuesta cancelación del restaurante. Evidencia GPS ambigua y métricas de riesgo moderado requieren validación manual.</t>
+          <t>ESCALAR: inconsistencia en evidencia GPS y ratio de compensación elevado requieren validación manual. | Reclamo por cargo tras cancelación del restaurante con GPS incompleto y historial de compensaciones frecuente.</t>
         </is>
       </c>
     </row>
@@ -11017,7 +11119,8 @@
       <c r="W100" t="inlineStr"/>
       <c r="X100" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y100" t="inlineStr"/>
@@ -11118,7 +11221,8 @@
       <c r="W101" t="inlineStr"/>
       <c r="X101" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y101" t="inlineStr"/>
@@ -11222,19 +11326,19 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>Reclamo subjetivo sobre estado del producto con evidencia GPS parcial y un flag de fraude previo. La ambigüedad en la verificación objetiva y el historial mixto requieren revisión humana.</t>
+          <t>Reclamo subjetivo difícil de verificar objetivamente. La combinación de un flag de fraude previo, evidencia GPS parcial y la naturaleza sensorial del reporte genera ambigüedad que excede la automatización.</t>
         </is>
       </c>
       <c r="X102" t="inlineStr"/>
       <c r="Y102" t="inlineStr">
         <is>
-          <t>evidencia_gps_parcial | reclamo_subjetivo | flag_fraude_previo</t>
+          <t>reclamo_subjetivo | flag_fraude_previo | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por GPS parcial, naturaleza subjetiva del reclamo y flag de fraude previo requieren validación manual. | Caso con reclamo subjetivo, GPS parcial y antecedente de fraude que impide decisión automatizada segura.</t>
+          <t>ESCALAR: ambigüedad por naturaleza subjetiva del reclamo, flag de fraude previo y GPS parcial requieren validación manual. | Solicitud por olor a comida descompuesta en cuenta con antigüedad moderada, historial con flag de fraude y geolocalización incompleta.</t>
         </is>
       </c>
     </row>
@@ -11331,15 +11435,19 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, historial limpio y sin reclamos recientes. La justificación por cancelación operativa es coherente y el monto solicitado se ajusta al promedio.</t>
+          <t>Perfil de usuario limpio con 821 días de antigüedad y sin historial de fraude. Reclamo por cancelación operativa sin señales de abuso o inconsistencia crítica.</t>
         </is>
       </c>
       <c r="X103" t="inlineStr"/>
-      <c r="Y103" t="inlineStr"/>
+      <c r="Y103" t="inlineStr">
+        <is>
+          <t>entrega_gps_no_confirmada</t>
+        </is>
+      </c>
       <c r="Z103" t="inlineStr"/>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo legítimo por cancelación de servicio sin señales de fraude o inconsistencias operativas.</t>
+          <t>APROBAR: reclamo operativo consistente con perfil de usuario sano y sin indicadores de fraude. | Solicitud de reembolso por cancelación de pedido sin repartidor en cuenta confiable sin actividad sospechosa reciente.</t>
         </is>
       </c>
     </row>
@@ -11436,19 +11544,19 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>Usuario con 541 días de antigüedad, 0 flags y 0 reclamos recientes. La solicitud de reembolso por cancelación operativa es coherente y el monto solicitado está dentro del rango normal. Al no existir contradicciones GPS ni indicadores de abuso, se considera legítimo.</t>
+          <t>Usuario con 541 días de antigüedad y 0 flags de fraude. El motivo de cancelación por falta de repartidor es operativamente coherente y el monto solicitado es razonable. No se detectan patrones de abuso ni inconsistencias críticas.</t>
         </is>
       </c>
       <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z104" t="inlineStr"/>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Reembolso por cancelación de pedido sin repartidor en cuenta sana sin historial de fraude.</t>
+          <t>APROBAR: reclamo legítimo sin señales de fraude, consistente con el contexto operativo y perfil de usuario confiable. | Solicitud de reembolso por cancelación operativa en cuenta antigua sin historial de reclamos.</t>
         </is>
       </c>
     </row>
@@ -11545,7 +11653,7 @@
       </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>Usuario con casi 4 años de antigüedad y historial limpio. Reclamo operativo coherente (cobro pendiente tras cancelación del restaurante) sin inconsistencias ni señales de fraude.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. El motivo es operativo y coherente con la solicitud de reembolso.</t>
         </is>
       </c>
       <c r="X105" t="inlineStr"/>
@@ -11557,7 +11665,7 @@
       <c r="Z105" t="inlineStr"/>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo y consistente con usuario de alta antigüedad y sin historial de riesgo. | Error de facturación post-cancelación validado en cuenta consolidada y sin riesgos previos.</t>
+          <t>APROBAR: reclamo legítimo consistente con evidencia operativa y perfil de usuario confiable. | Reembolso por cancelación de pedido en cuenta antigua y sin historial de riesgo.</t>
         </is>
       </c>
     </row>
@@ -11651,7 +11759,10 @@
       <c r="W106" t="inlineStr"/>
       <c r="X106" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y106" t="inlineStr"/>
@@ -11752,7 +11863,8 @@
       <c r="W107" t="inlineStr"/>
       <c r="X107" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y107" t="inlineStr"/>
@@ -11853,7 +11965,8 @@
       <c r="W108" t="inlineStr"/>
       <c r="X108" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y108" t="inlineStr"/>
@@ -11942,7 +12055,7 @@
       </c>
       <c r="T109" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>APROBAR</t>
         </is>
       </c>
       <c r="U109" t="inlineStr">
@@ -11952,24 +12065,24 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>APROBAR</t>
         </is>
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>Usuario sin historial de fraude y antigüedad moderada. El reclamo por doble cobro no muestra patrones de abuso, pero la pérdida de señal GPS impide validar la trazabilidad operativa requerida.</t>
+          <t>Reclamo de cobro duplicado sin señales de fraude. Usuario con antigüedad moderada y sin historial negativo. La falta de GPS no afecta la verificación financiera del cargo.</t>
         </is>
       </c>
       <c r="X109" t="inlineStr"/>
       <c r="Y109" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z109" t="inlineStr"/>
       <c r="AA109" t="inlineStr">
         <is>
-          <t>ESCALAR: falta evidencia GPS consistente y el tipo de reclamo requiere validación financiera manual antes de aprobar. | Solicitud de reembolso por duplicado en facturación. Sin evidencia GPS ni palabras críticas, pero requiere validación cruzada con pasarela de pagos.</t>
+          <t>APROBAR: reclamo operativo legítimo verificable en pasarela de pago sin indicadores de fraude. | Solicitud de reembolso por doble cargo en cuenta sin patrones abusivos ni contradicciones operativas.</t>
         </is>
       </c>
     </row>
@@ -12066,7 +12179,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>Pérdida de señal GPS impide validar entrega. Cuenta con 1 flag de fraude previo y reclamo subjetivo de producto incorrecto sin evidencia corroborante.</t>
+          <t>Evidencia GPS ausente combinada con un flag de fraude previo y frecuencia moderada de reclamos genera ambigüedad que impide la aprobación automatizada.</t>
         </is>
       </c>
       <c r="X110" t="inlineStr"/>
@@ -12078,7 +12191,7 @@
       <c r="Z110" t="inlineStr"/>
       <c r="AA110" t="inlineStr">
         <is>
-          <t>ESCALAR: datos insuficientes por GPS perdido y flag previo requieren validación humana del error de preparación. | Reclamo por error de producto en cuenta con historial mixto y sin evidencia geolocalizable.</t>
+          <t>ESCALAR: falta de evidencia GPS y flag de fraude previo requieren verificación humana para descartar abuso o error operativo. | Reclamo por producto incorrecto sin validación GPS en cuenta con historial de riesgo moderado.</t>
         </is>
       </c>
     </row>
@@ -12175,17 +12288,18 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', palabra crítica que activa automáticamente el protocolo de seguridad de marca y riesgo legal/sanitario. Esta señal se refuerza con alta frecuencia de reclamos (6 en 90d), señal GPS perdida que impide verificación operativa y un flag de fraude previo, haciendo inviable la aprobación automatizada.</t>
+          <t>El reclamo contiene el término crítico 'alergia', lo que activa automáticamente el protocolo de revisión humana por riesgos de salud y legales. Se complementa con alta frecuencia de reclamos y ausencia de evidencia GPS.</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | alta_frecuencia_reclamos | evidencia_gps_parcial</t>
+          <t>palabras_criticas_seguridad | alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z111" t="inlineStr">
@@ -12195,7 +12309,7 @@
       </c>
       <c r="AA111" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabras críticas de salud/legal (alergia) que requieren revisión humana conforme a reglas de seguridad de marca. | Reclamo por alergia alimentaria con evidencia GPS inconsistente y historial de alta frecuencia en cuenta moderadamente antigua.</t>
+          <t>ESCALAR: presencia de palabra crítica 'alergia' que requiere evaluación de riesgo legal/salud, corroborada por alta frecuencia de reclamos y falta de validación GPS. | Reclamo por alergia alimentaria en cuenta de 95 días con 6 incidentes en 90d y GPS sin señal.</t>
         </is>
       </c>
     </row>
@@ -12289,7 +12403,8 @@
       <c r="W112" t="inlineStr"/>
       <c r="X112" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y112" t="inlineStr"/>
@@ -12390,7 +12505,8 @@
       <c r="W113" t="inlineStr"/>
       <c r="X113" t="inlineStr">
         <is>
-          <t>A1 — Entrega demorada (&gt; p90 = 96 min) Y queja coherente con demora</t>
+          <t>A1 — Entrega demorada (&gt; p90 = 96 min) Y queja coherente con demora
+La telemetría respalda la queja (demora real documentada): no se penaliza al usuario legítimo.</t>
         </is>
       </c>
       <c r="Y113" t="inlineStr"/>
@@ -12491,7 +12607,10 @@
       <c r="W114" t="inlineStr"/>
       <c r="X114" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.</t>
         </is>
       </c>
       <c r="Y114" t="inlineStr"/>
@@ -12592,7 +12711,12 @@
       <c r="W115" t="inlineStr"/>
       <c r="X115" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y115" t="inlineStr"/>
@@ -12693,7 +12817,8 @@
       <c r="W116" t="inlineStr"/>
       <c r="X116" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y116" t="inlineStr"/>
@@ -12797,12 +12922,13 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', palabra crítica de seguridad que activa protocolo de escalación obligatoria. Adicionalmente, la cuenta tiene solo 10 días de antigüedad con 14 reclamos en 90 días y 2 flags de fraude previos, lo que indica un perfil de alto riesgo.</t>
+          <t>El reclamo contiene la palabra crítica 'alergia', lo que obliga a escalación por protocolo de seguridad y salud. Adicionalmente, la cuenta es extremadamente nueva (10d) con alta densidad de reclamos (14 en 90d) y dos flags de fraude previos, lo que confirma un perfil de alto riesgo que no puede resolverse automáticamente.</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y117" t="inlineStr">
@@ -12817,7 +12943,7 @@
       </c>
       <c r="AA117" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabras críticas de seguridad (alergia) que implican riesgo legal y de salud, sumado a señales claras de abuso de cuenta y fraude previo. | Reclamo por alergia alimentaria en cuenta nueva con historial de fraude y alta frecuencia de solicitudes. Riesgo legal/saludable requiere revisión humana inmediata.</t>
+          <t>ESCALAR: palabra crítica de seguridad presente ('alergia') combinada con cuenta nueva abusiva y historial de fraude previo, requiriendo evaluación humana especializada. | Reclamo por alergia en cuenta nueva con 14 intentos en 90d, 2 flags de fraude y score de riesgo alto. Requiere revisión humana por implicaciones de salud y fuerte evidencia de abuso.</t>
         </is>
       </c>
     </row>
@@ -12914,19 +13040,19 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>Alta frecuencia de reclamos (6 en 90d) y ratio de compensación elevado (0.84) sin evidencia GPS que valide el retraso o estado del pedido.</t>
+          <t>Usuario con 311 días de antigüedad pero 6 reclamos en 90 días. La ausencia de evidencia GPS genera ambigüedad para validar el retraso reportado.</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
       <c r="Y118" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | compensacion_elevada | entrega_gps_no_confirmada</t>
+          <t>alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z118" t="inlineStr"/>
       <c r="AA118" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de alta frecuencia, ratio de compensación elevado y falta de evidencia GPS requiere revisión humana para validar el retraso real. | Reclamo por retraso y calidad de comida en cuenta con historial de alta frecuencia y GPS no confirmado.</t>
+          <t>ESCALAR: alta frecuencia de reclamos combinada con falta de evidencia GPS para verificación objetiva requiere revisión humana. | Reclamo por retraso y calidad sin validación geolocal en cuenta con alta frecuencia de solicitudes.</t>
         </is>
       </c>
     </row>
@@ -13023,7 +13149,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, historial limpio y baja frecuencia de reclamos. El caso describe un error de cobro duplicado común sin señales de abuso.</t>
+          <t>Usuario con más de 3 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El tipo de incidencia (doble cobro) es verificable objetivamente vía pasarela de pagos y no presenta indicadores de abuso.</t>
         </is>
       </c>
       <c r="X119" t="inlineStr"/>
@@ -13035,7 +13161,7 @@
       <c r="Z119" t="inlineStr"/>
       <c r="AA119" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo sin indicadores de riesgo o inconsistencias. | Reclamo por cobro duplicado en cuenta antigua y sin antecedentes de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con un usuario de bajo riesgo y sin señales de fraude. | Error operativo de pago en cuenta antigua y sin historial negativo.</t>
         </is>
       </c>
     </row>
@@ -13132,19 +13258,19 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>Usuario con 506 días de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La justificación por cancelación operativa es coherente y no presenta inconsistencias con la evidencia disponible.</t>
+          <t>Usuario con 506 días de antigüedad, sin flags de fraude y frecuencia baja. La cancelación por falta de repartidor es un evento operativo coherente y el monto solicitado es razonable.</t>
         </is>
       </c>
       <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z120" t="inlineStr"/>
       <c r="AA120" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude o abuso. | Cancelación por falta de repartidor en cuenta estable y confiable.</t>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo legítimo por cancelación operativa en cuenta estable sin indicadores de riesgo.</t>
         </is>
       </c>
     </row>
@@ -13241,19 +13367,19 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>Usuario con 2+ años de antigüedad, 0 flags y baja frecuencia de reclamos. El reclamo por artículos faltantes es coherente y no presenta señales de fraude.</t>
+          <t>Usuario antiguo (731d) sin flags de fraude y baja frecuencia de reclamos. El reporte de faltantes es un error operativo frecuente y coherente.</t>
         </is>
       </c>
       <c r="X121" t="inlineStr"/>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z121" t="inlineStr"/>
       <c r="AA121" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo estándar por artículos faltantes en cuenta antigua y sin historial de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario confiable y sin señales de fraude. | Reclamo por faltantes en cuenta estable y limpia, sin inconsistencias operativas ni patrones de riesgo.</t>
         </is>
       </c>
     </row>
@@ -13335,7 +13461,7 @@
       </c>
       <c r="T122" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U122" t="inlineStr">
@@ -13345,12 +13471,12 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>Usuario con 198 días de antigüedad pero 5 reclamos en 90 días. La ausencia de evidencia GPS impide verificar la cancelación reportada, lo cual combinado con la alta frecuencia sugiere posible abuso o error sistémico.</t>
+          <t>Antigüedad moderada (198d) con 5 reclamos en 90 días. La falta de confirmación GPS coincide con la cancelación reportada, pero la alta frecuencia sin evidencia objetiva requiere validación manual.</t>
         </is>
       </c>
       <c r="X122" t="inlineStr"/>
@@ -13362,7 +13488,7 @@
       <c r="Z122" t="inlineStr"/>
       <c r="AA122" t="inlineStr">
         <is>
-          <t>RECHAZAR: alta frecuencia de reclamos sin evidencia GPS que respalde la cancelación reportada. | Reclamo por cancelación sin soporte GPS en cuenta con alta densidad de solicitudes recientes.</t>
+          <t>ESCALAR: combinación de alta frecuencia de reclamos y ausencia de evidencia GPS requiere revisión humana de logs operativos. | Reclamo por cancelación operativa en cuenta con alta densidad de solicitudes recientes y sin evidencia GPS de entrega.</t>
         </is>
       </c>
     </row>
@@ -13459,7 +13585,7 @@
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>Usuario con 1775 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado y ratio están dentro de parámetros normales. No se detectan inconsistencias ni términos de riesgo.</t>
+          <t>Usuario con casi 5 años de antigüedad, 0 flags y baja frecuencia de reclamos. Ausencia total de indicadores de fraude o inconsistencia.</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
@@ -13471,7 +13597,7 @@
       <c r="Z123" t="inlineStr"/>
       <c r="AA123" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo con perfil de usuario sano y ausencia de indicadores de riesgo. | Reclamo por calidad de producto en cuenta confiable sin señales de abuso o fraude.</t>
+          <t>APROBAR: reclamo legítimo respaldado por historial de usuario estable y ausencia de patrones abusivos. | Reclamo por calidad de alimento en cuenta altamente confiable sin señales de riesgo operativo.</t>
         </is>
       </c>
     </row>
@@ -13568,19 +13694,19 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años, 0 flags de fraude y frecuencia baja de reclamos. El monto solicitado y ratio son normales.</t>
+          <t>Usuario con más de 4 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El reporte de producto equivocado es un error operativo común. La pérdida de señal GPS no contradice el reclamo y el perfil conservador indica legitimidad.</t>
         </is>
       </c>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z124" t="inlineStr"/>
       <c r="AA124" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por producto equivocado en cuenta verificada sin señales de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario de larga trayectoria y sin historial negativo. | Error operativo de restaurante en cuenta antigua y confiable sin indicadores de fraude.</t>
         </is>
       </c>
     </row>
@@ -13677,19 +13803,19 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>Historial con flag de fraude y 6 reclamos en 90 días. Evidencia GPS nula para validar entrega, lo que invalida la coherencia del reclamo.</t>
+          <t>Cuenta con flag de fraude previo y 6 reclamos en 90 días. La evidencia GPS indica señal perdida, lo que genera inconsistencia con la afirmación de entrega de la app y el reclamo del usuario. Ratio de compensación elevado refuerza el riesgo.</t>
         </is>
       </c>
       <c r="X125" t="inlineStr"/>
       <c r="Y125" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z125" t="inlineStr"/>
       <c r="AA125" t="inlineStr">
         <is>
-          <t>RECHAZAR: alta frecuencia de reclamos, flag de fraude previo y falta de evidencia GPS que respalde la no recepción. | Inconsistencia entre estado de app, GPS perdido y reclamo de no recepción en cuenta con historial sospechoso.</t>
+          <t>RECHAZAR: evidencia clara de posible abuso combinando flag de fraude, alta frecuencia y falta de validación geoespacial. | Inconsistencia entre estado de entrega y evidencia GPS en cuenta con historial negativo y alta frecuencia de reclamos.</t>
         </is>
       </c>
     </row>
@@ -13783,7 +13909,8 @@
       <c r="W126" t="inlineStr"/>
       <c r="X126" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y126" t="inlineStr"/>
@@ -13884,7 +14011,12 @@
       <c r="W127" t="inlineStr"/>
       <c r="X127" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y127" t="inlineStr"/>
@@ -13985,7 +14117,10 @@
       <c r="W128" t="inlineStr"/>
       <c r="X128" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.</t>
         </is>
       </c>
       <c r="Y128" t="inlineStr"/>
@@ -14089,7 +14224,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a un año y cero flags de fraude. El reclamo es coherente y la pérdida de señal GPS es un fallo técnico común, no indica abuso.</t>
+          <t>Perfil de usuario sano con 353 días de antigüedad y cero reclamos recientes. La narrativa es coherente y no contiene palabras críticas. La pérdida de señal GPS no constituye evidencia de fraude.</t>
         </is>
       </c>
       <c r="X129" t="inlineStr"/>
@@ -14101,7 +14236,7 @@
       <c r="Z129" t="inlineStr"/>
       <c r="AA129" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario conservador sin señales de fraude, la inconsistencia se debe a falla técnica de rastreo. | Reclamo legítimo por entrega no recibida en cuenta limpia con señal GPS perdida.</t>
+          <t>APROBAR: reclamo legítimo sin indicadores de fraude, perfil conservador y narrativa coherente. | Reclamo por marcaje de entrega sin confirmación de timbre. Usuario sin historial de riesgo ni inconsistencias operativas.</t>
         </is>
       </c>
     </row>
@@ -14198,19 +14333,19 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>Usuario con 558 días de antigüedad, 0 flags y 0 reclamos recientes. La descripción del error (producto incorrecto) es coherente y no presenta contradicciones con la evidencia disponible.</t>
+          <t>Usuario con 558 días de antigüedad y 0 flags de fraude. Reclamo de ítem incorrecto coherente, monto razonable y sin patrones de abuso.</t>
         </is>
       </c>
       <c r="X130" t="inlineStr"/>
       <c r="Y130" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z130" t="inlineStr"/>
       <c r="AA130" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo por producto equivocado en cuenta estable sin historial de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Error operativo en entrega de bebida en cuenta verificada sin historial de riesgo.</t>
         </is>
       </c>
     </row>
@@ -14307,19 +14442,19 @@
       </c>
       <c r="W131" t="inlineStr">
         <is>
-          <t>Usuario con 576 días de antigüedad, cero reclamos recientes y sin flags de fraude. La solicitud es una discrepancia de cobro operativa, coherente y sin señales de abuso.</t>
+          <t>Usuario con 576 días de antigüedad, 0 flags y 0 reclamos recientes. La discrepancia de cobro es un error operativo común y no presenta indicadores de fraude.</t>
         </is>
       </c>
       <c r="X131" t="inlineStr"/>
       <c r="Y131" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z131" t="inlineStr"/>
       <c r="AA131" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de discrepancia de cobro en usuario con historial limpio y sin señales de riesgo. | Reclamo de discrepancia tarifaria en cuenta limpia y antigua, sin indicadores de fraude.</t>
+          <t>APROBAR: reclamo legítimo de usuario sin historial de riesgo ni inconsistencias. | Reclamo por diferencia de monto en resumen de pago en cuenta limpia.</t>
         </is>
       </c>
     </row>
@@ -14416,7 +14551,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>Reclamo por cobro tras cancelación. Sin flags de fraude, pero la evidencia GPS parcial combinada con alta frecuencia de reclamos (5 en 90d) y ratio de compensación elevado genera ambigüedad operativa que impide una decisión automatizada segura.</t>
+          <t>Reclamo por cobro tras cancelación con evidencia GPS parcial y alta frecuencia de reclamos (5 en 90d) junto a un ratio de compensación elevado (0.86). Requiere revisión para validar si es error de facturación o patrón recurrente.</t>
         </is>
       </c>
       <c r="X132" t="inlineStr"/>
@@ -14428,7 +14563,7 @@
       <c r="Z132" t="inlineStr"/>
       <c r="AA132" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por evidencia GPS parcial y alta frecuencia de reclamos con ratio de compensación elevado, requiere validación manual. | Solicitud de reembolso por cancelación con GPS parcial, alta frecuencia reciente y ratio de compensación alto.</t>
+          <t>ESCALAR: evidencia GPS parcial combinada con alta frecuencia de reclamos y ratio de compensación elevado requiere validación manual para descartar abuso o confirmar error de sistema. | Disputa de cobro por cancelación con GPS ambigua y historial de alta frecuencia/recompensa.</t>
         </is>
       </c>
     </row>
@@ -14525,7 +14660,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. La descripción del deterioro es coherente y no presenta contradicciones técnicas ni palabras críticas.</t>
+          <t>Usuario con 1260 días de antigüedad y 0 flags de fraude. El reclamo por calidad es coherente y no activa reglas de riesgo ni palabras críticas.</t>
         </is>
       </c>
       <c r="X133" t="inlineStr"/>
@@ -14537,7 +14672,7 @@
       <c r="Z133" t="inlineStr"/>
       <c r="AA133" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario conservador y ausencia de inconsistencias. | Reclamo por calidad de producto en cuenta confiable sin señales de riesgo operativo o fraude.</t>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario estable y ausencia de señales de fraude. | Queja por estado del producto en cuenta confiable sin indicadores de abuso.</t>
         </is>
       </c>
     </row>
@@ -14634,12 +14769,13 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', lo cual activa automáticamente las reglas de seguridad de marca y salud. Aunque el perfil del usuario es sano y sin historial de fraude, la naturaleza del reclamo requiere validación médica/legal.</t>
+          <t>El reclamo menciona explícitamente 'alergia', lo que activa el protocolo de palabras críticas de seguridad de marca y riesgo legal/salud, requiriendo revisión humana inmediata.</t>
         </is>
       </c>
       <c r="X134" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y134" t="inlineStr">
@@ -14654,7 +14790,7 @@
       </c>
       <c r="AA134" t="inlineStr">
         <is>
-          <t>ESCALAR: presencia de palabra crítica ('alergia') que genera riesgo de salud y potencial responsabilidad legal, requiriendo revisión humana obligatoria. | Reclamo por posible error de preparación con implicaciones de salud (alergia). Activa protocolo de escalamiento por palabras críticas.</t>
+          <t>ESCALAR: contiene término crítico de salud ('alergia') que requiere validación médica/legal y gestión de riesgo de marca. | Reclamo por alergia alimentaria en cuenta antigua sin historial de fraude, pero con señal crítica de salud que impide aprobación automatizada.</t>
         </is>
       </c>
     </row>
@@ -14751,19 +14887,19 @@
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>Usuario con 790 días de antigüedad y sin historial de fraude. El reporte de faltante es un error operativo común y coherente. No se activan reglas de riesgo ni términos críticos.</t>
+          <t>Usuario con 790 días de antigüedad y 0 flags de fraude. El reclamo por faltante es un incidente operativo común y coherente, sin activar reglas de riesgo automático.</t>
         </is>
       </c>
       <c r="X135" t="inlineStr"/>
       <c r="Y135" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z135" t="inlineStr"/>
       <c r="AA135" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario antiguo y sin señales de fraude. | Faltante de producto validado por perfil de usuario confiable y sin inconsistencias.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo estándar por faltante de producto en cuenta antigua y limpia, sin evidencia GPS contradictoria ni palabras críticas.</t>
         </is>
       </c>
     </row>
@@ -14860,17 +14996,18 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad de marca y riesgo legal/salud. Se refuerza con historial de fraude previo y cuenta nueva con alta frecuencia de reclamos.</t>
+          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad y salud, requiriendo revisión humana obligatoria. Adicionalmente, la cuenta presenta alta frecuencia de reclamos en 90 días, antigüedad muy reciente y 2 flags de fraude previos, lo que incrementa el riesgo.</t>
         </is>
       </c>
       <c r="X136" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y136" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | flag_fraude_previo | account_abuse</t>
+          <t>palabras_criticas_seguridad | account_abuse | flag_fraude_previo</t>
         </is>
       </c>
       <c r="Z136" t="inlineStr">
@@ -14880,7 +15017,7 @@
       </c>
       <c r="AA136" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabras críticas de seguridad de marca ('alergia') que implican riesgo legal/salud, sumado a señales de fraude previo y abuso de cuenta. | Reclamo por alergia en cuenta nueva con 2 flags de fraude y 12 reclamos en 90 días. Requiere revisión humana por términos de salud/legal.</t>
+          <t>ESCALAR: contiene palabras críticas de seguridad (alergia) que requieren validación humana, sumado a señales de abuso de cuenta y fraude previo. | Reclamo por alergia alimentaria en cuenta nueva con alta frecuencia de incidencias y antecedentes de fraude. La mención de riesgo de salud obliga a escalación manual.</t>
         </is>
       </c>
     </row>
@@ -14974,7 +15111,12 @@
       <c r="W137" t="inlineStr"/>
       <c r="X137" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R3 — freq_densidad &gt; p95 del dataset original; R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R3 — freq_densidad &gt; p95 del dataset original
+Ritmo de reclamos por día por encima del p95 del dataset: patrón de reclamos atípico.
+R6 — Usuario &lt; 90 días de antigüedad con &gt; p95 reclamos en 90d
+Cuenta nueva (&lt; 90 días) con récord de reclamos: la señal de fraude más fuerte del dataset.</t>
         </is>
       </c>
       <c r="Y137" t="inlineStr"/>
@@ -15078,15 +15220,19 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>Perfil de usuario muy antiguo y limpio sin historial de reclamos ni flags. Reclamo por ítem faltante es operativo y coherente con la evidencia disponible.</t>
+          <t>Usuario con antigüedad superior a 3 años, historial limpio y 0 reclamos recientes. El reclamo por ítem faltante es operativo y coherente, sin señales de fraude.</t>
         </is>
       </c>
       <c r="X138" t="inlineStr"/>
-      <c r="Y138" t="inlineStr"/>
+      <c r="Y138" t="inlineStr">
+        <is>
+          <t>entrega_gps_no_confirmada</t>
+        </is>
+      </c>
       <c r="Z138" t="inlineStr"/>
       <c r="AA138" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sin riesgos. | Reclamo estándar por producto faltante en cuenta confiable sin señales de fraude.</t>
+          <t>APROBAR: reclamo legítimo de usuario confiable sin historial de fraude ni patrones abusivos. | Reclamo estándar por producto faltante en cuenta antigua y sana, sin inconsistencias ni riesgos detectados.</t>
         </is>
       </c>
     </row>
@@ -15180,7 +15326,8 @@
       <c r="W139" t="inlineStr"/>
       <c r="X139" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y139" t="inlineStr"/>
@@ -15284,19 +15431,19 @@
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>Alta frecuencia de reclamos (5 en 90d) combinada con señal GPS perdida genera ambigüedad para validar el retraso real y la condición del pedido.</t>
+          <t>Reclamo por retraso y calidad con 5 incidencias en 90 días y sin rastreo GPS disponible. La ambigüedad en la evidencia y la densidad de reclamos requieren validación manual.</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
       <c r="Y140" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>alta_frecuencia_reclamos | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z140" t="inlineStr"/>
       <c r="AA140" t="inlineStr">
         <is>
-          <t>ESCALAR: datos insuficientes por pérdida de GPS y patrón de frecuencia elevada requieren validación humana del incidente operativo. | Reclamo por retraso y calidad de comida sin evidencia GPS que confirme o refute los tiempos de entrega, en cuenta con historial de múltiples solicitudes recientes.</t>
+          <t>ESCALAR: combinación de señal GPS perdida y alta frecuencia de reclamos requiere revisión humana para validar el retraso reportado. | Posible falla operativa por retraso, pero la falta de GPS y alta frecuencia de reclamos impiden la decisión automatizada.</t>
         </is>
       </c>
     </row>
@@ -15393,19 +15540,19 @@
       </c>
       <c r="W141" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad sólida (911d) y 0 flags de fraude, pero el reclamo contradice el estatus de la app y la evidencia GPS no está confirmada. El ratio de compensación histórico es elevado (0.955), generando ambigüedad que requiere validación humana.</t>
+          <t>Contradicción entre estado de la app y reporte del usuario sin respaldo GPS. Perfil antiguo sin flags de fraude, pero la falta de evidencia objetiva impide decisión automatizada.</t>
         </is>
       </c>
       <c r="X141" t="inlineStr"/>
       <c r="Y141" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | compensacion_elevada | descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z141" t="inlineStr"/>
       <c r="AA141" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por falta de evidencia GPS y ratio de compensación elevado requieren revisión manual. | Reclamo por no recepción con GPS no confirmado y alta tasa de compensación previa en cuenta antigua.</t>
+          <t>ESCALAR: ausencia de evidencia GPS y datos insuficientes para verificar objetivamente el reclamo. | Reclamo por no recepción con GPS no confirmado y perfil conservador, requiere validación manual.</t>
         </is>
       </c>
     </row>
@@ -15502,7 +15649,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, sin historial de fraude ni alta frecuencia de reclamos. La solicitud por producto incorrecto es coherente y el monto es razonable.</t>
+          <t>Usuario con más de 3 años de antigüedad, 0 flags y 0 reclamos recientes. El reclamo por ítem incorrecto es coherente y el monto es razonable. La pérdida de señal GPS no indica fraude al no haber contradicciones.</t>
         </is>
       </c>
       <c r="X142" t="inlineStr"/>
@@ -15514,7 +15661,7 @@
       <c r="Z142" t="inlineStr"/>
       <c r="AA142" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin inconsistencias. | Reclamo operativo por entrega de bebida errónea en cuenta antigua y confiable sin señales de riesgo.</t>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Error operativo del restaurante en usuario antiguo y sin historial de riesgo.</t>
         </is>
       </c>
     </row>
@@ -15608,7 +15755,12 @@
       <c r="W143" t="inlineStr"/>
       <c r="X143" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos; R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega; R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.
+R5 — Usuario dice 'Orden no llegó' pero GPS confirma entrega
+El reclamo dice 'Orden no llegó' pero el GPS confirma la entrega: contradicción directa con la telemetría.
+R7 — score_riesgo_previo (flags×2 + comps_90d×0.5) &gt; p90
+El score de riesgo previo (flags×2 + reclamos×0.5) supera el p90 del dataset: historial inaceptable.</t>
         </is>
       </c>
       <c r="Y143" t="inlineStr"/>
@@ -15709,7 +15861,8 @@
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr">
         <is>
-          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo</t>
+          <t>A3 — GPS confirmado, sin retraso, ratio normal, usuario antiguo
+Entrega confirmada, sin demora, compensación que no excede la orden y usuario con historial.</t>
         </is>
       </c>
       <c r="Y144" t="inlineStr"/>
@@ -15813,7 +15966,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, historial limpio y sin reclamos recientes. El motivo corresponde a un error de facturación por cancelación del restaurante, totalmente coherente con la evidencia operativa.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude ni frecuencia de reclamos. El motivo descrito corresponde a un error operativo estándar de facturación por cancelación del restaurante.</t>
         </is>
       </c>
       <c r="X145" t="inlineStr"/>
@@ -15825,7 +15978,7 @@
       <c r="Z145" t="inlineStr"/>
       <c r="AA145" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con usuario de alto perfil y sin señales de fraude o inconsistencias. | Reclamo operativo legítimo por cargo no revertido tras cancelación en cuenta antigua y sin antecedentes de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con un error administrativo, sin señales de fraude. | Error de facturación por cancelación del restaurante en cuenta antigua y sin historial sospechoso.</t>
         </is>
       </c>
     </row>
@@ -15919,7 +16072,8 @@
       <c r="W146" t="inlineStr"/>
       <c r="X146" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y146" t="inlineStr"/>
@@ -16023,17 +16177,18 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', activando la regla de palabras críticas que exige revisión humana por riesgo de salud y reputación. Se combina con 2 flags de fraude previos y evidencia GPS parcial, lo que invalida la aprobación automática.</t>
+          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad por riesgo legal/salud. Sumado a 2 flags de fraude previos y evidencia GPS parcial, se requiere revisión humana para validar la justificación médica y evitar exposición de marca.</t>
         </is>
       </c>
       <c r="X147" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | flag_fraude_previo | evidencia_gps_parcial</t>
+          <t>palabras_criticas_seguridad | flag_fraude_previo</t>
         </is>
       </c>
       <c r="Z147" t="inlineStr">
@@ -16043,7 +16198,7 @@
       </c>
       <c r="AA147" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabra crítica ('alergia') que activa protocolo de riesgo legal/salud, sumado a 2 flags de fraude previos y GPS parcial que dificultan la verificación objetiva. | Reclamo por alergia alimentaria en cuenta con historial de fraude y GPS ambigua. Requiere validación humana conforme a política de seguridad de marca.</t>
+          <t>ESCALAR: contiene término crítico ('alergia') que implica riesgo de salud/legal, reforzado por 2 flags de fraude previos y evidencia GPS inconclusa. Requiere validación humana obligatoria. | Reclamo por alergia alimentaria en cuenta con historial de fraude y GPS parcial. Activación automática por palabras críticas de seguridad.</t>
         </is>
       </c>
     </row>
@@ -16140,15 +16295,19 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>Perfil de usuario antiguo (1612d) sin flags de fraude ni alta frecuencia. El reclamo es una consulta de facturación estándar con monto dentro de rangos normales.</t>
+          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. Reclamo de discrepancia tarifaria sin indicadores de abuso.</t>
         </is>
       </c>
       <c r="X148" t="inlineStr"/>
-      <c r="Y148" t="inlineStr"/>
+      <c r="Y148" t="inlineStr">
+        <is>
+          <t>entrega_gps_no_confirmada</t>
+        </is>
+      </c>
       <c r="Z148" t="inlineStr"/>
       <c r="AA148" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo sin señales de fraude. | Discrepancia de cobro en cuenta confiable sin indicadores de abuso o riesgo.</t>
+          <t>APROBAR: reclamo operativo legítimo sin señales de fraude ni patrones abusivos. | Discrepancia entre monto cobrado y resumen de pedido reportada por usuario antiguo y confiable.</t>
         </is>
       </c>
     </row>
@@ -16245,12 +16404,13 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', palabra crítica de seguridad que activa protocolo de escalación obligatoria. Se combina con cuenta nueva (29d), alta frecuencia de reclamos (14 en 90d) y historial con 2 flags de fraude, lo que eleva el riesgo legal y operativo.</t>
+          <t>El reclamo menciona 'alergia', activando la regla de palabras críticas que exige revisión humana por riesgo de salud y responsabilidad legal. Adicionalmente, la cuenta tiene solo 29 días de antigüedad con 14 reclamos en 90 días y 2 flags de fraude previos, lo que indica un patrón de abuso y alto riesgo.</t>
         </is>
       </c>
       <c r="X149" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda</t>
+          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
+El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
         </is>
       </c>
       <c r="Y149" t="inlineStr">
@@ -16265,7 +16425,7 @@
       </c>
       <c r="AA149" t="inlineStr">
         <is>
-          <t>ESCALAR: presencia de palabra crítica ('alergia') que exige revisión manual por riesgo legal/salud, corroborado por perfil de cuenta nueva con alta reincidencia y flags de fraude previos. | Reclamo por alergia alimentaria en cuenta nueva con alta densidad de reclamos y antecedentes de fraude. Pre-marcado para revisión humana por implicaciones de salud y riesgo de marca.</t>
+          <t>ESCALAR: contiene palabra crítica ('alergia') que implica riesgo de salud y responsabilidad civil, sumado a historial de fraude y cuenta nueva con alta densidad de reclamos. | Reclamo por alergia en cuenta nueva con alta frecuencia, flags de fraude previos y evidencia pre-marcada para escalación por seguridad de marca.</t>
         </is>
       </c>
     </row>
@@ -16359,7 +16519,8 @@
       <c r="W150" t="inlineStr"/>
       <c r="X150" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos</t>
+          <t>R1 — Usuario con 2 o más flags de fraude previos
+El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
         </is>
       </c>
       <c r="Y150" t="inlineStr"/>
@@ -16448,7 +16609,7 @@
       </c>
       <c r="T151" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U151" t="inlineStr">
@@ -16458,24 +16619,24 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W151" t="inlineStr">
         <is>
-          <t>Cuenta con flag de fraude previo y ratio de compensación elevado (0.93). La evidencia GPS no confirma la entrega, generando ambigüedad que requiere revisión humana para validar o refutar el reclamo.</t>
+          <t>El perfil presenta un flag de fraude previo y un ratio de compensación muy alto (0.93), sumado a la falta de confirmación GPS que valide la entrega reclamada.</t>
         </is>
       </c>
       <c r="X151" t="inlineStr"/>
       <c r="Y151" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | entrega_gps_no_confirmada | compensacion_elevada</t>
+          <t>flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z151" t="inlineStr"/>
       <c r="AA151" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de flag de fraude previo, ratio de compensación alto y falta de evidencia GPS determina necesidad de revisión manual. | Reclamo por entrega no recibida sin validación GPS en cuenta con historial de fraude y alta propensión a compensaciones.</t>
+          <t>RECHAZAR: inconsistencia por falta de evidencia GPS combinada con flag de fraude previo y ratio de compensación elevado. | Reclamo sin respaldo geolocal y con historial de riesgo y compensaciones elevadas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: reglas en YAML, batch durable, página Documentación, reporte EDA y despliegue
- Motor de reglas solo desde thresholds.yaml (RuleEngine), sin tablas de reglas en DB.
- Batch durable en PostgreSQL (src/batch/) compartido con la API; timeouts y fallbacks.
- UI: página Documentación (auto-scan de docs/ + README/CHECKPOINTS), grafo del proceso
  reutilizable (src/ui/flow.py) y render de imágenes locales en markdown.
- Docs: reporte EDA con figuras (docs/media/eda), guía operativa de reglas, índice en
  README, sección 'Desplegar agente' para otra máquina, drift de docs corregido.
- Infra: mounts de README/CHECKPOINTS en UI, pyarrow + parquet en imagen de API.
- Tests: 55 passed (incluye batch durable y navegación 4 páginas).
</commit_message>
<xml_diff>
--- a/data/150casos_analizados.xlsx
+++ b/data/150casos_analizados.xlsx
@@ -646,19 +646,19 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años y 0 flags de fraude. Reclamo operativo sin señales de abuso o inconsistencia.</t>
+          <t>Usuario con más de 4 años de antigüedad, 0 flags de fraude y baja densidad de reclamos. El monto solicitado y el ratio de compensación están dentro de rangos normales. No hay inconsistencias GPS críticas ni palabras de riesgo.</t>
         </is>
       </c>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Error de preparación del restaurante en usuario antiguo y limpio, sin evidencia de fraude.</t>
+          <t>APROBAR: reclamo legítimo consistente con un perfil de usuario estable y sin historial negativo. | Reclamo operativo estándar en cuenta antigua y confiable sin indicadores de fraude.</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>maximosabor</t>
+          <t>USR-18450</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -755,7 +755,7 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas que obliga a escalación por riesgo de salud/marca. Aunque el GPS es parcial y existe un flag previo, la mención de condiciones médicas supera cualquier análisis automatizado.</t>
+          <t>El reclamo contiene la palabra crítica 'alergia', lo que activa automáticamente el protocolo de seguridad por riesgo de salud y potencial responsabilidad legal. La evidencia GPS es parcial y existe un flag de fraude previo, lo que impide una validación automatizada segura.</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -776,7 +776,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabra crítica 'alergia' que implica riesgo de salud y responsabilidad legal, requiriendo validación manual según política de seguridad de marca. | Reclamo por alergia alimentaria en cuenta con flag previo y GPS parcial, sujeto a revisión humana obligatoria por términos de seguridad de marca.</t>
+          <t>ESCALAR: presencia de término crítico ('alergia') que implica riesgo de salud y posible responsabilidad legal, combinado con GPS parcial y antecedente de fraude. | Reclamo por alergia alimentaria con GPS parcial y antecedente de fraude. Se confirma escalación por riesgo sanitario y legal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: seed reproducible (terminador COPY corrupto en 09_seed_completo.sql) y portabilidad
- make up ahora garantiza los datos: ejecuta make seed (idempotente, aplica esquema y carga los 250 casos solo si cases esta vacia)
- Dockerfiles api/ui: pip --retries 10 --timeout 300 + versiones fijadas (builds tolerantes a redes lentas)
- .gitattributes anti-CRLF (seed SQL e init.sh seguros en Windows)
- Elimina legacy batch_process/batch_chunk (tenian path absoluto de macOS)
- README: despliegue paso a paso por SO (macOS/Linux/Windows-WSL2/PowerShell), URL real del repo, y distribucion alineada al seed (250: 105/100/45; 150 reales: 65/58/27); xlsx 150 regenerado desde DB
</commit_message>
<xml_diff>
--- a/data/150casos_analizados.xlsx
+++ b/data/150casos_analizados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA151"/>
+  <dimension ref="A1:AB151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -552,6 +552,11 @@
           <t>resumen_llm</t>
         </is>
       </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>fallback</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -646,21 +651,22 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad, 0 flags de fraude y baja densidad de reclamos. El monto solicitado y el ratio de compensación están dentro de rangos normales. No hay inconsistencias GPS críticas ni palabras de riesgo.</t>
+          <t>El usuario posee una antigüedad superior a 4 años y un historial completamente limpio sin flags de fraude, lo cual constituye un indicador fuerte de legitimidad. La frecuencia de reclamos (2 en 90 días) se mantiene dentro de los parámetros normales para su perfil. Aunque la telemetría GPS no confirma la entrega, el tipo de incidencia reportada (error de plato/preparación) no depende exclusivamente de la geolocalización para ser verificada. El relato es coherente, el monto solicitado es propor...</t>
         </is>
       </c>
       <c r="X2" t="inlineStr"/>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>historial_intachable | frecuencia_reclamos_normal | monto_compensacion_razonable</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr"/>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con un perfil de usuario estable y sin historial negativo. | Reclamo operativo estándar en cuenta antigua y confiable sin indicadores de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR | Reclamo por error operativo en plato atendido a usuario de larga antigüedad e historial limpio, sin indicios de fraude.</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -755,30 +761,30 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>El reclamo contiene la palabra crítica 'alergia', lo que activa automáticamente el protocolo de seguridad por riesgo de salud y potencial responsabilidad legal. La evidencia GPS es parcial y existe un flag de fraude previo, lo que impide una validación automatizada segura.</t>
+          <t>El reclamo contiene la palabra crítica 'alergia', lo que activa automáticamente la regla de escalación por riesgos de salud y posibles implicaciones legales o de reputación para la plataforma. El contexto refuerza esta decisión: existe un flag de fraude previo en la cuenta, la evidencia GPS es parcial e insuficiente para validar la entrega, y se solicita un monto elevado ($153.91) con un ratio de compensación muy alto (0.9241). La combinación de un incidente de salud declarado, historial con ...</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>ESCALAR-1 — Reclamo menciona alergia, intoxicación, policía, sangre, abogado, demanda
-El reclamo menciona términos de riesgo legal o de salud (alergia, policía, demanda…). Lo revisa un humano, no el sistema.</t>
+          <t>ESCALAR por seguridad de marca: el reclamo contiene palabras críticas que requieren revisión humana.</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | evidencia_gps_parcial | flag_fraude_previo</t>
+          <t>palabras_criticas_seguridad | flag_fraude_previo | evidencia_gps_parcial | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>descripcion_reclamo contains_any [alergi, intoxic, policía, policia, sangre, insult, denunci, abogado, demanda, hospital, veneno] = alergi</t>
+          <t>flag_palabras_criticas: seguridad de marca</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>ESCALAR: presencia de término crítico ('alergia') que implica riesgo de salud y posible responsabilidad legal, combinado con GPS parcial y antecedente de fraude. | Reclamo por alergia alimentaria con GPS parcial y antecedente de fraude. Se confirma escalación por riesgo sanitario y legal.</t>
-        </is>
-      </c>
+          <t>ESCALAR | Reclamo por alergia alimentaria con flag de fraude previo, GPS parcial y alta exposición económica, requiriendo evaluación legal y de marca.</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -858,7 +864,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -868,26 +874,27 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>Reclamo por faltantes coherente, pero la cuenta tiene 1 flag de fraude previo y ratio de compensación alto (0.89). Se requiere validación manual para cruzar evidencia y revisar el antecedente.</t>
+          <t>El usuario presenta un flag de fraude previo combinado con un ratio de compensación muy alto (0.8975). El reclamo por faltantes es subjetivo y carece de validación GPS, lo que incrementa significativamente el riesgo de abuso.</t>
         </is>
       </c>
       <c r="X4" t="inlineStr"/>
       <c r="Y4" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | compensacion_elevada | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z4" t="inlineStr"/>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>ESCALAR: flag de fraude previo combinado con compensación elevada exige revisión humana para validar legitimidad. | Solicitud de faltantes en cuenta con historial mixto y alta frecuencia de pagos.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: historial con flag de fraude, ratio de compensación elevado y falta de evidencia objetiva para faltantes menores. | Reclamo por faltantes sin evidencia objetiva en cuenta con historial de fraude y alta tasa de compensación.</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -982,21 +989,22 @@
       </c>
       <c r="W5" t="inlineStr">
         <is>
-          <t>Cuenta antigua y sin historial de fraude, pero la evidencia GPS está perdida lo que impide validar o refutar la entrega. Reclamo subjetivo sin corroboración objetiva.</t>
+          <t>Cuenta antigua y sin historial de fraude, pero la pérdida de señal GPS impide corroborar la entrega. El ratio de compensación cercano a 1.0 y la falta de evidencia objetiva requieren validación manual.</t>
         </is>
       </c>
       <c r="X5" t="inlineStr"/>
       <c r="Y5" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>evidencia_gps_parcial | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z5" t="inlineStr"/>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>ESCALAR: falta de evidencia GPS para confirmar entrega y naturaleza subjetiva del reclamo requieren revisión humana. | Reclamo de no recepción con señal GPS perdida en cuenta confiable de larga antigüedad.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ambigüedad por señal GPS perdida y ratio de compensación elevado que impiden decisión automatizada segura. | Reclamo por no recepción con evidencia GPS incompleta en usuario de larga antigüedad.</t>
+        </is>
+      </c>
+      <c r="AB5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1091,21 +1099,18 @@
       </c>
       <c r="W6" t="inlineStr">
         <is>
-          <t>Usuario con 1458 días de antigüedad y 0 flags. Reclamo administrativo sobre cobro sin señales de fraude ni inconsistencia.</t>
+          <t>Usuario con 4+ años de antigüedad, sin flags ni frecuencia de reclamos. Reclamo de discrepancia de cobro objetivo y monto dentro de parámetros normales.</t>
         </is>
       </c>
       <c r="X6" t="inlineStr"/>
-      <c r="Y6" t="inlineStr">
-        <is>
-          <t>descripcion_incoherente</t>
-        </is>
-      </c>
+      <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr"/>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de discrepancia de cobro en cuenta sin riesgos. | Discrepancia de monto reportada por usuario leal sin historial de reclamos recientes.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de error de facturación en usuario con historial impecable y sin señales de fraude. | Discrepancia de cobro en cuenta limpia y antigua sin señales de fraude.</t>
+        </is>
+      </c>
+      <c r="AB6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1208,6 +1213,7 @@
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
+      <c r="AB7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1302,21 +1308,22 @@
       </c>
       <c r="W8" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 6 meses, baja frecuencia de reclamos y sin flags de fraude. No se activaron reglas de riesgo ni palabras críticas.</t>
+          <t>Perfil de usuario sólido (655 días de antigüedad, 0 flags, 2 reclamos en 90d). Aunque la verificación de caducidad es subjetiva y el GPS se perdió, no existen inconsistencias ni patrones de abuso que respalden un rechazo.</t>
         </is>
       </c>
       <c r="X8" t="inlineStr"/>
       <c r="Y8" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>reclamo_subjetivo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z8" t="inlineStr"/>
       <c r="AA8" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude ni criterios de rechazo o escalación. | Reclamo por producto caducado en cuenta limpia, sin inconsistencias operativas ni señales de abuso detectadas.</t>
-        </is>
-      </c>
+          <t>APROBAR: usuario con historial conservador y sin indicadores de riesgo que invaliden el reclamo. | Reclamo por producto caducado en cuenta antigua y limpia, sin señales de fraude detectadas.</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1411,7 +1418,7 @@
       </c>
       <c r="W9" t="inlineStr">
         <is>
-          <t>Perfil de usuario limpio con antigüedad moderada y baja frecuencia de reclamos. El tipo de incidencia (cobro duplicado) es operativo y no presenta inconsistencias con la evidencia disponible.</t>
+          <t>Usuario con antigüedad de 312 días, 0 flags de fraude y baja frecuencia de reclamos. El reporte de doble cobro es un error operativo frecuente y coherente con la información disponible.</t>
         </is>
       </c>
       <c r="X9" t="inlineStr"/>
@@ -1423,9 +1430,10 @@
       <c r="Z9" t="inlineStr"/>
       <c r="AA9" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Reclamo por cobro duplicado en cuenta sin historial de fraude ni señales de abuso. Evidencia GPS no aplicable al tipo de incidencia.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo por error de cobro duplicado en usuario con historial limpio y perfil conservador. | Error de facturación en cuenta limpia sin indicadores de abuso o inconsistencia crítica.</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1517,17 +1525,17 @@
       <c r="W10" t="inlineStr"/>
       <c r="X10" t="inlineStr">
         <is>
-          <t>R1 — Usuario con 2 o más flags de fraude previos
-El usuario tiene 2 o más flags de fraude previos: ya está señalado por el sistema.</t>
+          <t>RECHAZAR por señales de fraude: flags_fraude_previos &gt;= 2.</t>
         </is>
       </c>
       <c r="Y10" t="inlineStr"/>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>flags_fraude_previos &gt;= 2 = 2</t>
+          <t>flags_fraude_previos &gt;= 2</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr"/>
+      <c r="AB10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1622,21 +1630,22 @@
       </c>
       <c r="W11" t="inlineStr">
         <is>
-          <t>Usuario con 1656 días de antigüedad y 0 flags de fraude. El reclamo por faltante de producto es operativo, coherente y no activa reglas de riesgo.</t>
+          <t>Usuario veterano con 1656 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado es proporcional al pedido y la falta de confirmación GPS es irrelevante para incidencias de faltantes.</t>
         </is>
       </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z11" t="inlineStr"/>
       <c r="AA11" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario antiguo y sin señales de fraude. | Reclamo por faltante parcial validado para usuario confiable de larga data sin inconsistencias.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y monto razonable. | Reclamo por faltantes operativos en cuenta de alto valor e historial impecable.</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1741,6 +1750,7 @@
         </is>
       </c>
       <c r="AA12" t="inlineStr"/>
+      <c r="AB12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1843,6 +1853,7 @@
         </is>
       </c>
       <c r="AA13" t="inlineStr"/>
+      <c r="AB13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1937,21 +1948,22 @@
       </c>
       <c r="W14" t="inlineStr">
         <is>
-          <t>Usuario con 843 días de antigüedad y 0 flags de fraude. Reclamo operativo estándar por cobro tras cancelación, sin patrones abusivos ni palabras críticas.</t>
+          <t>Usuario con más de 2 años de antigüedad, historial limpio y única reclamación reciente. La cancelación del restaurante es un evento operativo coherente y verificable sin contradicciones.</t>
         </is>
       </c>
       <c r="X14" t="inlineStr"/>
       <c r="Y14" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z14" t="inlineStr"/>
       <c r="AA14" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude o inconsistencias operativas relevantes. | Solicitud de reembolso por cargo pendiente tras cancelación del restaurante en cuenta antigua y limpia.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo operativo legítimo sin señales de fraude o inconsistencia. | Solicitud de reembolso por cancelación operativa en cuenta establecida y sin riesgos previos.</t>
+        </is>
+      </c>
+      <c r="AB14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2054,6 +2066,7 @@
         </is>
       </c>
       <c r="AA15" t="inlineStr"/>
+      <c r="AB15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2148,21 +2161,22 @@
       </c>
       <c r="W16" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años y 0 flags de fraude. Reclamo por calidad de alimento sin inconsistencias ni patrones de abuso.</t>
+          <t>Usuario con antigüedad superior a 2 años y 0 flags de fraude. El reclamo es subjetivo pero coherente con fallas de calidad alimentaria, sin contradicciones evidentes.</t>
         </is>
       </c>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>reclamo_subjetivo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z16" t="inlineStr"/>
       <c r="AA16" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo coherente con perfil de usuario confiable y sin señales de fraude. | Reclamo legítimo por deterioro percibido en cuenta estable y sin historial negativo.</t>
-        </is>
-      </c>
+          <t>APROBAR: perfil de usuario confiable y reclamo sin señales de fraude o inconsistencia crítica. | Reclamo por olor desagradable en cuenta estable sin historial abusivo.</t>
+        </is>
+      </c>
+      <c r="AB16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2242,7 +2256,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
@@ -2252,26 +2266,27 @@
       </c>
       <c r="V17" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W17" t="inlineStr">
         <is>
-          <t>Cuenta nueva (75 días) con 6 reclamos en 90 días, lo que activa la regla de sospecha por múltiples reclamos en periodo reciente. El reclamo por cupón carece de evidencia objetiva y se combina con un patrón de alta frecuencia.</t>
+          <t>Cuenta nueva (75d) con alta frecuencia de reclamos (6 en 90d) y sin evidencia GPS. Requiere revisión para validar lógica de cupones vs patrón de uso.</t>
         </is>
       </c>
       <c r="X17" t="inlineStr"/>
       <c r="Y17" t="inlineStr">
         <is>
-          <t>antiguedad_moderada_con_alta_reincidencia | alta_frecuencia_reclamos | reclamo_subjetivo</t>
+          <t>antiguedad_moderada_con_alta_reincidencia | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr"/>
       <c r="AA17" t="inlineStr">
         <is>
-          <t>RECHAZAR: cuenta nueva con múltiples reclamos en 90 días y patrón de alta frecuencia que sugiere abuso potencial. | Reclamo por error de cupón en cuenta nueva con alta densidad de solicitudes en 90 días.</t>
-        </is>
-      </c>
+          <t>ESCALAR: cuenta nueva con múltiples reclamos y datos insuficientes para verificación automática, riesgo de abuso detectado. | Reclamo por error de cupón en cuenta reciente con alta densidad de solicitudes y falta de corroboración GPS.</t>
+        </is>
+      </c>
+      <c r="AB17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2366,21 +2381,22 @@
       </c>
       <c r="W18" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad moderada y 6 reclamos en 90 días. Evidencia GPS parcial y disputa de cobro generan ambigüedad operativa.</t>
+          <t>Reclamo por cobro tras cancelación del restaurante. Sin flags de fraude ni palabras críticas, pero la alta frecuencia (6 en 90d) y la evidencia GPS parcial generan ambigüedad operativa que requiere validación manual.</t>
         </is>
       </c>
       <c r="X18" t="inlineStr"/>
       <c r="Y18" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | evidencia_gps_parcial | compensacion_elevada</t>
+          <t>alta_frecuencia_reclamos | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z18" t="inlineStr"/>
       <c r="AA18" t="inlineStr">
         <is>
-          <t>ESCALAR: alta frecuencia de reclamos combinada con GPS parcial y naturaleza de disputa financiera requieren validación humana con pasarela/restaurante. | Reclamo por cargo pendiente tras cancelación del restaurante, con alta frecuencia de actividad y evidencia de ubicación incompleta.</t>
-        </is>
-      </c>
+          <t>ESCALAR: alta frecuencia de reclamos y evidencia GPS parcial requieren validación manual del estado real del pedido y política de reembolso. | Disputa de cobro por cancelación con patrón de frecuencia elevada y GPS inconclusa.</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2485,6 +2501,7 @@
         </is>
       </c>
       <c r="AA19" t="inlineStr"/>
+      <c r="AB19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2589,6 +2606,7 @@
         </is>
       </c>
       <c r="AA20" t="inlineStr"/>
+      <c r="AB20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2683,7 +2701,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>Usuario con 609 días de antigüedad y historial limpio. Reclamo por error de preparación sin contradicciones con la evidencia disponible. Monto solicitado dentro de parámetros normales y sin indicadores de abuso.</t>
+          <t>Usuario con antigüedad superior a un año, historial limpio y baja frecuencia de reclamos. El reclamo describe un error operativo común sin términos críticos ni inconsistencias.</t>
         </is>
       </c>
       <c r="X21" t="inlineStr"/>
@@ -2695,9 +2713,10 @@
       <c r="Z21" t="inlineStr"/>
       <c r="AA21" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Error operativo aislado en cuenta estable sin señales de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de riesgo. | Reclamo por producto incorrecto en cuenta estable sin indicadores de fraude.</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2777,7 +2796,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
@@ -2787,26 +2806,23 @@
       </c>
       <c r="V22" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W22" t="inlineStr">
         <is>
-          <t>Usuario con flag de fraude previo y alta frecuencia de reclamos (5 en 90d). La falta de confirmación GPS y la naturaleza subjetiva del reclamo (producto caducado) sin evidencia digital refuerzan el riesgo de abuso.</t>
+          <t>Historial con alta frecuencia de reclamos y ratio de compensación elevado, combinado con ausencia de evidencia GPS. La verificación de producto caducado requiere revisión manual.</t>
         </is>
       </c>
       <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr">
-        <is>
-          <t>flag_fraude_previo | alta_frecuencia_reclamos | entrega_gps_no_confirmada | reclamo_subjetivo</t>
-        </is>
-      </c>
+      <c r="Y22" t="inlineStr"/>
       <c r="Z22" t="inlineStr"/>
       <c r="AA22" t="inlineStr">
         <is>
-          <t>RECHAZAR: combinación de flag de fraude previo, alta frecuencia de reclamos y falta de evidencia GPS para validar una solicitud subjetiva. | Reclamo por producto caducado en cuenta con historial de fraude, alta densidad de solicitudes y sin validación geoespacial.</t>
-        </is>
-      </c>
+          <t>ESCALAR: combinación de alta frecuencia, ratio de compensación elevado y falta de evidencia GPS requiere validación humana. | Reclamo por vencimiento de producto en cuenta con patrón de compensaciones frecuentes y sin validación geolocalizada.</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2901,7 +2917,7 @@
       </c>
       <c r="W23" t="inlineStr">
         <is>
-          <t>Perfil limpio con 377 días de antigüedad y 0 flags. El reclamo corresponde a una discrepancia de precios/cupones, típica de errores operativos.</t>
+          <t>Usuario con antigüedad &gt;1 año y 0 flags de fraude. Reclamo por error de cupón sin inconsistencias críticas.</t>
         </is>
       </c>
       <c r="X23" t="inlineStr"/>
@@ -2913,9 +2929,10 @@
       <c r="Z23" t="inlineStr"/>
       <c r="AA23" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de abuso o inconsistencia crítica. | Reclamo por aplicación incorrecta de cupón en cuenta antigua sin historial de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo sin señales de fraude o patrones de abuso detectados. | Solicitud de ajuste por cupón no aplicado en cuenta estable sin historial abusivo.</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3018,6 +3035,7 @@
         </is>
       </c>
       <c r="AA24" t="inlineStr"/>
+      <c r="AB24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3112,21 +3130,22 @@
       </c>
       <c r="W25" t="inlineStr">
         <is>
-          <t>Usuario con 325 días de antigüedad y sin historial de fraude. El reclamo por ítem faltante es coherente con errores operativos habituales. No se detectan patrones de abuso, inconsistencias GPS críticas ni términos de riesgo.</t>
+          <t>Usuario con antigüedad de 325 días y 0 flags de fraude. Reclamo por faltante operativo sin señales de abuso, inconsistencia GPS o palabras críticas.</t>
         </is>
       </c>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z25" t="inlineStr"/>
       <c r="AA25" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sin riesgos detectados. | Reclamo estándar por producto faltante en cuenta con buen historial y sin señales de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente y sin señales de fraude detectadas. | Reclamo legítimo de faltante en cuenta verificada sin historial de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3221,21 +3240,22 @@
       </c>
       <c r="W26" t="inlineStr">
         <is>
-          <t>El perfil presenta señales de riesgo acumuladas: alta frecuencia de reclamos, flag de fraude previo, evidencia GPS parcial y ratio de compensación elevado, lo que contradice la coherencia esperada en un error operativo aislado.</t>
+          <t>Usuario con historial de 1 flag de fraude y 6 reclamos en 90 días. Evidencia GPS parcial que no respalda la afirmación de doble cobro.</t>
         </is>
       </c>
       <c r="X26" t="inlineStr"/>
       <c r="Y26" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_parcial | compensacion_elevada</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z26" t="inlineStr"/>
       <c r="AA26" t="inlineStr">
         <is>
-          <t>RECHAZAR: combinación de flag de fraude, alta frecuencia y GPS parcial indica patrón de abuso o inconsistencia verificable. | Reclamo por doble cobro en cuenta con historial negativo y evidencia logística incompleta.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: patrón de abuso confirmado por alta frecuencia de reclamos, flag de fraude previo e inconsistencia en evidencia GPS. | Reclamo de doble cobro en cuenta con alta frecuencia de incidencias y señal previa de fraude, sin validación geoespacial completa.</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3342,6 +3362,7 @@
         </is>
       </c>
       <c r="AA27" t="inlineStr"/>
+      <c r="AB27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3444,6 +3465,7 @@
         </is>
       </c>
       <c r="AA28" t="inlineStr"/>
+      <c r="AB28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3546,6 +3568,7 @@
         </is>
       </c>
       <c r="AA29" t="inlineStr"/>
+      <c r="AB29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3648,6 +3671,7 @@
         </is>
       </c>
       <c r="AA30" t="inlineStr"/>
+      <c r="AB30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3742,21 +3766,22 @@
       </c>
       <c r="W31" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, historial limpio y cero reclamos recientes. La omisión de elementos es un error operativo común y coherente.</t>
+          <t>Usuario con más de 3 años de antigüedad, historial limpio y cero reclamos recientes. La falta de salsas y cubiertos es un error operativo frecuente y coherente con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X31" t="inlineStr"/>
       <c r="Y31" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr"/>
       <c r="AA31" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario sin riesgos detectados. | Reclamo por artículos faltantes validado por perfil de usuario consolidado y sin indicadores de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario confiable y sin indicadores de abuso. | Reclamo por artículos faltantes en cuenta antigua y sin señales de fraude.</t>
+        </is>
+      </c>
+      <c r="AB31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3851,7 +3876,7 @@
       </c>
       <c r="W32" t="inlineStr">
         <is>
-          <t>Usuario con más de 2 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. La solicitud por producto caducado es un reclamo de calidad estándar sin contradicciones con la evidencia disponible ni términos críticos de riesgo legal o sanitario.</t>
+          <t>Usuario con 1016 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El reclamo por producto caducado es coherente y no activa umbrales de riesgo ni palabras críticas.</t>
         </is>
       </c>
       <c r="X32" t="inlineStr"/>
@@ -3863,9 +3888,10 @@
       <c r="Z32" t="inlineStr"/>
       <c r="AA32" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable, sin señales de riesgo y reclamo coherente con las reglas de negocio. | Reclamo de calidad alimentaria en cuenta antigua y limpia sin indicadores de fraude, abuso o inconsistencia operativa.</t>
-        </is>
-      </c>
+          <t>APROBAR: perfil de usuario confiable con historial limpio y reclamo plausible sin señales de fraude. | Reclamo de calidad alimentaria en cuenta veterana y limpia, sin inconsistencias operativas ni evidencia de abuso.</t>
+        </is>
+      </c>
+      <c r="AB32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3968,6 +3994,7 @@
         </is>
       </c>
       <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4062,21 +4089,22 @@
       </c>
       <c r="W34" t="inlineStr">
         <is>
-          <t>Usuario con 925 días de antigüedad, historial limpio y baja frecuencia de reclamos. Sin señales de fraude detectadas.</t>
+          <t>Perfil de usuario consolidado (&gt;2 años) con historial limpio y baja frecuencia. Ausencia de contradicciones GPS o palabras críticas. El reporte de no entrega es coherente con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X34" t="inlineStr"/>
       <c r="Y34" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z34" t="inlineStr"/>
       <c r="AA34" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de un usuario sin historial de fraude. | Reclamo por retraso y no entrega en cuenta antigua sin indicadores de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo basado en perfil conservador y ausencia de inconsistencias operativas o de fraude. | Solicitud por retraso/no entrega en cuenta antigua sin indicadores de fraude.</t>
+        </is>
+      </c>
+      <c r="AB34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4179,6 +4207,7 @@
         </is>
       </c>
       <c r="AA35" t="inlineStr"/>
+      <c r="AB35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4273,21 +4302,22 @@
       </c>
       <c r="W36" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad de 988 días, 0 flags de fraude y baja frecuencia de reclamos. La justificación de cancelación operativa es coherente y no contradice la evidencia disponible.</t>
+          <t>Usuario con antigüedad superior a 2 años, sin historial de fraude y baja frecuencia de reclamos. El motivo reportado (cancelación por falta de repartidor) es un fallo operativo estándar y coherente.</t>
         </is>
       </c>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z36" t="inlineStr"/>
       <c r="AA36" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario sano y sin indicadores de fraude. | Reclamo legítimo por cancelación de pedido en cuenta antigua y sin historial de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con el perfil del usuario y sin señales de fraude. | Reclamo por cancelación operativa en cuenta antigua y confiable sin indicadores de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4382,7 +4412,7 @@
       </c>
       <c r="W37" t="inlineStr">
         <is>
-          <t>El reclamo es subjetivo y la evidencia GPS es parcial, lo que impide verificar objetivamente el estado del producto. La existencia de un flag de fraude previo requiere validación manual.</t>
+          <t>Cuenta con antigüedad superior a un año y un flag previo, pero el reclamo es subjetivo y la evidencia GPS es parcial, lo que impide verificar objetivamente el estado del producto.</t>
         </is>
       </c>
       <c r="X37" t="inlineStr"/>
@@ -4394,9 +4424,10 @@
       <c r="Z37" t="inlineStr"/>
       <c r="AA37" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por GPS parcial y naturaleza subjetiva del reclamo en cuenta con flag previo. | Reclamo de calidad con evidencia limitada y historial mixto que exige revisión humana.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ambigüedad por evidencia GPS parcial y naturaleza subjetiva del reclamo, requiere revisión humana para validar fotos o reportes del restaurante/repartidor. | Reclamo por comida en mal estado sin evidencia objetiva clara ni GPS definitivo, con historial mixto.</t>
+        </is>
+      </c>
+      <c r="AB37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4491,7 +4522,7 @@
       </c>
       <c r="W38" t="inlineStr">
         <is>
-          <t>Usuario con 1760 días de antigüedad y 0 flags de fraude. El reclamo por retraso y repartidor inalcanzable es coherente con la pérdida de señal GPS. No se detectan patrones de abuso ni inconsistencias operativas.</t>
+          <t>Usuario con 1760 días de antigüedad, 0 flags y baja frecuencia de reclamos. El motivo (espera extrema e incapacidad de contacto con el repartidor) es coherente y no presenta indicadores de fraude.</t>
         </is>
       </c>
       <c r="X38" t="inlineStr"/>
@@ -4503,9 +4534,10 @@
       <c r="Z38" t="inlineStr"/>
       <c r="AA38" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y falta de evidencia GPS que refute la versión del cliente. | Cuenta antigua y limpia reporta no recepción por falla logística; la ausencia de GPS no contradice el reporte y el perfil sugiere legitimidad.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo respaldado por perfil de usuario altamente confiable y ausencia de señales de abuso o inconsistencias graves. | Reclamo por no entrega tras larga espera en cuenta antigua y confiable, con GPS perdido pero sin contradicciones operativas.</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4600,21 +4632,22 @@
       </c>
       <c r="W39" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. La cancelación por falta de repartidor es un evento operativo coherente y verificable.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y frecuencia de reclamos baja. El motivo de cancelación por falta de repartidor es un evento operativo común y coherente. No se detectan indicadores de abuso o inconsistencia.</t>
         </is>
       </c>
       <c r="X39" t="inlineStr"/>
       <c r="Y39" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable con historial limpio y motivo operativo válido. | Reclamo legítimo por cancelación operativa en cuenta antigua y limpia sin inconsistencias.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de fraude. | Reclamo legítimo por cancelación operativa en cuenta establecida y sin historial negativo.</t>
+        </is>
+      </c>
+      <c r="AB39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4709,21 +4742,22 @@
       </c>
       <c r="W40" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, sin historial de fraude y baja frecuencia de reclamos. El reporte de bebida incorrecta es coherente con un fallo operativo estándar.</t>
+          <t>Perfil de usuario altamente confiable con casi 3 años de antigüedad, 0 flags y baja frecuencia de reclamos. El monto solicitado es razonable y no existen inconsistencias que sugieran fraude.</t>
         </is>
       </c>
       <c r="X40" t="inlineStr"/>
       <c r="Y40" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z40" t="inlineStr"/>
       <c r="AA40" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario estable y monto dentro de parámetros normales. | Reclamo por producto equivocado en cuenta antigua y confiable, sin indicadores de abuso o inconsistencia crítica.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con un perfil de usuario sin historial negativo y sin señales de fraude. | Error operativo de surtido en cuenta antigua y limpia, sin indicadores de riesgo o abuso.</t>
+        </is>
+      </c>
+      <c r="AB40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4826,6 +4860,7 @@
         </is>
       </c>
       <c r="AA41" t="inlineStr"/>
+      <c r="AB41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4920,7 +4955,7 @@
       </c>
       <c r="W42" t="inlineStr">
         <is>
-          <t>Usuario con 1765 días de antigüedad, 0 flags y baja frecuencia de reclamos. Queja por retraso operativo coherente y sin evidencia contradictoria.</t>
+          <t>Usuario con 4+ años de antigüedad, sin flags de fraude y baja frecuencia de reclamos. El retraso es un incidente operativo común y coherente con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X42" t="inlineStr"/>
@@ -4932,9 +4967,10 @@
       <c r="Z42" t="inlineStr"/>
       <c r="AA42" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo por demora en entrega de usuario histórico sin señales de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y ausencia de indicadores de fraude. | Reclamo por retraso de entrega en cuenta antigua y limpia, sin inconsistencias ni señales de abuso.</t>
+        </is>
+      </c>
+      <c r="AB42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -5029,21 +5065,22 @@
       </c>
       <c r="W43" t="inlineStr">
         <is>
-          <t>Cuenta con 1 flag de fraude previo y evidencia GPS parcial para un reclamo de artículos faltantes difícil de verificar objetivamente.</t>
+          <t>Usuario con 1 flag de fraude previo y evidencia GPS parcial para un reclamo de artículos faltantes que requiere verificación manual.</t>
         </is>
       </c>
       <c r="X43" t="inlineStr"/>
       <c r="Y43" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z43" t="inlineStr"/>
       <c r="AA43" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de flag de fraude previo, GPS parcial y naturaleza subjetiva del reclamo requiere revisión humana para evitar errores operativos o falsos positivos. | Reclamo por falta de salsas y cubiertos en cuenta con historial mixto y GPS inconclusa.</t>
-        </is>
-      </c>
+          <t>ESCALAR: presencia de flag de fraude previo y GPS parcial requieren validación humana del inventario faltante. | Reclamo por falta de salsas y cubiertos en cuenta con historial mixto y cobertura GPS incompleta.</t>
+        </is>
+      </c>
+      <c r="AB43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -5123,7 +5160,7 @@
       </c>
       <c r="T44" t="inlineStr">
         <is>
-          <t>APROBAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U44" t="inlineStr">
@@ -5133,26 +5170,23 @@
       </c>
       <c r="V44" t="inlineStr">
         <is>
-          <t>APROBAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W44" t="inlineStr">
         <is>
-          <t>Usuario con 1796 días de antigüedad y 0 flags de fraude. Aunque la evidencia GPS está perdida, el perfil extremadamente conservador y la baja frecuencia de reclamos indican un incidente operativo legítimo.</t>
+          <t>Perfil de usuario altamente confiable (cuenta antigua, 0 flags, baja frecuencia). La ausencia de evidencia GPS genera ambigüedad operativa que impide la validación automática.</t>
         </is>
       </c>
       <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr">
-        <is>
-          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
-        </is>
-      </c>
+      <c r="Y44" t="inlineStr"/>
       <c r="Z44" t="inlineStr"/>
       <c r="AA44" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario altamente confiable y sin señales de abuso que justifican la compensación pese a la falta de validación GPS. | Reclamo por entrega no recibida en cuenta veterana sin antecedentes, con evidencia GPS incompleta.</t>
-        </is>
-      </c>
+          <t>ESCALAR: evidencia GPS insuficiente ('señal perdida') requiere revisión manual de registros del repartidor para confirmar ubicación de entrega. | Disputa de entrega sin rastreo GPS en cuenta limpia y antigua.</t>
+        </is>
+      </c>
+      <c r="AB44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -5247,7 +5281,7 @@
       </c>
       <c r="W45" t="inlineStr">
         <is>
-          <t>Usuario con 510 días de antigüedad, 0 flags de fraude y 0 reclamos recientes. El motivo descrito corresponde a un error de facturación estándar por cancelación del restaurante, sin inconsistencias ni señales de riesgo.</t>
+          <t>Usuario con 510 días de antigüedad, historial limpio y 0 reclamos recientes. El motivo de cancelación del restaurante es coherente y el monto solicitado está dentro de parámetros normales.</t>
         </is>
       </c>
       <c r="X45" t="inlineStr"/>
@@ -5259,9 +5293,10 @@
       <c r="Z45" t="inlineStr"/>
       <c r="AA45" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con la evidencia disponible y perfil de usuario confiable. | Cobro indebido por cancelación operativa en cuenta estable y sin historial de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con evidencia operativa, usuario sin señales de fraude ni patrones abusivos. | Reclamo operativo por cancelación de restaurante y cobro pendiente en cuenta establecida sin historial de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -5356,7 +5391,7 @@
       </c>
       <c r="W46" t="inlineStr">
         <is>
-          <t>Usuario con 4+ años de antigüedad y 0 flags de fraude. Reclamo de discrepancia monetaria sin indicadores de abuso o inconsistencia crítica.</t>
+          <t>Usuario con 1706 días de antigüedad y 0 flags de fraude. El reclamo por discrepancia de cobro es coherente con errores operativos comunes y no presenta indicadores de abuso.</t>
         </is>
       </c>
       <c r="X46" t="inlineStr"/>
@@ -5368,9 +5403,10 @@
       <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo de usuario con historial limpio y baja frecuencia. | Discrepancia de cobro en cuenta antigua y confiable, sin señales de fraude ni palabras críticas.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente de usuario confiable sin patrones de fraude. | Discrepancia de cobro en cuenta antigua y limpia sin señales de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -5477,6 +5513,7 @@
         </is>
       </c>
       <c r="AA47" t="inlineStr"/>
+      <c r="AB47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5581,6 +5618,7 @@
         </is>
       </c>
       <c r="AA48" t="inlineStr"/>
+      <c r="AB48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5675,21 +5713,22 @@
       </c>
       <c r="W49" t="inlineStr">
         <is>
-          <t>Usuario de larga antigüedad (1655d) sin historial de fraude ni alta frecuencia de reclamos. El motivo de cancelación por falta de repartidor es coherente con un error operativo estándar. No se activaron reglas de riesgo ni palabras críticas.</t>
+          <t>Usuario con 4+ años de antigüedad y 0 flags de fraude. Reclamo por cancelación operativa sin inconsistencias ni señales de abuso.</t>
         </is>
       </c>
       <c r="X49" t="inlineStr"/>
       <c r="Y49" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z49" t="inlineStr"/>
       <c r="AA49" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin indicios de fraude. | Reclamo por cancelación operativa en cuenta confiable sin señales de abuso o inconsistencias.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario sin riesgos. | Solicitud de reembolso por cancelación de pedido sin repartidor en cuenta antigua y confiable.</t>
+        </is>
+      </c>
+      <c r="AB49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5792,6 +5831,7 @@
         </is>
       </c>
       <c r="AA50" t="inlineStr"/>
+      <c r="AB50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5886,21 +5926,18 @@
       </c>
       <c r="W51" t="inlineStr">
         <is>
-          <t>Perfil limpio con antigüedad &gt;8 meses y baja frecuencia. Discrepancia de cobro típica sin indicadores de fraude.</t>
+          <t>Usuario con 306 días de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La discrepancia de monto es un error operativo estándar verificable por sistema.</t>
         </is>
       </c>
       <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr">
-        <is>
-          <t>reclamo_subjetivo | evidencia_gps_parcial</t>
-        </is>
-      </c>
+      <c r="Y51" t="inlineStr"/>
       <c r="Z51" t="inlineStr"/>
       <c r="AA51" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo de discrepancia administrativa sin señales de abuso o inconsistencia crítica. | Reclamo por diferencia de monto en resumen. Usuario con historial estable y GPS parcial no relevante para el tipo de incidencia.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de tipo financiero sin indicadores de fraude. | Reclamo por diferencia en resumen de cargo. Perfil conservador sin señales de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5995,21 +6032,18 @@
       </c>
       <c r="W52" t="inlineStr">
         <is>
-          <t>Usuario con más de 2 años de antigüedad, 0 flags y 0 reclamos recientes. El reclamo por artículos faltantes es un error operativo común y coherente. La ausencia de GPS no aplica a este tipo de incidencia.</t>
+          <t>Usuario con antigüedad de 906 días, sin flags de fraude y sin reclamos recientes. El reporte de artículos faltantes es un error operativo común y coherente, sin contradicciones con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr">
-        <is>
-          <t>reclamo_subjetivo</t>
-        </is>
-      </c>
+      <c r="Y52" t="inlineStr"/>
       <c r="Z52" t="inlineStr"/>
       <c r="AA52" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Reclamo estándar de artículos faltantes en cuenta antigua y limpia sin indicadores de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Incidencia operativa por falta de salsas y cubiertos en cuenta antigua y sin historial de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -6112,6 +6146,7 @@
         </is>
       </c>
       <c r="AA53" t="inlineStr"/>
+      <c r="AB53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -6206,21 +6241,22 @@
       </c>
       <c r="W54" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. Aunque la evidencia GPS está ausente, el perfil del usuario es conservador y el reclamo es coherente con disputas operativas comunes.</t>
+          <t>Usuario con más de 3 años de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La pérdida de señal GPS impide verificar la entrega, pero la narrativa es coherente y el perfil es conservador.</t>
         </is>
       </c>
       <c r="X54" t="inlineStr"/>
       <c r="Y54" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z54" t="inlineStr"/>
       <c r="AA54" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable sin señales de fraude, se compensa ante la falta de evidencia GPS concluyente. | Reclamo por entrega marcada incorrectamente en cuenta antigua y limpia, sin evidencia GPS disponible para verificación objetiva.</t>
-        </is>
-      </c>
+          <t>APROBAR: perfil de usuario confiable sin señales de fraude, la ausencia de GPS se compensa con historial positivo y narrativa plausible. | Reclamo por entrega no recibida en cuenta antigua y limpia, sin evidencia GPS contradictoria.</t>
+        </is>
+      </c>
+      <c r="AB54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -6323,6 +6359,7 @@
         </is>
       </c>
       <c r="AA55" t="inlineStr"/>
+      <c r="AB55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -6425,6 +6462,7 @@
         </is>
       </c>
       <c r="AA56" t="inlineStr"/>
+      <c r="AB56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -6519,21 +6557,22 @@
       </c>
       <c r="W57" t="inlineStr">
         <is>
-          <t>Alta frecuencia de reclamos (6 en 90d) combinada con flag de fraude previo y ausencia de evidencia GPS valida.</t>
+          <t>Usuario con flag de fraude previo y 6 reclamos en 90 días. Ratio de compensación elevado (0.81) sin evidencia GPS que respalde la cancelación reportada.</t>
         </is>
       </c>
       <c r="X57" t="inlineStr"/>
       <c r="Y57" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z57" t="inlineStr"/>
       <c r="AA57" t="inlineStr">
         <is>
-          <t>RECHAZAR: patrón de alta frecuencia y flag de fraude previo sin corroboración GPS. | Reclamo por cancelación operativa en cuenta con historial de reincidencia y sin validación geolocal.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: evidencia clara de abuso por historial con flag previo, alta frecuencia de reclamos y ratio de compensación elevado sin validación técnica. | Patrón de abuso confirmado por alta frecuencia, historial negativo y compensación desproporcionada sin soporte técnico.</t>
+        </is>
+      </c>
+      <c r="AB57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6628,21 +6667,22 @@
       </c>
       <c r="W58" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad de 373 días y 0 flags de fraude. El reclamo por calidad de alimento es coherente y el monto está dentro de parámetros normales. La evidencia GPS es parcial pero no contradice el reporte.</t>
+          <t>Usuario con 373 días de antigüedad y 0 flags de fraude. Frecuencia de reclamos moderada y ratio de compensación aceptable. La evidencia GPS es parcial pero no contradice el reporte, y el reclamo por calidad alimentaria es coherente con el contexto.</t>
         </is>
       </c>
       <c r="X58" t="inlineStr"/>
       <c r="Y58" t="inlineStr">
         <is>
-          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
+          <t>reclamo_subjetivo | entrega_gps_parcial</t>
         </is>
       </c>
       <c r="Z58" t="inlineStr"/>
       <c r="AA58" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin indicadores de fraude, consistente con políticas de compensación por calidad. | Reclamo por estado del alimento en cuenta antigua y limpia, sin patrones de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo por calidad de producto en cuenta sana con evidencia GPS ambigua pero sin inconsistencias.</t>
+        </is>
+      </c>
+      <c r="AB58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -6747,6 +6787,7 @@
         </is>
       </c>
       <c r="AA59" t="inlineStr"/>
+      <c r="AB59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -6849,6 +6890,7 @@
         </is>
       </c>
       <c r="AA60" t="inlineStr"/>
+      <c r="AB60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -6951,6 +6993,7 @@
         </is>
       </c>
       <c r="AA61" t="inlineStr"/>
+      <c r="AB61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -7057,6 +7100,7 @@
         </is>
       </c>
       <c r="AA62" t="inlineStr"/>
+      <c r="AB62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -7163,6 +7207,7 @@
         </is>
       </c>
       <c r="AA63" t="inlineStr"/>
+      <c r="AB63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -7265,6 +7310,7 @@
         </is>
       </c>
       <c r="AA64" t="inlineStr"/>
+      <c r="AB64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -7359,21 +7405,22 @@
       </c>
       <c r="W65" t="inlineStr">
         <is>
-          <t>Reclamo de discrepancia de cargo con GPS perdido y un flag de fraude previo. La falta de evidencia geolocalizada y el historial mixto impiden una decisión automatizada segura.</t>
+          <t>Usuario con flag de fraude previo y GPS sin señal. El reclamo por discrepancia de cobro requiere validación manual de logs internos.</t>
         </is>
       </c>
       <c r="X65" t="inlineStr"/>
       <c r="Y65" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | flag_fraude_previo | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z65" t="inlineStr"/>
       <c r="AA65" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por GPS perdido y flag previo en reclamo de facturación requiere revisión humana. | Disputa de facturación con evidencia GPS insuficiente y antecedentes de riesgo moderado que requieren validación manual.</t>
-        </is>
-      </c>
+          <t>ESCALAR: requiere auditoría manual para conciliar cobros y evaluar impacto del flag previo ante GPS perdida. | Discrepancia monetaria en cuenta con historial de riesgo y sin evidencia geolocalizable.</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -7453,7 +7500,7 @@
       </c>
       <c r="T66" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U66" t="inlineStr">
@@ -7463,26 +7510,27 @@
       </c>
       <c r="V66" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W66" t="inlineStr">
         <is>
-          <t>Cuenta con 1 flag de fraude previo y 6 reclamos en 90 días. La señal GPS perdida imposibilita verificar el retraso alegado, y el estado 'fría' es subjetivo. Se requiere análisis humano para equilibrar riesgo de fraude con posible queja legítima.</t>
+          <t>Cuenta con 1 flag de fraude previo y 6 reclamos en 90 días. La evidencia GPS está perdida y el motivo (comida fría) es subjetivo y difícil de verificar objetivamente.</t>
         </is>
       </c>
       <c r="X66" t="inlineStr"/>
       <c r="Y66" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z66" t="inlineStr"/>
       <c r="AA66" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de alta frecuencia de reclamos, flag de fraude previo y falta de evidencia GPS objetiva requiere revisión manual para determinar legitimidad. | Reclamo por retraso y temperatura inadecuada en cuenta con historial de riesgo y evidencia GPS incompleta.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: patrón de alta frecuencia combinado con flag de fraude previo y ausencia de evidencia GPS objetiva valida el rechazo por posible abuso. | Reclamo por temperatura del pedido sin soporte GPS verificable en usuario con historial de fraude y alta frecuencia.</t>
+        </is>
+      </c>
+      <c r="AB66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -7577,7 +7625,7 @@
       </c>
       <c r="W67" t="inlineStr">
         <is>
-          <t>Usuario con más de 2 años de antigüedad y 0 flags de fraude. El reclamo por error de cupón es coherente y no activa umbrales de riesgo operativos.</t>
+          <t>Usuario con antigüedad superior a 2 años, sin flags de fraude y baja frecuencia de reclamos. El error en la aplicación del cupón es un incidente operativo coherente y verificable.</t>
         </is>
       </c>
       <c r="X67" t="inlineStr"/>
@@ -7589,9 +7637,10 @@
       <c r="Z67" t="inlineStr"/>
       <c r="AA67" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario confiable sin inconsistencias ni riesgos detectados. | Disputa por descuento no aplicado en cuenta antigua sin historial de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable. | Error técnico en descuento en cuenta antigua sin historial negativo.</t>
+        </is>
+      </c>
+      <c r="AB67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -7686,7 +7735,7 @@
       </c>
       <c r="W68" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado es razonable y no contiene palabras críticas. La falta de confirmación GPS no contradice el reporte de ítem faltante.</t>
+          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. El reclamo por ítem faltante es un error operativo común y coherente. No se activaron reglas de riesgo ni hay señales de abuso.</t>
         </is>
       </c>
       <c r="X68" t="inlineStr"/>
@@ -7698,9 +7747,10 @@
       <c r="Z68" t="inlineStr"/>
       <c r="AA68" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo por producto faltante en cuenta antigua y sin historial de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin señales de fraude. | Error operativo de restaurante (bebida faltante) en usuario confiable de larga data sin patrones sospechosos.</t>
+        </is>
+      </c>
+      <c r="AB68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -7805,6 +7855,7 @@
         </is>
       </c>
       <c r="AA69" t="inlineStr"/>
+      <c r="AB69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -7899,7 +7950,7 @@
       </c>
       <c r="W70" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad y sin historial de fraude. El reclamo por doble cobro es un error financiero verificable, sin patrones de abuso ni inconsistencias.</t>
+          <t>Cuenta antigua con 0 flags y baja frecuencia. Monto y ratio dentro de parámetros normales. Sin contradicciones ni términos críticos.</t>
         </is>
       </c>
       <c r="X70" t="inlineStr"/>
@@ -7911,9 +7962,10 @@
       <c r="Z70" t="inlineStr"/>
       <c r="AA70" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario con trayectoria consolidada y sin indicadores de fraude. | Duplicidad de cobro reportada en cuenta antigua y confiable, sin señales de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: perfil de usuario sano y consolidado sin señales de fraude detectadas. | Reclamo por doble cobro en usuario consolidado sin indicadores de riesgo operativo.</t>
+        </is>
+      </c>
+      <c r="AB70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -8008,21 +8060,22 @@
       </c>
       <c r="W71" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. El reclamo por error de cupón es un incidente operativo común y coherente.</t>
+          <t>Usuario con 1660 días de antigüedad y 0 flags de fraude. Reclamo por error de cupón sin señales de inconsistencia o abuso.</t>
         </is>
       </c>
       <c r="X71" t="inlineStr"/>
       <c r="Y71" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z71" t="inlineStr"/>
       <c r="AA71" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude ni inconsistencias operativas. | Error técnico en la aplicación de descuento para cuenta confiable de larga data.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de usuario antiguo sin historial de fraude ni patrones sospechosos. | Error operativo en la aplicación de descuento para cuenta confiable de larga data.</t>
+        </is>
+      </c>
+      <c r="AB71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -8117,21 +8170,22 @@
       </c>
       <c r="W72" t="inlineStr">
         <is>
-          <t>Usuario con flag de fraude previo, alta frecuencia de reclamos (4 en 90d) y ratio de compensación elevado (0.91). Ausencia de evidencia GPS que valide la entrega o el faltante reportado.</t>
+          <t>Historial con flag de fraude previo, alta frecuencia de reclamos y ratio de compensación elevado sugieren patrón de abuso.</t>
         </is>
       </c>
       <c r="X72" t="inlineStr"/>
       <c r="Y72" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | compensacion_elevada | alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
+          <t>flag_fraude_previo | alta_frecuencia_reclamos | compensacion_elevada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z72" t="inlineStr"/>
       <c r="AA72" t="inlineStr">
         <is>
-          <t>RECHAZAR: combinación de flag de fraude, alta frecuencia y ratio de compensación elevado sin evidencia GPS confirma patrón de abuso. | Reclamo por artículos faltantes en cuenta con historial de riesgo y ratio de compensación alto, sin soporte geoespacial.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: combinación de flag de fraude previo, alta frecuencia de reclamos y ratio de compensación elevado indica riesgo de abuso sistemático. | Reclamo por faltantes sin evidencia verificable en usuario con historial de riesgo y alta tasa de compensaciones.</t>
+        </is>
+      </c>
+      <c r="AB72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -8226,7 +8280,7 @@
       </c>
       <c r="W73" t="inlineStr">
         <is>
-          <t>El reclamo contiene el término 'alergia', un indicador crítico de riesgo sanitario y legal que activa protocolos de seguridad de marca y exige revisión humana.</t>
+          <t>El reclamo contiene la palabra 'alergia', lo que activa la regla de palabras críticas de seguridad de marca. Aunque el usuario tiene un perfil limpio y antigüedad alta, la mención de un riesgo de salud requiere revisión humana para evitar responsabilidades legales o daños a la reputación.</t>
         </is>
       </c>
       <c r="X73" t="inlineStr">
@@ -8247,9 +8301,10 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t>ESCALAR: mención de término crítico de salud que implica responsabilidad legal y sanitaria, requiriendo validación manual conforme a políticas de seguridad de marca. | Usuario antiguo sin historial de fraude reporta error en pedido por alergia alimentaria. Aunque el perfil es sano y la frecuencia es baja, la mención de riesgo de salud obliga a escalar.</t>
-        </is>
-      </c>
+          <t>ESCALAR: mención de término crítico ('alergia') que implica riesgo de salud y requiere validación humana antes de resolver. | Reclamo por error de restaurante en cuenta antigua, pero la mención de alergia obliga a escalar por protocolo de seguridad y salud.</t>
+        </is>
+      </c>
+      <c r="AB73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -8344,7 +8399,7 @@
       </c>
       <c r="W74" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años, sin flags de fraude y baja frecuencia de reclamos. El error de entrega coincide con un incidente operativo común.</t>
+          <t>Usuario con antigüedad superior a 4 años y 0 flags de fraude. Reclamo por ítem incorrecto sin señales de abuso o inconsistencia crítica.</t>
         </is>
       </c>
       <c r="X74" t="inlineStr"/>
@@ -8356,9 +8411,10 @@
       <c r="Z74" t="inlineStr"/>
       <c r="AA74" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por producto incorrecto en cuenta antigua y sin historial de riesgo. Sin inconsistencias ni señales de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Error operativo menor en cuenta antigua y limpia. Sin evidencia de fraude.</t>
+        </is>
+      </c>
+      <c r="AB74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -8453,7 +8509,7 @@
       </c>
       <c r="W75" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas que exige revisión humana por implicaciones de salud y responsabilidad civil. Aunque el usuario tiene un flag de fraude previo y GPS no confirmado, el riesgo de marca/salud domina la decisión.</t>
+          <t>El reclamo menciona explícitamente 'alergia', activando la regla de palabras críticas de seguridad de marca que requiere revisión humana inmediata para mitigar riesgos sanitarios y legales.</t>
         </is>
       </c>
       <c r="X75" t="inlineStr">
@@ -8464,7 +8520,7 @@
       </c>
       <c r="Y75" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | flag_fraude_previo | entrega_gps_no_confirmada</t>
+          <t>palabras_criticas_seguridad</t>
         </is>
       </c>
       <c r="Z75" t="inlineStr">
@@ -8474,9 +8530,10 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabra crítica 'alergia' que implica riesgo de salud y posible responsabilidad legal, requiriendo validación humana obligatoria según política de marca. | Reclamo por alergia alimentaria en cuenta con historial mixto y sin evidencia GPS, sujeto a revisión por riesgo legal y de salud.</t>
-        </is>
-      </c>
+          <t>ESCALAR: contiene palabra crítica ('alergia') que implica riesgo de salud/legal, requiriendo validación humana según protocolo de seguridad de marca. | Reclamo por posible reacción alérgica en cuenta con 1 flag previo y GPS no confirmada, escalado automáticamente por término crítico de salud.</t>
+        </is>
+      </c>
+      <c r="AB75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -8581,6 +8638,7 @@
         </is>
       </c>
       <c r="AA76" t="inlineStr"/>
+      <c r="AB76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -8675,21 +8733,22 @@
       </c>
       <c r="W77" t="inlineStr">
         <is>
-          <t>GPS perdido impide verificar la entrega. Usuario con antigüedad y perfil limpio, pero la falta de evidencia objetiva genera ambigüedad.</t>
+          <t>Perfil de usuario limpio sin historial de fraude ni alta frecuencia. La pérdida de señal GPS impide verificar objetivamente la entrega, generando ambigüedad.</t>
         </is>
       </c>
       <c r="X77" t="inlineStr"/>
       <c r="Y77" t="inlineStr">
         <is>
-          <t>evidencia_gps_parcial | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z77" t="inlineStr"/>
       <c r="AA77" t="inlineStr">
         <is>
-          <t>ESCALAR: evidencia GPS perdida genera ambigüedad que requiere revisión humana para validar la entrega. | Reclamo de no recepción con señal GPS perdida y sin indicadores de fraude, requiriendo validación manual.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ausencia de evidencia GPS objetiva requiere validación manual para evitar errores operativos o fraude encubierto. | Reclamo por no recepción con evidencia geolocalizada ausente en cuenta con historial conservador.</t>
+        </is>
+      </c>
+      <c r="AB77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -8784,7 +8843,7 @@
       </c>
       <c r="W78" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 4 años, sin historial de fraude ni reclamos recientes. El retraso reportado es un incidente operativo común y coherente con la promesa de entrega.</t>
+          <t>Usuario con 4+ años de antigüedad y perfil limpio sin reclamos previos. El retraso reportado es coherente y no presenta indicadores de fraude.</t>
         </is>
       </c>
       <c r="X78" t="inlineStr"/>
@@ -8796,9 +8855,10 @@
       <c r="Z78" t="inlineStr"/>
       <c r="AA78" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de alto riesgo negativo y motivo operativo coherente. | Reclamo por retraso en entrega de usuario veterano y confiable. Sin señales de abuso o contradicciones graves.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de usuario con historial impecable y sin señales de abuso. | Reclamo por retraso de entrega en cuenta antigua y confiable. Señal GPS perdida pero sin contradicción con el reporte.</t>
+        </is>
+      </c>
+      <c r="AB78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -8901,6 +8961,7 @@
         </is>
       </c>
       <c r="AA79" t="inlineStr"/>
+      <c r="AB79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -9005,6 +9066,7 @@
         </is>
       </c>
       <c r="AA80" t="inlineStr"/>
+      <c r="AB80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -9107,6 +9169,7 @@
         </is>
       </c>
       <c r="AA81" t="inlineStr"/>
+      <c r="AB81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -9209,6 +9272,7 @@
         </is>
       </c>
       <c r="AA82" t="inlineStr"/>
+      <c r="AB82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -9303,7 +9367,7 @@
       </c>
       <c r="W83" t="inlineStr">
         <is>
-          <t>Usuario antiguo (1598d) sin flags de fraude y baja frecuencia de reclamos. El retraso de 1.5h es una causa coherente para que la comida pierda calidad. Monto dentro de límites y ratio aceptable.</t>
+          <t>Usuario con antigüedad superior a 4 años, sin flags de fraude y frecuencia baja de reclamos. El retraso reportado es un motivo válido y el monto solicitado está dentro del rango normal.</t>
         </is>
       </c>
       <c r="X83" t="inlineStr"/>
@@ -9315,9 +9379,10 @@
       <c r="Z83" t="inlineStr"/>
       <c r="AA83" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en historial positivo, monto controlado y justificación coherente con el retraso reportado. | Reclamo por retraso y calidad en cuenta antigua y limpia. Sin inconsistencias ni señales de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo basado en historial limpio, antigüedad alta y monto dentro de parámetros normales. | Reclamo por retraso en entrega en cuenta antigua y limpia, consistente con el perfil del usuario.</t>
+        </is>
+      </c>
+      <c r="AB83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -9412,21 +9477,22 @@
       </c>
       <c r="W84" t="inlineStr">
         <is>
-          <t>Usuario con 474 días de antigüedad y 0 flags de fraude. La evidencia GPS no confirma la entrega, por lo que no existe contradicción objetiva con su reporte. Bajo riesgo de abuso.</t>
+          <t>Usuario con 474 días de antigüedad, 0 flags de fraude y frecuencia de reclamos dentro de lo normal. Al no existir evidencia GPS que confirme la entrega, no hay contradicción objetiva que respalde un rechazo.</t>
         </is>
       </c>
       <c r="X84" t="inlineStr"/>
       <c r="Y84" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z84" t="inlineStr"/>
       <c r="AA84" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude ni evidencia contradictoria. | Disputa por entrega no recibida en cuenta limpia con evidencia GPS inconclusa.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y ausencia de señales de abuso. | Disputa de entrega no verificable por GPS en cuenta con historial limpio y monto razonable.</t>
+        </is>
+      </c>
+      <c r="AB84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -9529,6 +9595,7 @@
         </is>
       </c>
       <c r="AA85" t="inlineStr"/>
+      <c r="AB85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -9623,21 +9690,22 @@
       </c>
       <c r="W86" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad estable (704d), historial limpio y baja frecuencia. El motivo de cancelación por falta de repartidor es coherente y el monto solicitado es razonable. La pérdida de señal GPS no contradice la evidencia operativa.</t>
+          <t>Usuario con 704 días de antigüedad y 0 flags de fraude. El motivo de cancelación por falta de repartidor es operativo y coherente. No se activan reglas de fraude, el monto solicitado está dentro del umbral y la frecuencia es baja.</t>
         </is>
       </c>
       <c r="X86" t="inlineStr"/>
       <c r="Y86" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z86" t="inlineStr"/>
       <c r="AA86" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario confiable. | Reclamo operativo estándar por cancelación de pedido en cuenta estable sin señales de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo sin señales de fraude, consistente con el contexto operativo y perfil de usuario sano. | Reclamo operativo estándar por cancelación de plataforma en cuenta antigua y sin historial negativo.</t>
+        </is>
+      </c>
+      <c r="AB86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -9732,7 +9800,7 @@
       </c>
       <c r="W87" t="inlineStr">
         <is>
-          <t>Usuario antiguo (1222d) con 0 flags y baja frecuencia de reclamos. Aunque la señal GPS se perdió, la coherencia del reporte y el perfil conservador del cliente respaldan la acción.</t>
+          <t>Usuario con antigüedad superior a 3 años, 0 flags de fraude y baja frecuencia de reclamos. La narrativa de espera prolongada y falta de respuesta del conductor es coherente con la pérdida de señal GPS reportada.</t>
         </is>
       </c>
       <c r="X87" t="inlineStr"/>
@@ -9744,9 +9812,10 @@
       <c r="Z87" t="inlineStr"/>
       <c r="AA87" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de alto confianza sin contradicciones graves, se autoriza ante ausencia de evidencia GPS que refute el reclamo. | Reclamo por no entrega/retraso en cuenta confiable con evidencia GPS ausente pero sin indicadores de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de usuario antiguo sin señales de fraude, narrativa coherente ante ausencia de datos GPS. | Reclamo por entrega no completada en cuenta confiable y antigua, sin evidencia GPS pero con perfil limpio y relato consistente.</t>
+        </is>
+      </c>
+      <c r="AB87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -9853,6 +9922,7 @@
         </is>
       </c>
       <c r="AA88" t="inlineStr"/>
+      <c r="AB88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -9947,7 +10017,7 @@
       </c>
       <c r="W89" t="inlineStr">
         <is>
-          <t>Usuario con 522 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El perfil es conservador y no presenta indicadores de abuso. Aunque el GPS no confirma la entrega, la ausencia de señales de riesgo y la naturaleza del reclamo apuntan a un error operativo legítimo.</t>
+          <t>Usuario con 522 días de antigüedad y historial limpio. Reclamo por producto faltante sin contradicciones ni señales de fraude.</t>
         </is>
       </c>
       <c r="X89" t="inlineStr"/>
@@ -9959,9 +10029,10 @@
       <c r="Z89" t="inlineStr"/>
       <c r="AA89" t="inlineStr">
         <is>
-          <t>APROBAR: perfil de usuario confiable sin historial de fraude o alta frecuencia, se aprueba como error operativo. | Reclamo por producto faltante en cuenta limpia y antigua, sin evidencia GPS pero sin patrones sospechosos.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de riesgo. | Reclamo operativo estándar en cuenta verificada sin patrones abusivos.</t>
+        </is>
+      </c>
+      <c r="AB89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -10064,6 +10135,7 @@
         </is>
       </c>
       <c r="AA90" t="inlineStr"/>
+      <c r="AB90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -10158,21 +10230,22 @@
       </c>
       <c r="W91" t="inlineStr">
         <is>
-          <t>Usuario antiguo (757d) con historial limpio y baja frecuencia. Cancelación por falta de repartidor es un evento operativo coherente y sin contradicciones.</t>
+          <t>Usuario con 757 días de antigüedad, 0 flags y 1 reclamo en 90 días. La cancelación por falta de repartidor es un evento operativo coherente. No hay contradicciones GPS ni palabras críticas.</t>
         </is>
       </c>
       <c r="X91" t="inlineStr"/>
       <c r="Y91" t="inlineStr">
         <is>
-          <t>antiguedad_moderada_con_alta_reincidencia</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z91" t="inlineStr"/>
       <c r="AA91" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario confiable y motivo operativo coherente. | Reclamo por cancelación operativa en cuenta estable sin señales de fraude o inconsistencias.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con el contexto operativo y perfil de usuario confiable. | Reclamo estándar por cancelación operativa en cuenta antigua y sin historial de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -10275,6 +10348,7 @@
         </is>
       </c>
       <c r="AA92" t="inlineStr"/>
+      <c r="AB92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -10354,7 +10428,7 @@
       </c>
       <c r="T93" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U93" t="inlineStr">
@@ -10364,26 +10438,27 @@
       </c>
       <c r="V93" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W93" t="inlineStr">
         <is>
-          <t>Antecedente de fraude previo combinado con pérdida de señal GPS crea ambigüedad crítica para la validación automática.</t>
+          <t>Usuario con flag de fraude previo y GPS sin señal que impide validar entrega. Reclamo subjetivo sin evidencia corroborante.</t>
         </is>
       </c>
       <c r="X93" t="inlineStr"/>
       <c r="Y93" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | evidencia_gps_parcial | reclamo_subjetivo</t>
+          <t>flag_fraude_previo | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z93" t="inlineStr"/>
       <c r="AA93" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por evidencia GPS parcial y riesgo histórico requieren revisión manual. | Reclamo por no entrega con GPS perdido y flag histórico de fraude que impide confirmación objetiva.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: flag de fraude previo combinado con GPS perdido y falta de evidencia objetiva para validar la no entrega. | Reclamo por no llegada de pedido en cuenta con historial de fraude y sin rastreo GPS válido.</t>
+        </is>
+      </c>
+      <c r="AB93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -10486,6 +10561,7 @@
         </is>
       </c>
       <c r="AA94" t="inlineStr"/>
+      <c r="AB94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -10580,7 +10656,7 @@
       </c>
       <c r="W95" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 2 años, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado está dentro de parámetros normales y la queja por calidad de alimento es coherente con el perfil.</t>
+          <t>Usuario con antigüedad superior a 2 años, sin flags de fraude, baja frecuencia de reclamos y monto solicitado dentro de parámetros normales. La descripción es coherente con un problema operativo o de calidad.</t>
         </is>
       </c>
       <c r="X95" t="inlineStr"/>
@@ -10592,9 +10668,10 @@
       <c r="Z95" t="inlineStr"/>
       <c r="AA95" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario con historial limpio y métricas dentro de lo esperado. | Reclamo por deterioro de alimento en cuenta confiable sin inconsistencias operativas ni señales de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por calidad de producto en cuenta antigua y sin historial negativo.</t>
+        </is>
+      </c>
+      <c r="AB95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -10701,6 +10778,7 @@
         </is>
       </c>
       <c r="AA96" t="inlineStr"/>
+      <c r="AB96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -10795,7 +10873,7 @@
       </c>
       <c r="W97" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, 0 flags de fraude y baja frecuencia de reclamos. El faltante de productos es un error operativo común sin señales de abuso.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y frecuencia de reclamos baja. El reporte de faltante es un error operativo común y coherente.</t>
         </is>
       </c>
       <c r="X97" t="inlineStr"/>
@@ -10807,9 +10885,10 @@
       <c r="Z97" t="inlineStr"/>
       <c r="AA97" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por faltante de ítems en cuenta antigua y sin historial negativo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo sin señales de fraude o inconsistencias operativas. | Reclamo por faltante de producto en cuenta antigua y confiable, sin indicadores de riesgo ni inconsistencias.</t>
+        </is>
+      </c>
+      <c r="AB97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -10904,21 +10983,22 @@
       </c>
       <c r="W98" t="inlineStr">
         <is>
-          <t>Cuenta nueva (80d) con 3 reclamos en 90d y 1 flag de fraude previo. Sin evidencia GPS que valide el caso.</t>
+          <t>Cuenta nueva (80d) con flag de fraude previo y 3 reclamos en 90d. Ausencia de evidencia GPS que valide el error operativo. Patrón consistente con riesgo de abuso.</t>
         </is>
       </c>
       <c r="X98" t="inlineStr"/>
       <c r="Y98" t="inlineStr">
         <is>
-          <t>account_abuse | flag_fraude_previo | entrega_gps_no_confirmada</t>
+          <t>antiguedad_moderada_con_alta_reincidencia | flag_fraude_previo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z98" t="inlineStr"/>
       <c r="AA98" t="inlineStr">
         <is>
-          <t>RECHAZAR: cuenta nueva con alta frecuencia de reclamos y flag de fraude previo, sin evidencia GPS que respalde la inconsistencia. | Reclamo por error de producto en perfil de alto riesgo sin validación geoespacial.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: cuenta nueva con flag de fraude previo y alta frecuencia de reclamos sin evidencia GPS que respalde el caso. | Reclamo por producto equivocado en cuenta reciente con historial negativo y sin validación geolocalizada.</t>
+        </is>
+      </c>
+      <c r="AB98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -11013,7 +11093,7 @@
       </c>
       <c r="W99" t="inlineStr">
         <is>
-          <t>Evidencia GPS parcial y ratio de compensación alto generan ambigüedad para validar cancelación real sin revisión humana.</t>
+          <t>Cuenta con antigüedad moderada y sin flags de fraude, pero presenta GPS parcial que impide validar la cancelación del restaurante, sumado a un ratio de compensación elevado y frecuencia de reclamos notable en 90 días.</t>
         </is>
       </c>
       <c r="X99" t="inlineStr"/>
@@ -11025,9 +11105,10 @@
       <c r="Z99" t="inlineStr"/>
       <c r="AA99" t="inlineStr">
         <is>
-          <t>ESCALAR: inconsistencia en evidencia GPS y ratio de compensación elevado requieren validación manual. | Reclamo por cargo tras cancelación del restaurante con GPS incompleto y historial de compensaciones frecuente.</t>
-        </is>
-      </c>
+          <t>ESCALAR: evidencia GPS parcial y métricas elevadas (ratio y frecuencia) impiden decisión automatizada segura. | Reclamo por cargo no reflejado tras supuesta cancelación del restaurante. Evidencia GPS ambigua y métricas de riesgo moderado requieren validación manual.</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -11130,6 +11211,7 @@
         </is>
       </c>
       <c r="AA100" t="inlineStr"/>
+      <c r="AB100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -11232,6 +11314,7 @@
         </is>
       </c>
       <c r="AA101" t="inlineStr"/>
+      <c r="AB101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -11326,21 +11409,22 @@
       </c>
       <c r="W102" t="inlineStr">
         <is>
-          <t>Reclamo subjetivo difícil de verificar objetivamente. La combinación de un flag de fraude previo, evidencia GPS parcial y la naturaleza sensorial del reporte genera ambigüedad que excede la automatización.</t>
+          <t>Reclamo subjetivo sobre estado del producto con evidencia GPS parcial y un flag de fraude previo. La ambigüedad en la verificación objetiva y el historial mixto requieren revisión humana.</t>
         </is>
       </c>
       <c r="X102" t="inlineStr"/>
       <c r="Y102" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo | flag_fraude_previo | evidencia_gps_parcial</t>
+          <t>evidencia_gps_parcial | reclamo_subjetivo | flag_fraude_previo</t>
         </is>
       </c>
       <c r="Z102" t="inlineStr"/>
       <c r="AA102" t="inlineStr">
         <is>
-          <t>ESCALAR: ambigüedad por naturaleza subjetiva del reclamo, flag de fraude previo y GPS parcial requieren validación manual. | Solicitud por olor a comida descompuesta en cuenta con antigüedad moderada, historial con flag de fraude y geolocalización incompleta.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ambigüedad por GPS parcial, naturaleza subjetiva del reclamo y flag de fraude previo requieren validación manual. | Caso con reclamo subjetivo, GPS parcial y antecedente de fraude que impide decisión automatizada segura.</t>
+        </is>
+      </c>
+      <c r="AB102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -11435,21 +11519,18 @@
       </c>
       <c r="W103" t="inlineStr">
         <is>
-          <t>Perfil de usuario limpio con 821 días de antigüedad y sin historial de fraude. Reclamo por cancelación operativa sin señales de abuso o inconsistencia crítica.</t>
+          <t>Usuario con antigüedad superior a 2 años, historial limpio y sin reclamos recientes. La justificación por cancelación operativa es coherente y el monto solicitado se ajusta al promedio.</t>
         </is>
       </c>
       <c r="X103" t="inlineStr"/>
-      <c r="Y103" t="inlineStr">
-        <is>
-          <t>entrega_gps_no_confirmada</t>
-        </is>
-      </c>
+      <c r="Y103" t="inlineStr"/>
       <c r="Z103" t="inlineStr"/>
       <c r="AA103" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo consistente con perfil de usuario sano y sin indicadores de fraude. | Solicitud de reembolso por cancelación de pedido sin repartidor en cuenta confiable sin actividad sospechosa reciente.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo legítimo por cancelación de servicio sin señales de fraude o inconsistencias operativas.</t>
+        </is>
+      </c>
+      <c r="AB103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -11544,21 +11625,22 @@
       </c>
       <c r="W104" t="inlineStr">
         <is>
-          <t>Usuario con 541 días de antigüedad y 0 flags de fraude. El motivo de cancelación por falta de repartidor es operativamente coherente y el monto solicitado es razonable. No se detectan patrones de abuso ni inconsistencias críticas.</t>
+          <t>Usuario con 541 días de antigüedad, 0 flags y 0 reclamos recientes. La solicitud de reembolso por cancelación operativa es coherente y el monto solicitado está dentro del rango normal. Al no existir contradicciones GPS ni indicadores de abuso, se considera legítimo.</t>
         </is>
       </c>
       <c r="X104" t="inlineStr"/>
       <c r="Y104" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z104" t="inlineStr"/>
       <c r="AA104" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin señales de fraude, consistente con el contexto operativo y perfil de usuario confiable. | Solicitud de reembolso por cancelación operativa en cuenta antigua sin historial de reclamos.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de fraude. | Reembolso por cancelación de pedido sin repartidor en cuenta sana sin historial de fraude.</t>
+        </is>
+      </c>
+      <c r="AB104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -11653,7 +11735,7 @@
       </c>
       <c r="W105" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. El motivo es operativo y coherente con la solicitud de reembolso.</t>
+          <t>Usuario con casi 4 años de antigüedad y historial limpio. Reclamo operativo coherente (cobro pendiente tras cancelación del restaurante) sin inconsistencias ni señales de fraude.</t>
         </is>
       </c>
       <c r="X105" t="inlineStr"/>
@@ -11665,9 +11747,10 @@
       <c r="Z105" t="inlineStr"/>
       <c r="AA105" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con evidencia operativa y perfil de usuario confiable. | Reembolso por cancelación de pedido en cuenta antigua y sin historial de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo y consistente con usuario de alta antigüedad y sin historial de riesgo. | Error de facturación post-cancelación validado en cuenta consolidada y sin riesgos previos.</t>
+        </is>
+      </c>
+      <c r="AB105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -11772,6 +11855,7 @@
         </is>
       </c>
       <c r="AA106" t="inlineStr"/>
+      <c r="AB106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -11874,6 +11958,7 @@
         </is>
       </c>
       <c r="AA107" t="inlineStr"/>
+      <c r="AB107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -11976,6 +12061,7 @@
         </is>
       </c>
       <c r="AA108" t="inlineStr"/>
+      <c r="AB108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -12055,7 +12141,7 @@
       </c>
       <c r="T109" t="inlineStr">
         <is>
-          <t>APROBAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U109" t="inlineStr">
@@ -12065,26 +12151,27 @@
       </c>
       <c r="V109" t="inlineStr">
         <is>
-          <t>APROBAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W109" t="inlineStr">
         <is>
-          <t>Reclamo de cobro duplicado sin señales de fraude. Usuario con antigüedad moderada y sin historial negativo. La falta de GPS no afecta la verificación financiera del cargo.</t>
+          <t>Usuario sin historial de fraude y antigüedad moderada. El reclamo por doble cobro no muestra patrones de abuso, pero la pérdida de señal GPS impide validar la trazabilidad operativa requerida.</t>
         </is>
       </c>
       <c r="X109" t="inlineStr"/>
       <c r="Y109" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z109" t="inlineStr"/>
       <c r="AA109" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo verificable en pasarela de pago sin indicadores de fraude. | Solicitud de reembolso por doble cargo en cuenta sin patrones abusivos ni contradicciones operativas.</t>
-        </is>
-      </c>
+          <t>ESCALAR: falta evidencia GPS consistente y el tipo de reclamo requiere validación financiera manual antes de aprobar. | Solicitud de reembolso por duplicado en facturación. Sin evidencia GPS ni palabras críticas, pero requiere validación cruzada con pasarela de pagos.</t>
+        </is>
+      </c>
+      <c r="AB109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -12179,7 +12266,7 @@
       </c>
       <c r="W110" t="inlineStr">
         <is>
-          <t>Evidencia GPS ausente combinada con un flag de fraude previo y frecuencia moderada de reclamos genera ambigüedad que impide la aprobación automatizada.</t>
+          <t>Pérdida de señal GPS impide validar entrega. Cuenta con 1 flag de fraude previo y reclamo subjetivo de producto incorrecto sin evidencia corroborante.</t>
         </is>
       </c>
       <c r="X110" t="inlineStr"/>
@@ -12191,9 +12278,10 @@
       <c r="Z110" t="inlineStr"/>
       <c r="AA110" t="inlineStr">
         <is>
-          <t>ESCALAR: falta de evidencia GPS y flag de fraude previo requieren verificación humana para descartar abuso o error operativo. | Reclamo por producto incorrecto sin validación GPS en cuenta con historial de riesgo moderado.</t>
-        </is>
-      </c>
+          <t>ESCALAR: datos insuficientes por GPS perdido y flag previo requieren validación humana del error de preparación. | Reclamo por error de producto en cuenta con historial mixto y sin evidencia geolocalizable.</t>
+        </is>
+      </c>
+      <c r="AB110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -12288,7 +12376,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>El reclamo contiene el término crítico 'alergia', lo que activa automáticamente el protocolo de revisión humana por riesgos de salud y legales. Se complementa con alta frecuencia de reclamos y ausencia de evidencia GPS.</t>
+          <t>El reclamo menciona explícitamente 'alergia', palabra crítica que activa automáticamente el protocolo de seguridad de marca y riesgo legal/sanitario. Esta señal se refuerza con alta frecuencia de reclamos (6 en 90d), señal GPS perdida que impide verificación operativa y un flag de fraude previo, haciendo inviable la aprobación automatizada.</t>
         </is>
       </c>
       <c r="X111" t="inlineStr">
@@ -12299,7 +12387,7 @@
       </c>
       <c r="Y111" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
+          <t>palabras_criticas_seguridad | alta_frecuencia_reclamos | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z111" t="inlineStr">
@@ -12309,9 +12397,10 @@
       </c>
       <c r="AA111" t="inlineStr">
         <is>
-          <t>ESCALAR: presencia de palabra crítica 'alergia' que requiere evaluación de riesgo legal/salud, corroborada por alta frecuencia de reclamos y falta de validación GPS. | Reclamo por alergia alimentaria en cuenta de 95 días con 6 incidentes en 90d y GPS sin señal.</t>
-        </is>
-      </c>
+          <t>ESCALAR: contiene palabras críticas de salud/legal (alergia) que requieren revisión humana conforme a reglas de seguridad de marca. | Reclamo por alergia alimentaria con evidencia GPS inconsistente y historial de alta frecuencia en cuenta moderadamente antigua.</t>
+        </is>
+      </c>
+      <c r="AB111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -12414,6 +12503,7 @@
         </is>
       </c>
       <c r="AA112" t="inlineStr"/>
+      <c r="AB112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -12516,6 +12606,7 @@
         </is>
       </c>
       <c r="AA113" t="inlineStr"/>
+      <c r="AB113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -12620,6 +12711,7 @@
         </is>
       </c>
       <c r="AA114" t="inlineStr"/>
+      <c r="AB114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -12726,6 +12818,7 @@
         </is>
       </c>
       <c r="AA115" t="inlineStr"/>
+      <c r="AB115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -12828,6 +12921,7 @@
         </is>
       </c>
       <c r="AA116" t="inlineStr"/>
+      <c r="AB116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -12922,7 +13016,7 @@
       </c>
       <c r="W117" t="inlineStr">
         <is>
-          <t>El reclamo contiene la palabra crítica 'alergia', lo que obliga a escalación por protocolo de seguridad y salud. Adicionalmente, la cuenta es extremadamente nueva (10d) con alta densidad de reclamos (14 en 90d) y dos flags de fraude previos, lo que confirma un perfil de alto riesgo que no puede resolverse automáticamente.</t>
+          <t>El reclamo menciona 'alergia', palabra crítica de seguridad que activa protocolo de escalación obligatoria. Adicionalmente, la cuenta tiene solo 10 días de antigüedad con 14 reclamos en 90 días y 2 flags de fraude previos, lo que indica un perfil de alto riesgo.</t>
         </is>
       </c>
       <c r="X117" t="inlineStr">
@@ -12943,9 +13037,10 @@
       </c>
       <c r="AA117" t="inlineStr">
         <is>
-          <t>ESCALAR: palabra crítica de seguridad presente ('alergia') combinada con cuenta nueva abusiva y historial de fraude previo, requiriendo evaluación humana especializada. | Reclamo por alergia en cuenta nueva con 14 intentos en 90d, 2 flags de fraude y score de riesgo alto. Requiere revisión humana por implicaciones de salud y fuerte evidencia de abuso.</t>
-        </is>
-      </c>
+          <t>ESCALAR: contiene palabras críticas de seguridad (alergia) que implican riesgo legal y de salud, sumado a señales claras de abuso de cuenta y fraude previo. | Reclamo por alergia alimentaria en cuenta nueva con historial de fraude y alta frecuencia de solicitudes. Riesgo legal/saludable requiere revisión humana inmediata.</t>
+        </is>
+      </c>
+      <c r="AB117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -13040,21 +13135,22 @@
       </c>
       <c r="W118" t="inlineStr">
         <is>
-          <t>Usuario con 311 días de antigüedad pero 6 reclamos en 90 días. La ausencia de evidencia GPS genera ambigüedad para validar el retraso reportado.</t>
+          <t>Alta frecuencia de reclamos (6 en 90d) y ratio de compensación elevado (0.84) sin evidencia GPS que valide el retraso o estado del pedido.</t>
         </is>
       </c>
       <c r="X118" t="inlineStr"/>
       <c r="Y118" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | entrega_gps_no_confirmada</t>
+          <t>alta_frecuencia_reclamos | compensacion_elevada | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z118" t="inlineStr"/>
       <c r="AA118" t="inlineStr">
         <is>
-          <t>ESCALAR: alta frecuencia de reclamos combinada con falta de evidencia GPS para verificación objetiva requiere revisión humana. | Reclamo por retraso y calidad sin validación geolocal en cuenta con alta frecuencia de solicitudes.</t>
-        </is>
-      </c>
+          <t>ESCALAR: combinación de alta frecuencia, ratio de compensación elevado y falta de evidencia GPS requiere revisión humana para validar el retraso real. | Reclamo por retraso y calidad de comida en cuenta con historial de alta frecuencia y GPS no confirmado.</t>
+        </is>
+      </c>
+      <c r="AB118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -13149,7 +13245,7 @@
       </c>
       <c r="W119" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El tipo de incidencia (doble cobro) es verificable objetivamente vía pasarela de pagos y no presenta indicadores de abuso.</t>
+          <t>Usuario con más de 3 años de antigüedad, historial limpio y baja frecuencia de reclamos. El caso describe un error de cobro duplicado común sin señales de abuso.</t>
         </is>
       </c>
       <c r="X119" t="inlineStr"/>
@@ -13161,9 +13257,10 @@
       <c r="Z119" t="inlineStr"/>
       <c r="AA119" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con un usuario de bajo riesgo y sin señales de fraude. | Error operativo de pago en cuenta antigua y sin historial negativo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo operativo legítimo sin indicadores de riesgo o inconsistencias. | Reclamo por cobro duplicado en cuenta antigua y sin antecedentes de fraude.</t>
+        </is>
+      </c>
+      <c r="AB119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -13258,21 +13355,22 @@
       </c>
       <c r="W120" t="inlineStr">
         <is>
-          <t>Usuario con 506 días de antigüedad, sin flags de fraude y frecuencia baja. La cancelación por falta de repartidor es un evento operativo coherente y el monto solicitado es razonable.</t>
+          <t>Usuario con 506 días de antigüedad, sin flags de fraude y baja frecuencia de reclamos. La justificación por cancelación operativa es coherente y no presenta inconsistencias con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X120" t="inlineStr"/>
       <c r="Y120" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z120" t="inlineStr"/>
       <c r="AA120" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo legítimo por cancelación operativa en cuenta estable sin indicadores de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo sin señales de fraude o abuso. | Cancelación por falta de repartidor en cuenta estable y confiable.</t>
+        </is>
+      </c>
+      <c r="AB120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -13367,21 +13465,22 @@
       </c>
       <c r="W121" t="inlineStr">
         <is>
-          <t>Usuario antiguo (731d) sin flags de fraude y baja frecuencia de reclamos. El reporte de faltantes es un error operativo frecuente y coherente.</t>
+          <t>Usuario con 2+ años de antigüedad, 0 flags y baja frecuencia de reclamos. El reclamo por artículos faltantes es coherente y no presenta señales de fraude.</t>
         </is>
       </c>
       <c r="X121" t="inlineStr"/>
       <c r="Y121" t="inlineStr">
         <is>
-          <t>descripcion_incoherente</t>
+          <t>reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z121" t="inlineStr"/>
       <c r="AA121" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con el perfil de usuario confiable y sin señales de fraude. | Reclamo por faltantes en cuenta estable y limpia, sin inconsistencias operativas ni patrones de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de abuso. | Reclamo estándar por artículos faltantes en cuenta antigua y sin historial de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -13461,7 +13560,7 @@
       </c>
       <c r="T122" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="U122" t="inlineStr">
@@ -13471,12 +13570,12 @@
       </c>
       <c r="V122" t="inlineStr">
         <is>
-          <t>ESCALAR</t>
+          <t>RECHAZAR</t>
         </is>
       </c>
       <c r="W122" t="inlineStr">
         <is>
-          <t>Antigüedad moderada (198d) con 5 reclamos en 90 días. La falta de confirmación GPS coincide con la cancelación reportada, pero la alta frecuencia sin evidencia objetiva requiere validación manual.</t>
+          <t>Usuario con 198 días de antigüedad pero 5 reclamos en 90 días. La ausencia de evidencia GPS impide verificar la cancelación reportada, lo cual combinado con la alta frecuencia sugiere posible abuso o error sistémico.</t>
         </is>
       </c>
       <c r="X122" t="inlineStr"/>
@@ -13488,9 +13587,10 @@
       <c r="Z122" t="inlineStr"/>
       <c r="AA122" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de alta frecuencia de reclamos y ausencia de evidencia GPS requiere revisión humana de logs operativos. | Reclamo por cancelación operativa en cuenta con alta densidad de solicitudes recientes y sin evidencia GPS de entrega.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: alta frecuencia de reclamos sin evidencia GPS que respalde la cancelación reportada. | Reclamo por cancelación sin soporte GPS en cuenta con alta densidad de solicitudes recientes.</t>
+        </is>
+      </c>
+      <c r="AB122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -13585,7 +13685,7 @@
       </c>
       <c r="W123" t="inlineStr">
         <is>
-          <t>Usuario con casi 5 años de antigüedad, 0 flags y baja frecuencia de reclamos. Ausencia total de indicadores de fraude o inconsistencia.</t>
+          <t>Usuario con 1775 días de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El monto solicitado y ratio están dentro de parámetros normales. No se detectan inconsistencias ni términos de riesgo.</t>
         </is>
       </c>
       <c r="X123" t="inlineStr"/>
@@ -13597,9 +13697,10 @@
       <c r="Z123" t="inlineStr"/>
       <c r="AA123" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo respaldado por historial de usuario estable y ausencia de patrones abusivos. | Reclamo por calidad de alimento en cuenta altamente confiable sin señales de riesgo operativo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo con perfil de usuario sano y ausencia de indicadores de riesgo. | Reclamo por calidad de producto en cuenta confiable sin señales de abuso o fraude.</t>
+        </is>
+      </c>
+      <c r="AB123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -13694,21 +13795,22 @@
       </c>
       <c r="W124" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad, 0 flags de fraude y baja frecuencia de reclamos. El reporte de producto equivocado es un error operativo común. La pérdida de señal GPS no contradice el reclamo y el perfil conservador indica legitimidad.</t>
+          <t>Usuario con antigüedad superior a 4 años, 0 flags de fraude y frecuencia baja de reclamos. El monto solicitado y ratio son normales.</t>
         </is>
       </c>
       <c r="X124" t="inlineStr"/>
       <c r="Y124" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z124" t="inlineStr"/>
       <c r="AA124" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario de larga trayectoria y sin historial negativo. | Error operativo de restaurante en cuenta antigua y confiable sin indicadores de fraude.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo por producto equivocado en cuenta verificada sin señales de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -13803,21 +13905,22 @@
       </c>
       <c r="W125" t="inlineStr">
         <is>
-          <t>Cuenta con flag de fraude previo y 6 reclamos en 90 días. La evidencia GPS indica señal perdida, lo que genera inconsistencia con la afirmación de entrega de la app y el reclamo del usuario. Ratio de compensación elevado refuerza el riesgo.</t>
+          <t>Historial con flag de fraude y 6 reclamos en 90 días. Evidencia GPS nula para validar entrega, lo que invalida la coherencia del reclamo.</t>
         </is>
       </c>
       <c r="X125" t="inlineStr"/>
       <c r="Y125" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada | compensacion_elevada</t>
+          <t>alta_frecuencia_reclamos | flag_fraude_previo | entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z125" t="inlineStr"/>
       <c r="AA125" t="inlineStr">
         <is>
-          <t>RECHAZAR: evidencia clara de posible abuso combinando flag de fraude, alta frecuencia y falta de validación geoespacial. | Inconsistencia entre estado de entrega y evidencia GPS en cuenta con historial negativo y alta frecuencia de reclamos.</t>
-        </is>
-      </c>
+          <t>RECHAZAR: alta frecuencia de reclamos, flag de fraude previo y falta de evidencia GPS que respalde la no recepción. | Inconsistencia entre estado de app, GPS perdido y reclamo de no recepción en cuenta con historial sospechoso.</t>
+        </is>
+      </c>
+      <c r="AB125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -13920,6 +14023,7 @@
         </is>
       </c>
       <c r="AA126" t="inlineStr"/>
+      <c r="AB126" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -14026,6 +14130,7 @@
         </is>
       </c>
       <c r="AA127" t="inlineStr"/>
+      <c r="AB127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -14130,6 +14235,7 @@
         </is>
       </c>
       <c r="AA128" t="inlineStr"/>
+      <c r="AB128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -14224,7 +14330,7 @@
       </c>
       <c r="W129" t="inlineStr">
         <is>
-          <t>Perfil de usuario sano con 353 días de antigüedad y cero reclamos recientes. La narrativa es coherente y no contiene palabras críticas. La pérdida de señal GPS no constituye evidencia de fraude.</t>
+          <t>Usuario con antigüedad superior a un año y cero flags de fraude. El reclamo es coherente y la pérdida de señal GPS es un fallo técnico común, no indica abuso.</t>
         </is>
       </c>
       <c r="X129" t="inlineStr"/>
@@ -14236,9 +14342,10 @@
       <c r="Z129" t="inlineStr"/>
       <c r="AA129" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo sin indicadores de fraude, perfil conservador y narrativa coherente. | Reclamo por marcaje de entrega sin confirmación de timbre. Usuario sin historial de riesgo ni inconsistencias operativas.</t>
-        </is>
-      </c>
+          <t>APROBAR: perfil de usuario conservador sin señales de fraude, la inconsistencia se debe a falla técnica de rastreo. | Reclamo legítimo por entrega no recibida en cuenta limpia con señal GPS perdida.</t>
+        </is>
+      </c>
+      <c r="AB129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -14333,21 +14440,22 @@
       </c>
       <c r="W130" t="inlineStr">
         <is>
-          <t>Usuario con 558 días de antigüedad y 0 flags de fraude. Reclamo de ítem incorrecto coherente, monto razonable y sin patrones de abuso.</t>
+          <t>Usuario con 558 días de antigüedad, 0 flags y 0 reclamos recientes. La descripción del error (producto incorrecto) es coherente y no presenta contradicciones con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X130" t="inlineStr"/>
       <c r="Y130" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z130" t="inlineStr"/>
       <c r="AA130" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Error operativo en entrega de bebida en cuenta verificada sin historial de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Reclamo por producto equivocado en cuenta estable sin historial de fraude.</t>
+        </is>
+      </c>
+      <c r="AB130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -14442,21 +14550,22 @@
       </c>
       <c r="W131" t="inlineStr">
         <is>
-          <t>Usuario con 576 días de antigüedad, 0 flags y 0 reclamos recientes. La discrepancia de cobro es un error operativo común y no presenta indicadores de fraude.</t>
+          <t>Usuario con 576 días de antigüedad, cero reclamos recientes y sin flags de fraude. La solicitud es una discrepancia de cobro operativa, coherente y sin señales de abuso.</t>
         </is>
       </c>
       <c r="X131" t="inlineStr"/>
       <c r="Y131" t="inlineStr">
         <is>
-          <t>reclamo_subjetivo</t>
+          <t>descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z131" t="inlineStr"/>
       <c r="AA131" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario sin historial de riesgo ni inconsistencias. | Reclamo por diferencia de monto en resumen de pago en cuenta limpia.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo de discrepancia de cobro en usuario con historial limpio y sin señales de riesgo. | Reclamo de discrepancia tarifaria en cuenta limpia y antigua, sin indicadores de fraude.</t>
+        </is>
+      </c>
+      <c r="AB131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -14551,7 +14660,7 @@
       </c>
       <c r="W132" t="inlineStr">
         <is>
-          <t>Reclamo por cobro tras cancelación con evidencia GPS parcial y alta frecuencia de reclamos (5 en 90d) junto a un ratio de compensación elevado (0.86). Requiere revisión para validar si es error de facturación o patrón recurrente.</t>
+          <t>Reclamo por cobro tras cancelación. Sin flags de fraude, pero la evidencia GPS parcial combinada con alta frecuencia de reclamos (5 en 90d) y ratio de compensación elevado genera ambigüedad operativa que impide una decisión automatizada segura.</t>
         </is>
       </c>
       <c r="X132" t="inlineStr"/>
@@ -14563,9 +14672,10 @@
       <c r="Z132" t="inlineStr"/>
       <c r="AA132" t="inlineStr">
         <is>
-          <t>ESCALAR: evidencia GPS parcial combinada con alta frecuencia de reclamos y ratio de compensación elevado requiere validación manual para descartar abuso o confirmar error de sistema. | Disputa de cobro por cancelación con GPS ambigua y historial de alta frecuencia/recompensa.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ambigüedad por evidencia GPS parcial y alta frecuencia de reclamos con ratio de compensación elevado, requiere validación manual. | Solicitud de reembolso por cancelación con GPS parcial, alta frecuencia reciente y ratio de compensación alto.</t>
+        </is>
+      </c>
+      <c r="AB132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -14660,7 +14770,7 @@
       </c>
       <c r="W133" t="inlineStr">
         <is>
-          <t>Usuario con 1260 días de antigüedad y 0 flags de fraude. El reclamo por calidad es coherente y no activa reglas de riesgo ni palabras críticas.</t>
+          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude y baja frecuencia de reclamos. La descripción del deterioro es coherente y no presenta contradicciones técnicas ni palabras críticas.</t>
         </is>
       </c>
       <c r="X133" t="inlineStr"/>
@@ -14672,9 +14782,10 @@
       <c r="Z133" t="inlineStr"/>
       <c r="AA133" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo basado en perfil de usuario estable y ausencia de señales de fraude. | Queja por estado del producto en cuenta confiable sin indicadores de abuso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo basado en perfil de usuario conservador y ausencia de inconsistencias. | Reclamo por calidad de producto en cuenta confiable sin señales de riesgo operativo o fraude.</t>
+        </is>
+      </c>
+      <c r="AB133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -14769,7 +14880,7 @@
       </c>
       <c r="W134" t="inlineStr">
         <is>
-          <t>El reclamo menciona explícitamente 'alergia', lo que activa el protocolo de palabras críticas de seguridad de marca y riesgo legal/salud, requiriendo revisión humana inmediata.</t>
+          <t>El reclamo menciona explícitamente 'alergia', lo cual activa automáticamente las reglas de seguridad de marca y salud. Aunque el perfil del usuario es sano y sin historial de fraude, la naturaleza del reclamo requiere validación médica/legal.</t>
         </is>
       </c>
       <c r="X134" t="inlineStr">
@@ -14790,9 +14901,10 @@
       </c>
       <c r="AA134" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene término crítico de salud ('alergia') que requiere validación médica/legal y gestión de riesgo de marca. | Reclamo por alergia alimentaria en cuenta antigua sin historial de fraude, pero con señal crítica de salud que impide aprobación automatizada.</t>
-        </is>
-      </c>
+          <t>ESCALAR: presencia de palabra crítica ('alergia') que genera riesgo de salud y potencial responsabilidad legal, requiriendo revisión humana obligatoria. | Reclamo por posible error de preparación con implicaciones de salud (alergia). Activa protocolo de escalamiento por palabras críticas.</t>
+        </is>
+      </c>
+      <c r="AB134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -14887,21 +14999,22 @@
       </c>
       <c r="W135" t="inlineStr">
         <is>
-          <t>Usuario con 790 días de antigüedad y 0 flags de fraude. El reclamo por faltante es un incidente operativo común y coherente, sin activar reglas de riesgo automático.</t>
+          <t>Usuario con 790 días de antigüedad y sin historial de fraude. El reporte de faltante es un error operativo común y coherente. No se activan reglas de riesgo ni términos críticos.</t>
         </is>
       </c>
       <c r="X135" t="inlineStr"/>
       <c r="Y135" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada</t>
         </is>
       </c>
       <c r="Z135" t="inlineStr"/>
       <c r="AA135" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin indicadores de fraude. | Reclamo estándar por faltante de producto en cuenta antigua y limpia, sin evidencia GPS contradictoria ni palabras críticas.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario antiguo y sin señales de fraude. | Faltante de producto validado por perfil de usuario confiable y sin inconsistencias.</t>
+        </is>
+      </c>
+      <c r="AB135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -14996,7 +15109,7 @@
       </c>
       <c r="W136" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad y salud, requiriendo revisión humana obligatoria. Adicionalmente, la cuenta presenta alta frecuencia de reclamos en 90 días, antigüedad muy reciente y 2 flags de fraude previos, lo que incrementa el riesgo.</t>
+          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad de marca y riesgo legal/salud. Se refuerza con historial de fraude previo y cuenta nueva con alta frecuencia de reclamos.</t>
         </is>
       </c>
       <c r="X136" t="inlineStr">
@@ -15007,7 +15120,7 @@
       </c>
       <c r="Y136" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | account_abuse | flag_fraude_previo</t>
+          <t>palabras_criticas_seguridad | flag_fraude_previo | account_abuse</t>
         </is>
       </c>
       <c r="Z136" t="inlineStr">
@@ -15017,9 +15130,10 @@
       </c>
       <c r="AA136" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabras críticas de seguridad (alergia) que requieren validación humana, sumado a señales de abuso de cuenta y fraude previo. | Reclamo por alergia alimentaria en cuenta nueva con alta frecuencia de incidencias y antecedentes de fraude. La mención de riesgo de salud obliga a escalación manual.</t>
-        </is>
-      </c>
+          <t>ESCALAR: contiene palabras críticas de seguridad de marca ('alergia') que implican riesgo legal/salud, sumado a señales de fraude previo y abuso de cuenta. | Reclamo por alergia en cuenta nueva con 2 flags de fraude y 12 reclamos en 90 días. Requiere revisión humana por términos de salud/legal.</t>
+        </is>
+      </c>
+      <c r="AB136" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -15126,6 +15240,7 @@
         </is>
       </c>
       <c r="AA137" t="inlineStr"/>
+      <c r="AB137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -15220,21 +15335,18 @@
       </c>
       <c r="W138" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, historial limpio y 0 reclamos recientes. El reclamo por ítem faltante es operativo y coherente, sin señales de fraude.</t>
+          <t>Perfil de usuario muy antiguo y limpio sin historial de reclamos ni flags. Reclamo por ítem faltante es operativo y coherente con la evidencia disponible.</t>
         </is>
       </c>
       <c r="X138" t="inlineStr"/>
-      <c r="Y138" t="inlineStr">
-        <is>
-          <t>entrega_gps_no_confirmada</t>
-        </is>
-      </c>
+      <c r="Y138" t="inlineStr"/>
       <c r="Z138" t="inlineStr"/>
       <c r="AA138" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo de usuario confiable sin historial de fraude ni patrones abusivos. | Reclamo estándar por producto faltante en cuenta antigua y sana, sin inconsistencias ni riesgos detectados.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sin riesgos. | Reclamo estándar por producto faltante en cuenta confiable sin señales de fraude.</t>
+        </is>
+      </c>
+      <c r="AB138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -15337,6 +15449,7 @@
         </is>
       </c>
       <c r="AA139" t="inlineStr"/>
+      <c r="AB139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -15431,21 +15544,22 @@
       </c>
       <c r="W140" t="inlineStr">
         <is>
-          <t>Reclamo por retraso y calidad con 5 incidencias en 90 días y sin rastreo GPS disponible. La ambigüedad en la evidencia y la densidad de reclamos requieren validación manual.</t>
+          <t>Alta frecuencia de reclamos (5 en 90d) combinada con señal GPS perdida genera ambigüedad para validar el retraso real y la condición del pedido.</t>
         </is>
       </c>
       <c r="X140" t="inlineStr"/>
       <c r="Y140" t="inlineStr">
         <is>
-          <t>alta_frecuencia_reclamos | evidencia_gps_parcial</t>
+          <t>alta_frecuencia_reclamos | entrega_gps_no_confirmada | reclamo_subjetivo</t>
         </is>
       </c>
       <c r="Z140" t="inlineStr"/>
       <c r="AA140" t="inlineStr">
         <is>
-          <t>ESCALAR: combinación de señal GPS perdida y alta frecuencia de reclamos requiere revisión humana para validar el retraso reportado. | Posible falla operativa por retraso, pero la falta de GPS y alta frecuencia de reclamos impiden la decisión automatizada.</t>
-        </is>
-      </c>
+          <t>ESCALAR: datos insuficientes por pérdida de GPS y patrón de frecuencia elevada requieren validación humana del incidente operativo. | Reclamo por retraso y calidad de comida sin evidencia GPS que confirme o refute los tiempos de entrega, en cuenta con historial de múltiples solicitudes recientes.</t>
+        </is>
+      </c>
+      <c r="AB140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -15540,21 +15654,22 @@
       </c>
       <c r="W141" t="inlineStr">
         <is>
-          <t>Contradicción entre estado de la app y reporte del usuario sin respaldo GPS. Perfil antiguo sin flags de fraude, pero la falta de evidencia objetiva impide decisión automatizada.</t>
+          <t>Usuario con antigüedad sólida (911d) y 0 flags de fraude, pero el reclamo contradice el estatus de la app y la evidencia GPS no está confirmada. El ratio de compensación histórico es elevado (0.955), generando ambigüedad que requiere validación humana.</t>
         </is>
       </c>
       <c r="X141" t="inlineStr"/>
       <c r="Y141" t="inlineStr">
         <is>
-          <t>entrega_gps_no_confirmada | reclamo_subjetivo</t>
+          <t>entrega_gps_no_confirmada | compensacion_elevada | descripcion_incoherente</t>
         </is>
       </c>
       <c r="Z141" t="inlineStr"/>
       <c r="AA141" t="inlineStr">
         <is>
-          <t>ESCALAR: ausencia de evidencia GPS y datos insuficientes para verificar objetivamente el reclamo. | Reclamo por no recepción con GPS no confirmado y perfil conservador, requiere validación manual.</t>
-        </is>
-      </c>
+          <t>ESCALAR: ambigüedad por falta de evidencia GPS y ratio de compensación elevado requieren revisión manual. | Reclamo por no recepción con GPS no confirmado y alta tasa de compensación previa en cuenta antigua.</t>
+        </is>
+      </c>
+      <c r="AB141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -15649,7 +15764,7 @@
       </c>
       <c r="W142" t="inlineStr">
         <is>
-          <t>Usuario con más de 3 años de antigüedad, 0 flags y 0 reclamos recientes. El reclamo por ítem incorrecto es coherente y el monto es razonable. La pérdida de señal GPS no indica fraude al no haber contradicciones.</t>
+          <t>Usuario con más de 3 años de antigüedad, sin historial de fraude ni alta frecuencia de reclamos. La solicitud por producto incorrecto es coherente y el monto es razonable.</t>
         </is>
       </c>
       <c r="X142" t="inlineStr"/>
@@ -15661,9 +15776,10 @@
       <c r="Z142" t="inlineStr"/>
       <c r="AA142" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con perfil de usuario confiable y sin señales de abuso. | Error operativo del restaurante en usuario antiguo y sin historial de riesgo.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo legítimo consistente con perfil de usuario sano y sin inconsistencias. | Reclamo operativo por entrega de bebida errónea en cuenta antigua y confiable sin señales de riesgo.</t>
+        </is>
+      </c>
+      <c r="AB142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -15770,6 +15886,7 @@
         </is>
       </c>
       <c r="AA143" t="inlineStr"/>
+      <c r="AB143" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -15872,6 +15989,7 @@
         </is>
       </c>
       <c r="AA144" t="inlineStr"/>
+      <c r="AB144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -15966,7 +16084,7 @@
       </c>
       <c r="W145" t="inlineStr">
         <is>
-          <t>Usuario con antigüedad superior a 3 años, sin flags de fraude ni frecuencia de reclamos. El motivo descrito corresponde a un error operativo estándar de facturación por cancelación del restaurante.</t>
+          <t>Usuario con más de 3 años de antigüedad, historial limpio y sin reclamos recientes. El motivo corresponde a un error de facturación por cancelación del restaurante, totalmente coherente con la evidencia operativa.</t>
         </is>
       </c>
       <c r="X145" t="inlineStr"/>
@@ -15978,9 +16096,10 @@
       <c r="Z145" t="inlineStr"/>
       <c r="AA145" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo legítimo consistente con un error administrativo, sin señales de fraude. | Error de facturación por cancelación del restaurante en cuenta antigua y sin historial sospechoso.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo consistente con usuario de alto perfil y sin señales de fraude o inconsistencias. | Reclamo operativo legítimo por cargo no revertido tras cancelación en cuenta antigua y sin antecedentes de fraude.</t>
+        </is>
+      </c>
+      <c r="AB145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -16083,6 +16202,7 @@
         </is>
       </c>
       <c r="AA146" t="inlineStr"/>
+      <c r="AB146" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -16177,7 +16297,7 @@
       </c>
       <c r="W147" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', palabra crítica que activa protocolo de seguridad por riesgo legal/salud. Sumado a 2 flags de fraude previos y evidencia GPS parcial, se requiere revisión humana para validar la justificación médica y evitar exposición de marca.</t>
+          <t>El reclamo menciona 'alergia', activando la regla de palabras críticas que exige revisión humana por riesgo de salud y reputación. Se combina con 2 flags de fraude previos y evidencia GPS parcial, lo que invalida la aprobación automática.</t>
         </is>
       </c>
       <c r="X147" t="inlineStr">
@@ -16188,7 +16308,7 @@
       </c>
       <c r="Y147" t="inlineStr">
         <is>
-          <t>palabras_criticas_seguridad | flag_fraude_previo</t>
+          <t>palabras_criticas_seguridad | flag_fraude_previo | evidencia_gps_parcial</t>
         </is>
       </c>
       <c r="Z147" t="inlineStr">
@@ -16198,9 +16318,10 @@
       </c>
       <c r="AA147" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene término crítico ('alergia') que implica riesgo de salud/legal, reforzado por 2 flags de fraude previos y evidencia GPS inconclusa. Requiere validación humana obligatoria. | Reclamo por alergia alimentaria en cuenta con historial de fraude y GPS parcial. Activación automática por palabras críticas de seguridad.</t>
-        </is>
-      </c>
+          <t>ESCALAR: contiene palabra crítica ('alergia') que activa protocolo de riesgo legal/salud, sumado a 2 flags de fraude previos y GPS parcial que dificultan la verificación objetiva. | Reclamo por alergia alimentaria en cuenta con historial de fraude y GPS ambigua. Requiere validación humana conforme a política de seguridad de marca.</t>
+        </is>
+      </c>
+      <c r="AB147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -16295,21 +16416,18 @@
       </c>
       <c r="W148" t="inlineStr">
         <is>
-          <t>Usuario con más de 4 años de antigüedad y 0 flags de fraude. Reclamo de discrepancia tarifaria sin indicadores de abuso.</t>
+          <t>Perfil de usuario antiguo (1612d) sin flags de fraude ni alta frecuencia. El reclamo es una consulta de facturación estándar con monto dentro de rangos normales.</t>
         </is>
       </c>
       <c r="X148" t="inlineStr"/>
-      <c r="Y148" t="inlineStr">
-        <is>
-          <t>entrega_gps_no_confirmada</t>
-        </is>
-      </c>
+      <c r="Y148" t="inlineStr"/>
       <c r="Z148" t="inlineStr"/>
       <c r="AA148" t="inlineStr">
         <is>
-          <t>APROBAR: reclamo operativo legítimo sin señales de fraude ni patrones abusivos. | Discrepancia entre monto cobrado y resumen de pedido reportada por usuario antiguo y confiable.</t>
-        </is>
-      </c>
+          <t>APROBAR: reclamo operativo legítimo sin señales de fraude. | Discrepancia de cobro en cuenta confiable sin indicadores de abuso o riesgo.</t>
+        </is>
+      </c>
+      <c r="AB148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -16404,7 +16522,7 @@
       </c>
       <c r="W149" t="inlineStr">
         <is>
-          <t>El reclamo menciona 'alergia', activando la regla de palabras críticas que exige revisión humana por riesgo de salud y responsabilidad legal. Adicionalmente, la cuenta tiene solo 29 días de antigüedad con 14 reclamos en 90 días y 2 flags de fraude previos, lo que indica un patrón de abuso y alto riesgo.</t>
+          <t>El reclamo menciona 'alergia', palabra crítica de seguridad que activa protocolo de escalación obligatoria. Se combina con cuenta nueva (29d), alta frecuencia de reclamos (14 en 90d) y historial con 2 flags de fraude, lo que eleva el riesgo legal y operativo.</t>
         </is>
       </c>
       <c r="X149" t="inlineStr">
@@ -16425,9 +16543,10 @@
       </c>
       <c r="AA149" t="inlineStr">
         <is>
-          <t>ESCALAR: contiene palabra crítica ('alergia') que implica riesgo de salud y responsabilidad civil, sumado a historial de fraude y cuenta nueva con alta densidad de reclamos. | Reclamo por alergia en cuenta nueva con alta frecuencia, flags de fraude previos y evidencia pre-marcada para escalación por seguridad de marca.</t>
-        </is>
-      </c>
+          <t>ESCALAR: presencia de palabra crítica ('alergia') que exige revisión manual por riesgo legal/salud, corroborado por perfil de cuenta nueva con alta reincidencia y flags de fraude previos. | Reclamo por alergia alimentaria en cuenta nueva con alta densidad de reclamos y antecedentes de fraude. Pre-marcado para revisión humana por implicaciones de salud y riesgo de marca.</t>
+        </is>
+      </c>
+      <c r="AB149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -16530,6 +16649,7 @@
         </is>
       </c>
       <c r="AA150" t="inlineStr"/>
+      <c r="AB150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -16609,7 +16729,7 @@
       </c>
       <c r="T151" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="U151" t="inlineStr">
@@ -16619,26 +16739,27 @@
       </c>
       <c r="V151" t="inlineStr">
         <is>
-          <t>RECHAZAR</t>
+          <t>ESCALAR</t>
         </is>
       </c>
       <c r="W151" t="inlineStr">
         <is>
-          <t>El perfil presenta un flag de fraude previo y un ratio de compensación muy alto (0.93), sumado a la falta de confirmación GPS que valide la entrega reclamada.</t>
+          <t>Cuenta con flag de fraude previo y ratio de compensación elevado (0.93). La evidencia GPS no confirma la entrega, generando ambigüedad que requiere revisión humana para validar o refutar el reclamo.</t>
         </is>
       </c>
       <c r="X151" t="inlineStr"/>
       <c r="Y151" t="inlineStr">
         <is>
-          <t>flag_fraude_previo | compensacion_elevada | entrega_gps_no_confirmada</t>
+          <t>flag_fraude_previo | entrega_gps_no_confirmada | compensacion_elevada</t>
         </is>
       </c>
       <c r="Z151" t="inlineStr"/>
       <c r="AA151" t="inlineStr">
         <is>
-          <t>RECHAZAR: inconsistencia por falta de evidencia GPS combinada con flag de fraude previo y ratio de compensación elevado. | Reclamo sin respaldo geolocal y con historial de riesgo y compensaciones elevadas.</t>
-        </is>
-      </c>
+          <t>ESCALAR: combinación de flag de fraude previo, ratio de compensación alto y falta de evidencia GPS determina necesidad de revisión manual. | Reclamo por entrega no recibida sin validación GPS en cuenta con historial de fraude y alta propensión a compensaciones.</t>
+        </is>
+      </c>
+      <c r="AB151" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>